<commit_message>
📊 Daily Chinese DB update: 2026-09-07 | 1085/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1073"/>
+  <dimension ref="A1:I1086"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50847,6 +50847,617 @@
         </is>
       </c>
     </row>
+    <row r="1074">
+      <c r="A1074" t="inlineStr">
+        <is>
+          <t>CHI-20260907-001</t>
+        </is>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1074" t="inlineStr">
+        <is>
+          <t>官宣</t>
+        </is>
+      </c>
+      <c r="E1074" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1074" t="inlineStr">
+        <is>
+          <t>guān xuān</t>
+        </is>
+      </c>
+      <c r="G1074" t="inlineStr">
+        <is>
+          <t>공식 발표하다, 공식적으로 공개하다</t>
+        </is>
+      </c>
+      <c r="H1074" t="inlineStr">
+        <is>
+          <t>드라마나 SNS에서 연예인의 열애나 기업의 중대 발표를 공식적으로 알릴 때 쓰는 표현</t>
+        </is>
+      </c>
+      <c r="I1074" t="inlineStr">
+        <is>
+          <t>他们终于在微博上官宣了这段恋情。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" t="inlineStr">
+        <is>
+          <t>CHI-20260907-002</t>
+        </is>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1075" t="inlineStr">
+        <is>
+          <t>到岗</t>
+        </is>
+      </c>
+      <c r="E1075" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1075" t="inlineStr">
+        <is>
+          <t>dào gǎng</t>
+        </is>
+      </c>
+      <c r="G1075" t="inlineStr">
+        <is>
+          <t>근무지에 도착하다, 업무를 시작하다</t>
+        </is>
+      </c>
+      <c r="H1075" t="inlineStr">
+        <is>
+          <t>직장인들이 출근하여 업무 준비를 마쳤을 때 주로 사용하는 표현</t>
+        </is>
+      </c>
+      <c r="I1075" t="inlineStr">
+        <is>
+          <t>所有工作人员必须在八点前准时到岗。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="inlineStr">
+        <is>
+          <t>CHI-20260907-003</t>
+        </is>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C1076" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1076" t="inlineStr">
+        <is>
+          <t>走访</t>
+        </is>
+      </c>
+      <c r="E1076" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1076" t="inlineStr">
+        <is>
+          <t>zǒu fǎng</t>
+        </is>
+      </c>
+      <c r="G1076" t="inlineStr">
+        <is>
+          <t>방문하다, 순방하다</t>
+        </is>
+      </c>
+      <c r="H1076" t="inlineStr">
+        <is>
+          <t>공직자나 관계자가 현장을 직접 찾아가 살펴보거나 상담할 때 쓰는 격식 있는 표현</t>
+        </is>
+      </c>
+      <c r="I1076" t="inlineStr">
+        <is>
+          <t>领导下基层走访了解民生问题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="inlineStr">
+        <is>
+          <t>CHI-20260907-004</t>
+        </is>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C1077" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1077" t="inlineStr">
+        <is>
+          <t>联手</t>
+        </is>
+      </c>
+      <c r="E1077" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1077" t="inlineStr">
+        <is>
+          <t>lián shǒu</t>
+        </is>
+      </c>
+      <c r="G1077" t="inlineStr">
+        <is>
+          <t>협력하다, 손잡다</t>
+        </is>
+      </c>
+      <c r="H1077" t="inlineStr">
+        <is>
+          <t>기업이나 부서 간에 협업을 진행할 때 뉴스나 비즈니스에서 자주 등장함</t>
+        </is>
+      </c>
+      <c r="I1077" t="inlineStr">
+        <is>
+          <t>两家知名企业决定联手开发新产品。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" t="inlineStr">
+        <is>
+          <t>CHI-20260907-005</t>
+        </is>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1078" t="inlineStr">
+        <is>
+          <t>亮绿灯</t>
+        </is>
+      </c>
+      <c r="E1078" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1078" t="inlineStr">
+        <is>
+          <t>liàng lǜ dēng</t>
+        </is>
+      </c>
+      <c r="G1078" t="inlineStr">
+        <is>
+          <t>허가하다, 승인하다, 편의를 봐주다</t>
+        </is>
+      </c>
+      <c r="H1078" t="inlineStr">
+        <is>
+          <t>프로젝트 진행이나 정책 추진에 있어 장애물을 제거하고 승인해 줄 때 사용하는 비유적 표현</t>
+        </is>
+      </c>
+      <c r="I1078" t="inlineStr">
+        <is>
+          <t>政府为高科技项目亮了绿灯。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="inlineStr">
+        <is>
+          <t>CHI-20260907-006</t>
+        </is>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1079" t="inlineStr">
+        <is>
+          <t>放宽</t>
+        </is>
+      </c>
+      <c r="E1079" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1079" t="inlineStr">
+        <is>
+          <t>fàng kuān</t>
+        </is>
+      </c>
+      <c r="G1079" t="inlineStr">
+        <is>
+          <t>완화하다, 넓히다</t>
+        </is>
+      </c>
+      <c r="H1079" t="inlineStr">
+        <is>
+          <t>채용 조건이나 제한 등을 느슨하게 만들 때 사용하는 표현</t>
+        </is>
+      </c>
+      <c r="I1079" t="inlineStr">
+        <is>
+          <t>公司决定放宽对应聘者的学历要求。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="inlineStr">
+        <is>
+          <t>CHI-20260907-007</t>
+        </is>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1080" t="inlineStr">
+        <is>
+          <t>到位</t>
+        </is>
+      </c>
+      <c r="E1080" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1080" t="inlineStr">
+        <is>
+          <t>dào wèi</t>
+        </is>
+      </c>
+      <c r="G1080" t="inlineStr">
+        <is>
+          <t>완벽하다, 정확하다, 충분하다</t>
+        </is>
+      </c>
+      <c r="H1080" t="inlineStr">
+        <is>
+          <t>업무 처리가 아주 꼼꼼하고 빈틈없을 때 칭찬하는 표현</t>
+        </is>
+      </c>
+      <c r="I1080" t="inlineStr">
+        <is>
+          <t>你的工作准备得很到位。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="inlineStr">
+        <is>
+          <t>CHI-20260907-008</t>
+        </is>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1081" t="inlineStr">
+        <is>
+          <t>瓶颈</t>
+        </is>
+      </c>
+      <c r="E1081" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1081" t="inlineStr">
+        <is>
+          <t>píng jǐng</t>
+        </is>
+      </c>
+      <c r="G1081" t="inlineStr">
+        <is>
+          <t>병목 현상, 발전이 정체된 상태</t>
+        </is>
+      </c>
+      <c r="H1081" t="inlineStr">
+        <is>
+          <t>업무나 실력이 더 이상 발전하지 못하고 정체된 시기를 비유</t>
+        </is>
+      </c>
+      <c r="I1081" t="inlineStr">
+        <is>
+          <t>我最近在工作中遇到了职业瓶颈。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="inlineStr">
+        <is>
+          <t>CHI-20260907-009</t>
+        </is>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1082" t="inlineStr">
+        <is>
+          <t>见怪不怪</t>
+        </is>
+      </c>
+      <c r="E1082" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F1082" t="inlineStr">
+        <is>
+          <t>jiàn guài bù guài</t>
+        </is>
+      </c>
+      <c r="G1082" t="inlineStr">
+        <is>
+          <t>이상하게 여길 것도 없다, 흔한 일이다</t>
+        </is>
+      </c>
+      <c r="H1082" t="inlineStr">
+        <is>
+          <t>어떤 상황이 너무 자주 일어나 놀랍지도 않을 때 사용하는 표현</t>
+        </is>
+      </c>
+      <c r="I1082" t="inlineStr">
+        <is>
+          <t>对于这种小事，我们已经见怪不怪了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="inlineStr">
+        <is>
+          <t>CHI-20260907-010</t>
+        </is>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1083" t="inlineStr">
+        <is>
+          <t>吹了</t>
+        </is>
+      </c>
+      <c r="E1083" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1083" t="inlineStr">
+        <is>
+          <t>chuī le</t>
+        </is>
+      </c>
+      <c r="G1083" t="inlineStr">
+        <is>
+          <t>끝났다, 무산되었다</t>
+        </is>
+      </c>
+      <c r="H1083" t="inlineStr">
+        <is>
+          <t>계획이나 연애 관계 등이 허무하게 끝났을 때 쓰는 가벼운 구어체</t>
+        </is>
+      </c>
+      <c r="I1083" t="inlineStr">
+        <is>
+          <t>那个合作项目因为资金问题吹了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="inlineStr">
+        <is>
+          <t>CHI-20260907-011</t>
+        </is>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1084" t="inlineStr">
+        <is>
+          <t>碰头</t>
+        </is>
+      </c>
+      <c r="E1084" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1084" t="inlineStr">
+        <is>
+          <t>pèng tóu</t>
+        </is>
+      </c>
+      <c r="G1084" t="inlineStr">
+        <is>
+          <t>만나서 상의하다, 간단히 회의하다</t>
+        </is>
+      </c>
+      <c r="H1084" t="inlineStr">
+        <is>
+          <t>본격적인 회의 전 짧게 얼굴을 보고 의견을 나누는 행위</t>
+        </is>
+      </c>
+      <c r="I1084" t="inlineStr">
+        <is>
+          <t>我们明天早上碰个头，把方案定下来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="inlineStr">
+        <is>
+          <t>CHI-20260907-012</t>
+        </is>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1085" t="inlineStr">
+        <is>
+          <t>上轨道</t>
+        </is>
+      </c>
+      <c r="E1085" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1085" t="inlineStr">
+        <is>
+          <t>shàng guǐ dào</t>
+        </is>
+      </c>
+      <c r="G1085" t="inlineStr">
+        <is>
+          <t>정상 궤도에 오르다, 제대로 돌아가다</t>
+        </is>
+      </c>
+      <c r="H1085" t="inlineStr">
+        <is>
+          <t>일이나 프로젝트가 시행착오를 마치고 안정적으로 돌아가기 시작할 때</t>
+        </is>
+      </c>
+      <c r="I1085" t="inlineStr">
+        <is>
+          <t>经过调整，新业务终于步上轨道了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="inlineStr">
+        <is>
+          <t>CHI-20260907-013</t>
+        </is>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1086" t="inlineStr">
+        <is>
+          <t>接轨</t>
+        </is>
+      </c>
+      <c r="E1086" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1086" t="inlineStr">
+        <is>
+          <t>jiē guǐ</t>
+        </is>
+      </c>
+      <c r="G1086" t="inlineStr">
+        <is>
+          <t>접목하다, 기준을 맞추다</t>
+        </is>
+      </c>
+      <c r="H1086" t="inlineStr">
+        <is>
+          <t>解码生态法典筑...</t>
+        </is>
+      </c>
+      <c r="I1086" t="inlineStr">
+        <is>
+          <t>我们的产品标准必须尽快与国际接轨。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-08 | 1095/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1086"/>
+  <dimension ref="A1:I1096"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51458,6 +51458,476 @@
         </is>
       </c>
     </row>
+    <row r="1087">
+      <c r="A1087" t="inlineStr">
+        <is>
+          <t>CHI-20260908-001</t>
+        </is>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1087" t="inlineStr">
+        <is>
+          <t>慢半拍</t>
+        </is>
+      </c>
+      <c r="E1087" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1087" t="inlineStr">
+        <is>
+          <t>màn bàn pāi</t>
+        </is>
+      </c>
+      <c r="G1087" t="inlineStr">
+        <is>
+          <t>한 박자 늦다, 대처가 굼뜨다</t>
+        </is>
+      </c>
+      <c r="H1087" t="inlineStr">
+        <is>
+          <t>刚开学时久坐少动的学生，猛然上体育课时动作和反应总会慢半拍。</t>
+        </is>
+      </c>
+      <c r="I1087" t="inlineStr">
+        <is>
+          <t>我今天感冒了，脑子有点慢半拍，你刚才说的话我没太听懂。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" t="inlineStr">
+        <is>
+          <t>CHI-20260908-002</t>
+        </is>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1088" t="inlineStr">
+        <is>
+          <t>拉关系</t>
+        </is>
+      </c>
+      <c r="E1088" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1088" t="inlineStr">
+        <is>
+          <t>lā guān xi</t>
+        </is>
+      </c>
+      <c r="G1088" t="inlineStr">
+        <is>
+          <t>환심을 사다, 인맥을 동원하여 줄을 대다</t>
+        </is>
+      </c>
+      <c r="H1088" t="inlineStr">
+        <is>
+          <t>在国际合作中，靠那些拉关系的偏门手段是走不远的长久之计。</t>
+        </is>
+      </c>
+      <c r="I1088" t="inlineStr">
+        <is>
+          <t>与其整天想着和领导拉关系，不如踏踏实实提高自己的业务水平。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" t="inlineStr">
+        <is>
+          <t>CHI-20260908-003</t>
+        </is>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1089" t="inlineStr">
+        <is>
+          <t>白手起家</t>
+        </is>
+      </c>
+      <c r="E1089" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1089" t="inlineStr">
+        <is>
+          <t>bái shǒu qǐ jiā</t>
+        </is>
+      </c>
+      <c r="G1089" t="inlineStr">
+        <is>
+          <t>맨손으로 자수성가하다</t>
+        </is>
+      </c>
+      <c r="H1089" t="inlineStr">
+        <is>
+          <t>在我家编撰的家史中，最让人动容的是祖父当年白手起家的移民奋斗史。</t>
+        </is>
+      </c>
+      <c r="I1089" t="inlineStr">
+        <is>
+          <t>他没有依靠父母的任何资助，硬是凭着一股干劲白手起家创办了公司。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" t="inlineStr">
+        <is>
+          <t>CHI-20260908-004</t>
+        </is>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1090" t="inlineStr">
+        <is>
+          <t>半瓶醋</t>
+        </is>
+      </c>
+      <c r="E1090" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1090" t="inlineStr">
+        <is>
+          <t>bàn píng cù</t>
+        </is>
+      </c>
+      <c r="G1090" t="inlineStr">
+        <is>
+          <t>어설픈 지식인, 선무당, 수박 겉핥기식 지식</t>
+        </is>
+      </c>
+      <c r="H1090" t="inlineStr">
+        <is>
+          <t>在健康饮食和科学运动方面，不要盲目相信那些网上‘半瓶醋’博主的建议。</t>
+        </is>
+      </c>
+      <c r="I1090" t="inlineStr">
+        <is>
+          <t>他对电脑技术只是个半瓶醋，却总喜欢装成大师教别人修电脑。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" t="inlineStr">
+        <is>
+          <t>CHI-20260908-005</t>
+        </is>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1091" t="inlineStr">
+        <is>
+          <t>耍花招</t>
+        </is>
+      </c>
+      <c r="E1091" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1091" t="inlineStr">
+        <is>
+          <t>shuǎ huā zhāo</t>
+        </is>
+      </c>
+      <c r="G1091" t="inlineStr">
+        <is>
+          <t>꼼수를 쓰다, 잔머리를 굴리다</t>
+        </is>
+      </c>
+      <c r="H1091" t="inlineStr">
+        <is>
+          <t>办事要诚实，千万别跟合作伙伴耍花招。</t>
+        </is>
+      </c>
+      <c r="I1091" t="inlineStr">
+        <is>
+          <t>大家都看穿了他的心思，他再怎么耍花招也没用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>CHI-20260908-006</t>
+        </is>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1092" t="inlineStr">
+        <is>
+          <t>纳闷儿</t>
+        </is>
+      </c>
+      <c r="E1092" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1092" t="inlineStr">
+        <is>
+          <t>nà mènr</t>
+        </is>
+      </c>
+      <c r="G1092" t="inlineStr">
+        <is>
+          <t>의아해하다, 속으로 이상하게 생각하다</t>
+        </is>
+      </c>
+      <c r="H1092" t="inlineStr">
+        <is>
+          <t>我觉得很纳闷儿，他怎么突然改变主意了？</t>
+        </is>
+      </c>
+      <c r="I1092" t="inlineStr">
+        <is>
+          <t>大家都准时到了，唯独他没来，我心里挺纳闷儿的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="inlineStr">
+        <is>
+          <t>CHI-20260908-007</t>
+        </is>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1093" t="inlineStr">
+        <is>
+          <t>凑合</t>
+        </is>
+      </c>
+      <c r="E1093" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1093" t="inlineStr">
+        <is>
+          <t>còu he</t>
+        </is>
+      </c>
+      <c r="G1093" t="inlineStr">
+        <is>
+          <t>그런대로 아쉬운 대로 하다, 대충 때우다</t>
+        </is>
+      </c>
+      <c r="H1093" t="inlineStr">
+        <is>
+          <t>这件衣服虽然有点旧，但还能凑合穿。</t>
+        </is>
+      </c>
+      <c r="I1093" t="inlineStr">
+        <is>
+          <t>今天中午实在没时间，咱们就随便凑合一顿吧。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="inlineStr">
+        <is>
+          <t>CHI-20260908-008</t>
+        </is>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1094" t="inlineStr">
+        <is>
+          <t>跑龙套</t>
+        </is>
+      </c>
+      <c r="E1094" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1094" t="inlineStr">
+        <is>
+          <t>pǎo lóng tào</t>
+        </is>
+      </c>
+      <c r="G1094" t="inlineStr">
+        <is>
+          <t>단역을 맡다, 보조 역할을 하다, 들러리를 서다</t>
+        </is>
+      </c>
+      <c r="H1094" t="inlineStr">
+        <is>
+          <t>他在演艺圈跑龙套多年，终于当上了主角。</t>
+        </is>
+      </c>
+      <c r="I1094" t="inlineStr">
+        <is>
+          <t>在这个大项目中，我只是个跑龙套的，没起多大核心作用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="inlineStr">
+        <is>
+          <t>CHI-20260908-009</t>
+        </is>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1095" t="inlineStr">
+        <is>
+          <t>下马威</t>
+        </is>
+      </c>
+      <c r="E1095" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1095" t="inlineStr">
+        <is>
+          <t>xià mǎ wēi</t>
+        </is>
+      </c>
+      <c r="G1095" t="inlineStr">
+        <is>
+          <t>기선 제압, 첫판부터 군기를 잡음</t>
+        </is>
+      </c>
+      <c r="H1095" t="inlineStr">
+        <is>
+          <t>新官上任三把火，他是想给下属一个下马威。</t>
+        </is>
+      </c>
+      <c r="I1095" t="inlineStr">
+        <is>
+          <t>刚进公司第一天，主管就交给我一堆难办的任务，显然是想给我个下马威。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="inlineStr">
+        <is>
+          <t>CHI-20260908-010</t>
+        </is>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1096" t="inlineStr">
+        <is>
+          <t>侃大山</t>
+        </is>
+      </c>
+      <c r="E1096" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1096" t="inlineStr">
+        <is>
+          <t>kǎn dà shān</t>
+        </is>
+      </c>
+      <c r="G1096" t="inlineStr">
+        <is>
+          <t>한가롭게 잡담하다, 수다를 떨다</t>
+        </is>
+      </c>
+      <c r="H1096" t="inlineStr">
+        <is>
+          <t>晚饭后，邻居们喜欢聚在树底下闲聊侃大山。</t>
+        </is>
+      </c>
+      <c r="I1096" t="inlineStr">
+        <is>
+          <t>咱们别老坐着侃大山了，赶紧把正事干了吧。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-09 | 1100/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1096"/>
+  <dimension ref="A1:I1101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51928,6 +51928,241 @@
         </is>
       </c>
     </row>
+    <row r="1097">
+      <c r="A1097" t="inlineStr">
+        <is>
+          <t>CHI-20260909-001</t>
+        </is>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1097" t="inlineStr">
+        <is>
+          <t>吃老本</t>
+        </is>
+      </c>
+      <c r="E1097" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1097" t="inlineStr">
+        <is>
+          <t>chī lǎoběn</t>
+        </is>
+      </c>
+      <c r="G1097" t="inlineStr">
+        <is>
+          <t>과거의 밑천이나 성과에 안주하며 게으름을 피우다</t>
+        </is>
+      </c>
+      <c r="H1097" t="inlineStr">
+        <is>
+          <t>大学里不能总吃老本，高中的好成绩不代表以后也能高枕无忧。</t>
+        </is>
+      </c>
+      <c r="I1097" t="inlineStr">
+        <is>
+          <t>现在的行业竞争太激烈了，只靠吃老本早晚会被淘汰。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="inlineStr">
+        <is>
+          <t>CHI-20260909-002</t>
+        </is>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1098" t="inlineStr">
+        <is>
+          <t>过河拆桥</t>
+        </is>
+      </c>
+      <c r="E1098" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1098" t="inlineStr">
+        <is>
+          <t>guò hé chāi qiáo</t>
+        </is>
+      </c>
+      <c r="G1098" t="inlineStr">
+        <is>
+          <t>목적을 달성한 후 고마움을 모르고 배은망덕하게 굴다</t>
+        </is>
+      </c>
+      <c r="H1098" t="inlineStr">
+        <is>
+          <t>中国一直在帮助其他国家发展，绝对不会做出过河拆桥、抽走梯子的事。</t>
+        </is>
+      </c>
+      <c r="I1098" t="inlineStr">
+        <is>
+          <t>当初是我借钱帮他渡过难关，没想到他现在过河拆桥，连电话都不接了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="inlineStr">
+        <is>
+          <t>CHI-20260909-003</t>
+        </is>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1099" t="inlineStr">
+        <is>
+          <t>落井下石</t>
+        </is>
+      </c>
+      <c r="E1099" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1099" t="inlineStr">
+        <is>
+          <t>luò jǐng xià shí</t>
+        </is>
+      </c>
+      <c r="G1099" t="inlineStr">
+        <is>
+          <t>곤경에 처한 사람을 도와주기는커녕 더 곤란하게 만들다</t>
+        </is>
+      </c>
+      <c r="H1099" t="inlineStr">
+        <is>
+          <t>在别人遇到困难需要支持的时候，我们应该伸出援手，而不是落井下石。</t>
+        </is>
+      </c>
+      <c r="I1099" t="inlineStr">
+        <is>
+          <t>他已经因为破产够痛苦的了，你这时候去催债简直就是落井下石。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="inlineStr">
+        <is>
+          <t>CHI-20260909-004</t>
+        </is>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1100" t="inlineStr">
+        <is>
+          <t>措手不及</t>
+        </is>
+      </c>
+      <c r="E1100" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1100" t="inlineStr">
+        <is>
+          <t>cuò shǒu bù jí</t>
+        </is>
+      </c>
+      <c r="G1100" t="inlineStr">
+        <is>
+          <t>대처할 겨를도 없이 당황하다, 허를 찔리다</t>
+        </is>
+      </c>
+      <c r="H1100" t="inlineStr">
+        <is>
+          <t>面对突然提高难度的大学摸底考，不少大一新生被打得措手不及。</t>
+        </is>
+      </c>
+      <c r="I1100" t="inlineStr">
+        <is>
+          <t>这次突如其来的市场变化，让很多中小型企业措手不及。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="inlineStr">
+        <is>
+          <t>CHI-20260909-005</t>
+        </is>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1101" t="inlineStr">
+        <is>
+          <t>一针见血</t>
+        </is>
+      </c>
+      <c r="E1101" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1101" t="inlineStr">
+        <is>
+          <t>yī zhēn jiàn xiě</t>
+        </is>
+      </c>
+      <c r="G1101" t="inlineStr">
+        <is>
+          <t>정곡을 찌르다, 요점을 아주 예리하게 지적하다</t>
+        </is>
+      </c>
+      <c r="H1101" t="inlineStr">
+        <is>
+          <t>他的这篇评论虽然字数不多，却一针见血地指出了目前社会存在的问题。</t>
+        </is>
+      </c>
+      <c r="I1101" t="inlineStr">
+        <is>
+          <t>分析师一针见血地指出了该公司股价暴跌的核心原因。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-10 | 1106/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1101"/>
+  <dimension ref="A1:I1107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -52163,6 +52163,288 @@
         </is>
       </c>
     </row>
+    <row r="1102">
+      <c r="A1102" t="inlineStr">
+        <is>
+          <t>CHI-20260910-001</t>
+        </is>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1102" t="inlineStr">
+        <is>
+          <t>化平凡为神奇</t>
+        </is>
+      </c>
+      <c r="E1102" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F1102" t="inlineStr">
+        <is>
+          <t>huà píng fán wéi shén qí</t>
+        </is>
+      </c>
+      <c r="G1102" t="inlineStr">
+        <is>
+          <t>평범함을 비범함으로 바꾸다, 평범한 것을 기적으로 만들다</t>
+        </is>
+      </c>
+      <c r="H1102" t="inlineStr">
+        <is>
+          <t>关注职业教育老师如何在不同的“三尺讲台”上“化平凡为神奇”。</t>
+        </is>
+      </c>
+      <c r="I1102" t="inlineStr">
+        <is>
+          <t>优秀的规划师能够化平凡为神奇，把破旧的老街区变成热门打卡地。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" t="inlineStr">
+        <is>
+          <t>CHI-20260910-002</t>
+        </is>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1103" t="inlineStr">
+        <is>
+          <t>眼前一亮</t>
+        </is>
+      </c>
+      <c r="E1103" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1103" t="inlineStr">
+        <is>
+          <t>yǎn qián yī liàng</t>
+        </is>
+      </c>
+      <c r="G1103" t="inlineStr">
+        <is>
+          <t>(새롭거나 훌륭한 것을 보고) 눈이 번쩍 뜨이다, 시선을 사로잡다</t>
+        </is>
+      </c>
+      <c r="H1103" t="inlineStr">
+        <is>
+          <t>把宋锦织进牛仔、在实验室里“养”面料，这季时装周的创意让人眼前一亮。</t>
+        </is>
+      </c>
+      <c r="I1103" t="inlineStr">
+        <is>
+          <t>她的平面设计作品非常独特，评委们看了都眼前一亮。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="inlineStr">
+        <is>
+          <t>CHI-20260910-003</t>
+        </is>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1104" t="inlineStr">
+        <is>
+          <t>慕名而来</t>
+        </is>
+      </c>
+      <c r="E1104" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F1104" t="inlineStr">
+        <is>
+          <t>mù míng ér lái</t>
+        </is>
+      </c>
+      <c r="G1104" t="inlineStr">
+        <is>
+          <t>명성을 듣고 찾아오다</t>
+        </is>
+      </c>
+      <c r="H1104" t="inlineStr">
+        <is>
+          <t>城市的独特特质吸引了许多台湾青年，他们都慕名而来。</t>
+        </is>
+      </c>
+      <c r="I1104" t="inlineStr">
+        <is>
+          <t>这家餐厅的招牌菜非常出名，每天都有很多游客慕名而来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="inlineStr">
+        <is>
+          <t>CHI-20260910-004</t>
+        </is>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1105" t="inlineStr">
+        <is>
+          <t>小题大做</t>
+        </is>
+      </c>
+      <c r="E1105" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F1105" t="inlineStr">
+        <is>
+          <t>xiǎo tí dà zuò</t>
+        </is>
+      </c>
+      <c r="G1105" t="inlineStr">
+        <is>
+          <t>작은 일을 크게 벌이다, 침소봉대하다</t>
+        </is>
+      </c>
+      <c r="H1105" t="inlineStr">
+        <is>
+          <t>不必放大高考与入学考试的分数落差，不要小题大做。</t>
+        </is>
+      </c>
+      <c r="I1105" t="inlineStr">
+        <is>
+          <t>他只是不小心迟到了五分钟，你没必要这样小题大做。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" t="inlineStr">
+        <is>
+          <t>CHI-20260910-005</t>
+        </is>
+      </c>
+      <c r="B1106" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C1106" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1106" t="inlineStr">
+        <is>
+          <t>换位思考</t>
+        </is>
+      </c>
+      <c r="E1106" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1106" t="inlineStr">
+        <is>
+          <t>huàn wèi sī kǎo</t>
+        </is>
+      </c>
+      <c r="G1106" t="inlineStr">
+        <is>
+          <t>역지사지하다, 입장을 바꾸어 생각하다</t>
+        </is>
+      </c>
+      <c r="H1106" t="inlineStr">
+        <is>
+          <t>城市治理不仅要有力度，更要懂得换位思考，体谅小摊贩的难处。</t>
+        </is>
+      </c>
+      <c r="I1106" t="inlineStr">
+        <is>
+          <t>夫妻之间如果能多一些换位思考，就能减少很多不必要的争吵。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" t="inlineStr">
+        <is>
+          <t>CHI-20260910-006</t>
+        </is>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C1107" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1107" t="inlineStr">
+        <is>
+          <t>摇钱树</t>
+        </is>
+      </c>
+      <c r="E1107" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1107" t="inlineStr">
+        <is>
+          <t>yáo qián shù</t>
+        </is>
+      </c>
+      <c r="G1107" t="inlineStr">
+        <is>
+          <t>돈줄, 화수분 (쉽게 돈을 벌어다 주는 사람이나 사물)</t>
+        </is>
+      </c>
+      <c r="H1107" t="inlineStr">
+        <is>
+          <t>那个明星成了经纪公司的摇钱树，每天的行程都被排得满满的。</t>
+        </is>
+      </c>
+      <c r="I1107" t="inlineStr">
+        <is>
+          <t>这款畅销游戏已经成为了公司最核心的摇钱树。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-11 | 1121/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1107"/>
+  <dimension ref="A1:I1122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -52445,6 +52445,711 @@
         </is>
       </c>
     </row>
+    <row r="1108">
+      <c r="A1108" t="inlineStr">
+        <is>
+          <t>CHI-20260911-001</t>
+        </is>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C1108" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1108" t="inlineStr">
+        <is>
+          <t>一落千丈</t>
+        </is>
+      </c>
+      <c r="E1108" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1108" t="inlineStr">
+        <is>
+          <t>yí luò qiān zhàng</t>
+        </is>
+      </c>
+      <c r="G1108" t="inlineStr">
+        <is>
+          <t>실력, 성적, 명성 등이 한순간에 급격히 떨어지다</t>
+        </is>
+      </c>
+      <c r="H1108" t="inlineStr">
+        <is>
+          <t>고교 시절 우수한 성적을 거두었던 학생이 대학에 와서 첫 시험에 낙제점을 받으며 성적이 곤두박질친 상황을 묘사합니다.</t>
+        </is>
+      </c>
+      <c r="I1108" t="inlineStr">
+        <is>
+          <t>自从他迷上网络游戏后，学习成绩就一落千丈。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" t="inlineStr">
+        <is>
+          <t>CHI-20260911-002</t>
+        </is>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C1109" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1109" t="inlineStr">
+        <is>
+          <t>货真价实</t>
+        </is>
+      </c>
+      <c r="E1109" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1109" t="inlineStr">
+        <is>
+          <t>huò zhēn jià shí</t>
+        </is>
+      </c>
+      <c r="G1109" t="inlineStr">
+        <is>
+          <t>품질이 확실하고 가격이 아깝지 않은 진짜배기</t>
+        </is>
+      </c>
+      <c r="H1109" t="inlineStr">
+        <is>
+          <t>명품 캐리어 추천 글에서 외부 충격에 강하고 내구성이 뛰어난 진짜 믿고 살 수 있는 고품질 제품임을 보증할 때 씁니다.</t>
+        </is>
+      </c>
+      <c r="I1109" t="inlineStr">
+        <is>
+          <t>这款行李箱选用航空级材质，绝对是货真价实的良心产品。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="inlineStr">
+        <is>
+          <t>CHI-20260911-003</t>
+        </is>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C1110" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1110" t="inlineStr">
+        <is>
+          <t>做表面功夫</t>
+        </is>
+      </c>
+      <c r="E1110" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1110" t="inlineStr">
+        <is>
+          <t>zuò biǎomiàn gōngfu</t>
+        </is>
+      </c>
+      <c r="G1110" t="inlineStr">
+        <is>
+          <t>겉치레만 하다, 생색만 내고 실속은 없다</t>
+        </is>
+      </c>
+      <c r="H1110" t="inlineStr">
+        <is>
+          <t>친환경 생태 보존을 외치면서 실상은 홍보용 만화나 보여주기식 이벤트에만 치중하고 실제 현장 관리는 등한시하는 행태를 꼬집습니다.</t>
+        </is>
+      </c>
+      <c r="I1110" t="inlineStr">
+        <is>
+          <t>我们做企业环保不能光做表面功夫，必须把排污治理落到实处。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="inlineStr">
+        <is>
+          <t>CHI-20260911-004</t>
+        </is>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1111" t="inlineStr">
+        <is>
+          <t>砸锅卖铁</t>
+        </is>
+      </c>
+      <c r="E1111" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1111" t="inlineStr">
+        <is>
+          <t>zá guō mài tiě</t>
+        </is>
+      </c>
+      <c r="G1111" t="inlineStr">
+        <is>
+          <t>모든 가산을 털어서라도 돈을 마련하다, 전력을 다하다</t>
+        </is>
+      </c>
+      <c r="H1111" t="inlineStr">
+        <is>
+          <t>가난한 집안 형편 속에서도 자녀의 대학교육이나 사업 자금 마련을 위해 모든 것을 아낌없이 쏟아붓는 절박하고 헌신적인 부모의 마음을 묘사할 때 사용합니다.</t>
+        </is>
+      </c>
+      <c r="I1111" t="inlineStr">
+        <is>
+          <t>为了供儿子出国留学，父母就算砸锅卖铁也在所不惜。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>CHI-20260911-005</t>
+        </is>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1112" t="inlineStr">
+        <is>
+          <t>不合群</t>
+        </is>
+      </c>
+      <c r="E1112" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1112" t="inlineStr">
+        <is>
+          <t>bù hé qún</t>
+        </is>
+      </c>
+      <c r="G1112" t="inlineStr">
+        <is>
+          <t>남들과 어울리지 못하다, 독고다이로 행동하다</t>
+        </is>
+      </c>
+      <c r="H1112" t="inlineStr">
+        <is>
+          <t>명문대 졸업 후 남들이 부러워하는 고연봉 직군을 뒤로하고 홀로 조용히 서점을 운영하는 독특하고 개성 있는 삶을 선택한 인물을 바라보는 주변의 시선입니다.</t>
+        </is>
+      </c>
+      <c r="I1112" t="inlineStr">
+        <is>
+          <t>他性格比较内向，平时在班里显得有点不合群。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>CHI-20260911-006</t>
+        </is>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1113" t="inlineStr">
+        <is>
+          <t>半吊子</t>
+        </is>
+      </c>
+      <c r="E1113" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1113" t="inlineStr">
+        <is>
+          <t>bàn diào zi</t>
+        </is>
+      </c>
+      <c r="G1113" t="inlineStr">
+        <is>
+          <t>어설픈 지식을 가진 사람, 선무당</t>
+        </is>
+      </c>
+      <c r="H1113" t="inlineStr">
+        <is>
+          <t>환경 보호나 첨단 기술의 겉핥기식 개념만 알고 있으면서 실제 현장 업무나 깊이 있는 학업에서는 무지함이 낱낱이 드러나는 이들을 일컫는 표현입니다.</t>
+        </is>
+      </c>
+      <c r="I1113" t="inlineStr">
+        <is>
+          <t>别听那个半吊子瞎指挥，他根本不懂技术。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="inlineStr">
+        <is>
+          <t>CHI-20260911-007</t>
+        </is>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1114" t="inlineStr">
+        <is>
+          <t>博人眼球</t>
+        </is>
+      </c>
+      <c r="E1114" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1114" t="inlineStr">
+        <is>
+          <t>bó rén yǎn qiú</t>
+        </is>
+      </c>
+      <c r="G1114" t="inlineStr">
+        <is>
+          <t>이목을 끌다, 관심을 유도하다</t>
+        </is>
+      </c>
+      <c r="H1114" t="inlineStr">
+        <is>
+          <t>패션쇼에서 예술성이나 실용성보다는 대중의 흥미를 유발하고 트렌디하게 보이기 위해 연출한 화려하고 기발한 퍼포먼스를 가리킵니다.</t>
+        </is>
+      </c>
+      <c r="I1114" t="inlineStr">
+        <is>
+          <t>现在很多网红为了博人眼球，故意在直播间里做些出格的事。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="inlineStr">
+        <is>
+          <t>CHI-20260911-008</t>
+        </is>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1115" t="inlineStr">
+        <is>
+          <t>不入流</t>
+        </is>
+      </c>
+      <c r="E1115" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1115" t="inlineStr">
+        <is>
+          <t>bù rù liú</t>
+        </is>
+      </c>
+      <c r="G1115" t="inlineStr">
+        <is>
+          <t>급이 떨어지다, 삼류다, 주류에 끼지 못하다</t>
+        </is>
+      </c>
+      <c r="H1115" t="inlineStr">
+        <is>
+          <t>고급 여행용 가방 시장에서 허술한 마감과 낮은 내구성으로 명품 경쟁에서 아예 밀려나 버린 저가 모조품이나 삼류 브랜드를 평가할 때 씁니다.</t>
+        </is>
+      </c>
+      <c r="I1115" t="inlineStr">
+        <is>
+          <t>那种粗制滥造的山寨货，在高端市场根本就不入流。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>CHI-20260911-009</t>
+        </is>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1116" t="inlineStr">
+        <is>
+          <t>跌破眼镜</t>
+        </is>
+      </c>
+      <c r="E1116" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1116" t="inlineStr">
+        <is>
+          <t>diē pò yǎn jìng</t>
+        </is>
+      </c>
+      <c r="G1116" t="inlineStr">
+        <is>
+          <t>크게 놀라다, 예상을 뒤엎다, 어안이 벙벙하다</t>
+        </is>
+      </c>
+      <c r="H1116" t="inlineStr">
+        <is>
+          <t>高考数学得132分的人，开学考试竟然只得了12分，真是让人跌破眼镜。</t>
+        </is>
+      </c>
+      <c r="I1116" t="inlineStr">
+        <is>
+          <t>那个一向不被看好的创业公司竟然拿到了巨额投资，让所有业内人士都跌破眼镜。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>CHI-20260911-010</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1117" t="inlineStr">
+        <is>
+          <t>落到实处</t>
+        </is>
+      </c>
+      <c r="E1117" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1117" t="inlineStr">
+        <is>
+          <t>luò dào shí chù</t>
+        </is>
+      </c>
+      <c r="G1117" t="inlineStr">
+        <is>
+          <t>실천으로 옮기다, 구체적으로 실행하다</t>
+        </is>
+      </c>
+      <c r="H1117" t="inlineStr">
+        <is>
+          <t>只有把环保政策落到实处，才能真正改善我们的生活环境。</t>
+        </is>
+      </c>
+      <c r="I1117" t="inlineStr">
+        <is>
+          <t>会议上讨论的方案再好，如果不落到实处，也只是纸上谈兵。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>CHI-20260911-011</t>
+        </is>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1118" t="inlineStr">
+        <is>
+          <t>伸出援手</t>
+        </is>
+      </c>
+      <c r="E1118" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1118" t="inlineStr">
+        <is>
+          <t>shēn chū yuán shǒu</t>
+        </is>
+      </c>
+      <c r="G1118" t="inlineStr">
+        <is>
+          <t>도움의 손길을 내밀다, 지원하다</t>
+        </is>
+      </c>
+      <c r="H1118" t="inlineStr">
+        <is>
+          <t>中方愿根据尼方需要，在灾后重建中积极伸出援手。</t>
+        </is>
+      </c>
+      <c r="I1118" t="inlineStr">
+        <is>
+          <t>邻国发生地震后，许多国际组织纷纷伸出援手，提供救援物资。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>CHI-20260911-012</t>
+        </is>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1119" t="inlineStr">
+        <is>
+          <t>针锋相对</t>
+        </is>
+      </c>
+      <c r="E1119" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1119" t="inlineStr">
+        <is>
+          <t>zhēn fēng xiāng duì</t>
+        </is>
+      </c>
+      <c r="G1119" t="inlineStr">
+        <is>
+          <t>한 치의 양보도 없이 팽팽히 맞서다, 침과 끝이 맞서다</t>
+        </is>
+      </c>
+      <c r="H1119" t="inlineStr">
+        <is>
+          <t>面对外部势力的无理干涉，外交部发言人的表态针锋相对，立场坚定。</t>
+        </is>
+      </c>
+      <c r="I1119" t="inlineStr">
+        <is>
+          <t>在今天的辩论赛上，双方辩友针锋相对，现场气氛十分紧张。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>CHI-20260911-013</t>
+        </is>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1120" t="inlineStr">
+        <is>
+          <t>经得起</t>
+        </is>
+      </c>
+      <c r="E1120" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1120" t="inlineStr">
+        <is>
+          <t>jīng de qǐ</t>
+        </is>
+      </c>
+      <c r="G1120" t="inlineStr">
+        <is>
+          <t>견뎌 내다, 감당하다, 시험을 통과하다</t>
+        </is>
+      </c>
+      <c r="H1120" t="inlineStr">
+        <is>
+          <t>高端行李箱必须要经得起高强度的抗撞击测试，才能推向市场。</t>
+        </is>
+      </c>
+      <c r="I1120" t="inlineStr">
+        <is>
+          <t>我们的产品质量经得起时间的检验，请客户放心购买。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>CHI-20260911-014</t>
+        </is>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1121" t="inlineStr">
+        <is>
+          <t>有板有眼</t>
+        </is>
+      </c>
+      <c r="E1121" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1121" t="inlineStr">
+        <is>
+          <t>yǒu bǎn yǒu yǎn</t>
+        </is>
+      </c>
+      <c r="G1121" t="inlineStr">
+        <is>
+          <t>조리 있고 짜임새가 있다, 규칙적이고 빈틈이 없다</t>
+        </is>
+      </c>
+      <c r="H1121" t="inlineStr">
+        <is>
+          <t>那个区人大把“走进人大”活动组织得有板有眼，推进得非常系统。</t>
+        </is>
+      </c>
+      <c r="I1121" t="inlineStr">
+        <is>
+          <t>虽然是第一次主持大型活动，但他的发言有板有眼，非常有大将之风。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>CHI-20260911-015</t>
+        </is>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1122" t="inlineStr">
+        <is>
+          <t>顺藤摸瓜</t>
+        </is>
+      </c>
+      <c r="E1122" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1122" t="inlineStr">
+        <is>
+          <t>shùn téng mō guā</t>
+        </is>
+      </c>
+      <c r="G1122" t="inlineStr">
+        <is>
+          <t>덩굴을 따라가며 오이를 찾다, 단서를 추적하여 사건의 전모를 밝혀내다</t>
+        </is>
+      </c>
+      <c r="H1122" t="inlineStr">
+        <is>
+          <t>监管部门通过视察村级资产，顺藤摸瓜发现了资金管理的深层隐患。</t>
+        </is>
+      </c>
+      <c r="I1122" t="inlineStr">
+        <is>
+          <t>警方根据嫌疑人留下的微小线索，顺藤摸瓜，终于抓获了幕后主使。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-14 | 1132/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1122"/>
+  <dimension ref="A1:I1133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53150,6 +53150,523 @@
         </is>
       </c>
     </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>CHI-20260914-001</t>
+        </is>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1123" t="inlineStr">
+        <is>
+          <t>不甘心</t>
+        </is>
+      </c>
+      <c r="E1123" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1123" t="inlineStr">
+        <is>
+          <t>bù gān xīn</t>
+        </is>
+      </c>
+      <c r="G1123" t="inlineStr">
+        <is>
+          <t>미련이 남다, 단념할 수 없다 (아쉬움이 커서 포기하지 못함)</t>
+        </is>
+      </c>
+      <c r="H1123" t="inlineStr">
+        <is>
+          <t>베이징대에 합격하고도 아쉬움에 등록을 포기했던 학생은 '단념할 수 없어(不甘心)' 올해 다시 한번 시험을 치렀다.</t>
+        </is>
+      </c>
+      <c r="I1123" t="inlineStr">
+        <is>
+          <t>已经坚持了这么久，现在放弃我真的很不甘心。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>CHI-20260914-002</t>
+        </is>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1124" t="inlineStr">
+        <is>
+          <t>做工作</t>
+        </is>
+      </c>
+      <c r="E1124" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1124" t="inlineStr">
+        <is>
+          <t>zuò gōng zuò</t>
+        </is>
+      </c>
+      <c r="G1124" t="inlineStr">
+        <is>
+          <t>설득하다, 마음을 움직이려 공을 들이다 (대화를 통해 상대방을 설득함)</t>
+        </is>
+      </c>
+      <c r="H1124" t="inlineStr">
+        <is>
+          <t>지역 주민들의 생생한 법안 의견을 조율하기 위해 주민 대표들이 일일이 가정을 방문하며 열심히 '설득 작업(做工作)'을 펼쳤다.</t>
+        </is>
+      </c>
+      <c r="I1124" t="inlineStr">
+        <is>
+          <t>小王想离职，经理正在办公室里给他做工作呢。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>CHI-20260914-003</t>
+        </is>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1125" t="inlineStr">
+        <is>
+          <t>白费劲</t>
+        </is>
+      </c>
+      <c r="E1125" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1125" t="inlineStr">
+        <is>
+          <t>bái fèi jìn</t>
+        </is>
+      </c>
+      <c r="G1125" t="inlineStr">
+        <is>
+          <t>헛수고하다, 괜히 힘만 빼다</t>
+        </is>
+      </c>
+      <c r="H1125" t="inlineStr">
+        <is>
+          <t>사전에 정밀한 조사나 철저한 대책 수립이 수반되지 않는다면, 환경 정비 사업도 결국 '괜한 헛수고(白费劲)'로 끝날 우려가 크다.</t>
+        </is>
+      </c>
+      <c r="I1125" t="inlineStr">
+        <is>
+          <t>如果基础没打好，后面再怎么努力也是白费劲。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>CHI-20260914-004</t>
+        </is>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1126" t="inlineStr">
+        <is>
+          <t>想得开</t>
+        </is>
+      </c>
+      <c r="E1126" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1126" t="inlineStr">
+        <is>
+          <t>xiǎng de kāi</t>
+        </is>
+      </c>
+      <c r="G1126" t="inlineStr">
+        <is>
+          <t>마음을 털어버리다, 낙천적으로 생각하다, 구애받지 않다</t>
+        </is>
+      </c>
+      <c r="H1126" t="inlineStr">
+        <is>
+          <t>아들이 최고 명문대를 포기하고 1년을 더 공부하겠다고 나섰을 때, 부모가 '마음을 너그럽게 비우고(想得开)' 지지해 준 덕에 다시 도전할 수 있었다.</t>
+        </is>
+      </c>
+      <c r="I1126" t="inlineStr">
+        <is>
+          <t>事情既然已经发生了，你想得开一些，日子还得往前看。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>CHI-20260914-005</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1127" t="inlineStr">
+        <is>
+          <t>不当回事</t>
+        </is>
+      </c>
+      <c r="E1127" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1127" t="inlineStr">
+        <is>
+          <t>bù dàng huí shì</t>
+        </is>
+      </c>
+      <c r="G1127" t="inlineStr">
+        <is>
+          <t>대수롭지 않게 여기다, 귓등으로 흘리다, 가볍게 보다</t>
+        </is>
+      </c>
+      <c r="H1127" t="inlineStr">
+        <is>
+          <t>정부나 외교부가 발표하는 긴급 위험 경보를 '가볍게 여기고 무시했다가는(不当回事)' 예기치 못한 안전사고에 직면할 수 있다.</t>
+        </is>
+      </c>
+      <c r="I1127" t="inlineStr">
+        <is>
+          <t>医生反复强调不能吃辛辣食物，你别总是不当回事。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>CHI-20260914-006</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1128" t="inlineStr">
+        <is>
+          <t>义不容辞</t>
+        </is>
+      </c>
+      <c r="E1128" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1128" t="inlineStr">
+        <is>
+          <t>yì bù róng cí</t>
+        </is>
+      </c>
+      <c r="G1128" t="inlineStr">
+        <is>
+          <t>도덕적이나 의리상 거절할 수 없다, 마땅히 해야 할 의무다</t>
+        </is>
+      </c>
+      <c r="H1128" t="inlineStr">
+        <is>
+          <t>解决中小企业回款难问题，央国企义不容辞。</t>
+        </is>
+      </c>
+      <c r="I1128" t="inlineStr">
+        <is>
+          <t>帮助有困难的邻居是我们义不容辞的责任。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>CHI-20260914-007</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1129" t="inlineStr">
+        <is>
+          <t>看笑话</t>
+        </is>
+      </c>
+      <c r="E1129" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1129" t="inlineStr">
+        <is>
+          <t>kàn xiào hua</t>
+        </is>
+      </c>
+      <c r="G1129" t="inlineStr">
+        <is>
+          <t>비웃다, 남의 실수를 구경거리로 삼다</t>
+        </is>
+      </c>
+      <c r="H1129" t="inlineStr">
+        <is>
+          <t>那些质疑他选择的人，最后都成了看笑话的看客。</t>
+        </is>
+      </c>
+      <c r="I1129" t="inlineStr">
+        <is>
+          <t>他顶着巨大的压力默默努力，就是不想让别人看笑话。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>CHI-20260914-008</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1130" t="inlineStr">
+        <is>
+          <t>行行出状元</t>
+        </is>
+      </c>
+      <c r="E1130" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1130" t="inlineStr">
+        <is>
+          <t>háng háng chū zhuàng yuán</t>
+        </is>
+      </c>
+      <c r="G1130" t="inlineStr">
+        <is>
+          <t>어느 분야든 열심히 노력하면 최고가 될 수 있다</t>
+        </is>
+      </c>
+      <c r="H1130" t="inlineStr">
+        <is>
+          <t>人大硕士做家政还拿了一等奖，真是行行出状元。</t>
+        </is>
+      </c>
+      <c r="I1130" t="inlineStr">
+        <is>
+          <t>别瞧不起这些普通岗位，俗话说行行出状元。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>CHI-20260914-009</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1131" t="inlineStr">
+        <is>
+          <t>无中生有</t>
+        </is>
+      </c>
+      <c r="E1131" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1131" t="inlineStr">
+        <is>
+          <t>wú zhōng shēng yǒu</t>
+        </is>
+      </c>
+      <c r="G1131" t="inlineStr">
+        <is>
+          <t>없는 사실을 지어내다, 날조하다</t>
+        </is>
+      </c>
+      <c r="H1131" t="inlineStr">
+        <is>
+          <t>省教育厅辟谣，所谓的“连放13天假”完全是无中生有。</t>
+        </is>
+      </c>
+      <c r="I1131" t="inlineStr">
+        <is>
+          <t>这篇网传报道完全是无中生有，大家千万不要相信。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>CHI-20260914-010</t>
+        </is>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1132" t="inlineStr">
+        <is>
+          <t>低调行事</t>
+        </is>
+      </c>
+      <c r="E1132" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1132" t="inlineStr">
+        <is>
+          <t>dī diào xíng shì</t>
+        </is>
+      </c>
+      <c r="G1132" t="inlineStr">
+        <is>
+          <t>낮은 자세로 일하다, 겸손하고 신중하게 행동하다</t>
+        </is>
+      </c>
+      <c r="H1132" t="inlineStr">
+        <is>
+          <t>黄晓明低调办理入学流程，展现了低调行事的态度。</t>
+        </is>
+      </c>
+      <c r="I1132" t="inlineStr">
+        <is>
+          <t>他虽然资产过亿，但平时依然开着普通车，低调行事。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>CHI-20260914-011</t>
+        </is>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1133" t="inlineStr">
+        <is>
+          <t>不约而同</t>
+        </is>
+      </c>
+      <c r="E1133" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F1133" t="inlineStr">
+        <is>
+          <t>bù yuē ér tóng</t>
+        </is>
+      </c>
+      <c r="G1133" t="inlineStr">
+        <is>
+          <t>약속이라도 한 듯이 의견이나 행동이 일치하다</t>
+        </is>
+      </c>
+      <c r="H1133" t="inlineStr">
+        <is>
+          <t>看到两千年前的“环保古灯”，大家不约而同地感叹古人的智慧。</t>
+        </is>
+      </c>
+      <c r="I1133" t="inlineStr">
+        <is>
+          <t>听到这个令人兴奋的好消息，大家不约而同地欢呼起来。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-15 | 1135/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1133"/>
+  <dimension ref="A1:I1136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53667,6 +53667,147 @@
         </is>
       </c>
     </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>CHI-20260915-001</t>
+        </is>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1134" t="inlineStr">
+        <is>
+          <t>顶呱呱</t>
+        </is>
+      </c>
+      <c r="E1134" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1134" t="inlineStr">
+        <is>
+          <t>dǐng guā guā</t>
+        </is>
+      </c>
+      <c r="G1134" t="inlineStr">
+        <is>
+          <t>최고다, 끝내주게 훌륭하다, 일류이다</t>
+        </is>
+      </c>
+      <c r="H1134" t="inlineStr">
+        <is>
+          <t>아무리 무거운 짐을 가득 싣고 던져져도 파손되지 않는 최고급 고강도 명품 캐리어의 성능을 설명하는 호평</t>
+        </is>
+      </c>
+      <c r="I1134" t="inlineStr">
+        <is>
+          <t>他不仅业务能力顶呱呱，人品在公司也是出了名的好。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>CHI-20260915-002</t>
+        </is>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1135" t="inlineStr">
+        <is>
+          <t>顺手牵羊</t>
+        </is>
+      </c>
+      <c r="E1135" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1135" t="inlineStr">
+        <is>
+          <t>顺手牵羊</t>
+        </is>
+      </c>
+      <c r="G1135" t="inlineStr">
+        <is>
+          <t>기회를 틈타 남의 물건을 슬쩍 훔쳐 가다</t>
+        </is>
+      </c>
+      <c r="H1135" t="inlineStr">
+        <is>
+          <t>车站人流密集，有些不法分子常趁学生不备，顺手牵羊拿走其行李箱。</t>
+        </is>
+      </c>
+      <c r="I1135" t="inlineStr">
+        <is>
+          <t>坐地铁时一定要看管好自己的手机，提防小偷顺手牵羊。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>CHI-20260915-003</t>
+        </is>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1136" t="inlineStr">
+        <is>
+          <t>墨守成规</t>
+        </is>
+      </c>
+      <c r="E1136" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1136" t="inlineStr">
+        <is>
+          <t>mò shǒu chéng guī</t>
+        </is>
+      </c>
+      <c r="G1136" t="inlineStr">
+        <is>
+          <t>구습을 고수하다, 융통성 없이 낡은 규정에만 얽매이다</t>
+        </is>
+      </c>
+      <c r="H1136" t="inlineStr">
+        <is>
+          <t>面对新高考改革的挑战，我们绝不能墨守成规，而要积极探索新的教学模式。</t>
+        </is>
+      </c>
+      <c r="I1136" t="inlineStr">
+        <is>
+          <t>在瞬息万变的市场中，如果只知墨守成规，企业很快就会被淘汰。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-16 | 1144/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1136"/>
+  <dimension ref="A1:I1145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53808,6 +53808,429 @@
         </is>
       </c>
     </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>CHI-20260916-001</t>
+        </is>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1137" t="inlineStr">
+        <is>
+          <t>卷铺盖</t>
+        </is>
+      </c>
+      <c r="E1137" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1137" t="inlineStr">
+        <is>
+          <t>juǎn pū gai</t>
+        </is>
+      </c>
+      <c r="G1137" t="inlineStr">
+        <is>
+          <t>짐을 싸서 떠나다, 해고당하다, 야반도주하다</t>
+        </is>
+      </c>
+      <c r="H1137" t="inlineStr">
+        <is>
+          <t>가맹 계약이나 학원비를 가로챈 사기꾼 일당이 단속을 피해 밤사이에 흔적도 없이 짐을 싸서 도망치거나, 회사에서 징계 해고를 당하는 오피스 상황</t>
+        </is>
+      </c>
+      <c r="I1137" t="inlineStr">
+        <is>
+          <t>他因为严重违反公司规定，被老板命令立刻卷铺盖走人。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>CHI-20260916-002</t>
+        </is>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1138" t="inlineStr">
+        <is>
+          <t>打成一片</t>
+        </is>
+      </c>
+      <c r="E1138" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1138" t="inlineStr">
+        <is>
+          <t>dǎ chéng yī piàn</t>
+        </is>
+      </c>
+      <c r="G1138" t="inlineStr">
+        <is>
+          <t>격의 없이 어울리다, 하나로 융화되다</t>
+        </is>
+      </c>
+      <c r="H1138" t="inlineStr">
+        <is>
+          <t>새로 전입 온 외교관이나 자원봉사자가 낯선 시골 주민들과 벽을 허물고 친형제처럼 살갑게 융화되어 소통하는 모습</t>
+        </is>
+      </c>
+      <c r="I1138" t="inlineStr">
+        <is>
+          <t>新来的总经理非常随和，很快就和基层员工打成一片了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>CHI-20260916-003</t>
+        </is>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1139" t="inlineStr">
+        <is>
+          <t>说风凉话</t>
+        </is>
+      </c>
+      <c r="E1139" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1139" t="inlineStr">
+        <is>
+          <t>shuō fēng liáng huà</t>
+        </is>
+      </c>
+      <c r="G1139" t="inlineStr">
+        <is>
+          <t>방관자처럼 빈정거리다, 무책임하게 훈수 두다</t>
+        </is>
+      </c>
+      <c r="H1139" t="inlineStr">
+        <is>
+          <t>자신은 정작 아무런 도움도 주지 않으면서 다른 사람들이 땀 흘리며 고생해서 이뤄낸 성과나 실패에 대해 뒤에서 쉽게 평가하는 이기적인 태도</t>
+        </is>
+      </c>
+      <c r="I1139" t="inlineStr">
+        <is>
+          <t>别人遇到困难时，你不帮忙也就算了，别在旁边说风凉话。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>CHI-20260916-004</t>
+        </is>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1140" t="inlineStr">
+        <is>
+          <t>豁出去</t>
+        </is>
+      </c>
+      <c r="E1140" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1140" t="inlineStr">
+        <is>
+          <t>huō chū qù</t>
+        </is>
+      </c>
+      <c r="G1140" t="inlineStr">
+        <is>
+          <t>모든 것을 내던지다, 물불 가리지 않고 달려들다</t>
+        </is>
+      </c>
+      <c r="H1140" t="inlineStr">
+        <is>
+          <t>중요한 대입 시험이나 최후의 기회를 앞두고 더 이상 물러설 곳이 없다고 생각하여 잠을 아껴가며 결사의 각오로 공부에 매진하는 상황</t>
+        </is>
+      </c>
+      <c r="I1140" t="inlineStr">
+        <is>
+          <t>为了能在这次高考中取得好成绩，我决定豁出去拼一把。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>CHI-20260916-005</t>
+        </is>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1141" t="inlineStr">
+        <is>
+          <t>心神不宁</t>
+        </is>
+      </c>
+      <c r="E1141" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1141" t="inlineStr">
+        <is>
+          <t>xīn shén bù níng</t>
+        </is>
+      </c>
+      <c r="G1141" t="inlineStr">
+        <is>
+          <t>불안하고 안절부절못하다, 집중하지 못하고 안색이 어둡다</t>
+        </is>
+      </c>
+      <c r="H1141" t="inlineStr">
+        <is>
+          <t>중요한 시험 성적 발표를 기다리거나 가족의 수술 소식을 앞두고 안절부절못하며 손에 아무것도 잡히지 않는 초조한 수험생이나 가족의 심리</t>
+        </is>
+      </c>
+      <c r="I1141" t="inlineStr">
+        <is>
+          <t>自从来听到那个不好的消息后，她整天都显得心神不宁。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>CHI-20260916-006</t>
+        </is>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1142" t="inlineStr">
+        <is>
+          <t>见义勇为</t>
+        </is>
+      </c>
+      <c r="E1142" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F1142" t="inlineStr">
+        <is>
+          <t>jiàn yì yǒng wéi</t>
+        </is>
+      </c>
+      <c r="G1142" t="inlineStr">
+        <is>
+          <t>정의를 위해 용감하게 나서다</t>
+        </is>
+      </c>
+      <c r="H1142" t="inlineStr">
+        <is>
+          <t>那个因见义勇为救人而错过高考的学子，赢得了大家的赞赏。</t>
+        </is>
+      </c>
+      <c r="I1142" t="inlineStr">
+        <is>
+          <t>面对突发的火灾，这位年轻小伙子见义勇为，冲进火场救出了邻居。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>CHI-20260916-007</t>
+        </is>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1143" t="inlineStr">
+        <is>
+          <t>不知所措</t>
+        </is>
+      </c>
+      <c r="E1143" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F1143" t="inlineStr">
+        <is>
+          <t>bù zhī suǒ cuò</t>
+        </is>
+      </c>
+      <c r="G1143" t="inlineStr">
+        <is>
+          <t>어찌할 바를 모르다, 갈팡질팡하다</t>
+        </is>
+      </c>
+      <c r="H1143" t="inlineStr">
+        <is>
+          <t>面对突发的高考安全状况，有些家长和考生显得不知所措。</t>
+        </is>
+      </c>
+      <c r="I1143" t="inlineStr">
+        <is>
+          <t>第一次面对这么大的媒体阵仗，这位年轻的创作者显得有些不知所措。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>CHI-20260916-008</t>
+        </is>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1144" t="inlineStr">
+        <is>
+          <t>竭尽全力</t>
+        </is>
+      </c>
+      <c r="E1144" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F1144" t="inlineStr">
+        <is>
+          <t>jié jìn quán lì</t>
+        </is>
+      </c>
+      <c r="G1144" t="inlineStr">
+        <is>
+          <t>온 힘을 다하다, 전력을 다하다</t>
+        </is>
+      </c>
+      <c r="H1144" t="inlineStr">
+        <is>
+          <t>为了能顺利考入理想的大学，高三学子们都在竭尽全力地拼搏。</t>
+        </is>
+      </c>
+      <c r="I1144" t="inlineStr">
+        <is>
+          <t>只要你竭尽全力去做了，不管最后结果如何，都不会留下遗憾。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>CHI-20260916-009</t>
+        </is>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1145" t="inlineStr">
+        <is>
+          <t>众所周知</t>
+        </is>
+      </c>
+      <c r="E1145" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F1145" t="inlineStr">
+        <is>
+          <t>zhòng sǒù zhōu zhī</t>
+        </is>
+      </c>
+      <c r="G1145" t="inlineStr">
+        <is>
+          <t>모두가 아는 바와 같이, 주지하다시피</t>
+        </is>
+      </c>
+      <c r="H1145" t="inlineStr">
+        <is>
+          <t>众所周知，保护生态环境是实现可持续发展的关键所在。</t>
+        </is>
+      </c>
+      <c r="I1145" t="inlineStr">
+        <is>
+          <t>众所周知，高考是改变很多普通学子命运的重要途径之一。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-17 | 1151/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1145"/>
+  <dimension ref="A1:I1152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54231,6 +54231,335 @@
         </is>
       </c>
     </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>CHI-20260917-001</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1146" t="inlineStr">
+        <is>
+          <t>不搭界</t>
+        </is>
+      </c>
+      <c r="E1146" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1146" t="inlineStr">
+        <is>
+          <t>bù dā jiè</t>
+        </is>
+      </c>
+      <c r="G1146" t="inlineStr">
+        <is>
+          <t>전혀 상관이 없다, 아무런 관련이 없다</t>
+        </is>
+      </c>
+      <c r="H1146" t="inlineStr">
+        <is>
+          <t>회사 내 조직 개편 소식에 걱정이 태산인 디자인 팀원에게 이번 인사는 우리 부서 업무와 아무런 연관이 없음을 말해주는 상황</t>
+        </is>
+      </c>
+      <c r="I1146" t="inlineStr">
+        <is>
+          <t>这次的业务调整跟我们部门根本不搭界，你不用担心会被裁员。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>CHI-20260917-002</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1147" t="inlineStr">
+        <is>
+          <t>砸饭碗</t>
+        </is>
+      </c>
+      <c r="E1147" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1147" t="inlineStr">
+        <is>
+          <t>zá fàn wǎn</t>
+        </is>
+      </c>
+      <c r="G1147" t="inlineStr">
+        <is>
+          <t>일자리를 잃다, 생계 수단(밥줄)을 끊어버리다</t>
+        </is>
+      </c>
+      <c r="H1147" t="inlineStr">
+        <is>
+          <t>오피스 환경에서 기밀 문서가 외부로 심각하게 누출되어 관련 부서 전원의 근로 계약 해지가 검토되는 위태로운 순간</t>
+        </is>
+      </c>
+      <c r="I1147" t="inlineStr">
+        <is>
+          <t>你在工作上犯下这种严重的错误，这无异于自己砸自己的饭碗。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>CHI-20260917-003</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1148" t="inlineStr">
+        <is>
+          <t>行稳致远</t>
+        </is>
+      </c>
+      <c r="E1148" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1148" t="inlineStr">
+        <is>
+          <t>xíng wěn zhì yuǎn</t>
+        </is>
+      </c>
+      <c r="G1148" t="inlineStr">
+        <is>
+          <t>기초를 튼튼히 하여 지속적이고 안정적으로 멀리 나아가다</t>
+        </is>
+      </c>
+      <c r="H1148" t="inlineStr">
+        <is>
+          <t>坚持生态优先，推动稀贵金属产业行稳致远。</t>
+        </is>
+      </c>
+      <c r="I1148" t="inlineStr">
+        <is>
+          <t>我们的创业项目不能只看眼前利益，只有稳扎稳打才能行稳致远。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>CHI-20260917-004</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1149" t="inlineStr">
+        <is>
+          <t>说漏嘴</t>
+        </is>
+      </c>
+      <c r="E1149" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1149" t="inlineStr">
+        <is>
+          <t>shuō lòu zuǐ</t>
+        </is>
+      </c>
+      <c r="G1149" t="inlineStr">
+        <is>
+          <t>말실수를 하여 무심결에 비밀을 털어놓다</t>
+        </is>
+      </c>
+      <c r="H1149" t="inlineStr">
+        <is>
+          <t>外交官在正式的外交谈判场合中说话要格外谨慎，绝不能说漏嘴。</t>
+        </is>
+      </c>
+      <c r="I1149" t="inlineStr">
+        <is>
+          <t>我们本想瞒着他准备一场惊喜派对，结果小张在聚餐时说漏嘴了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>CHI-20260917-005</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1150" t="inlineStr">
+        <is>
+          <t>唱主角</t>
+        </is>
+      </c>
+      <c r="E1150" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1150" t="inlineStr">
+        <is>
+          <t>chàng zhǔ jué</t>
+        </is>
+      </c>
+      <c r="G1150" t="inlineStr">
+        <is>
+          <t>가장 중요한 핵심적인 역할을 맡아 극을 이끌어가다</t>
+        </is>
+      </c>
+      <c r="H1150" t="inlineStr">
+        <is>
+          <t>在构建未来的新型食品供应链中，屋顶农场和生态科技将唱主角。</t>
+        </is>
+      </c>
+      <c r="I1150" t="inlineStr">
+        <is>
+          <t>在本次的中非合作洽谈中，环保和可持续发展议题唱起了主角。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>CHI-20260917-006</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1151" t="inlineStr">
+        <is>
+          <t>闭门造车</t>
+        </is>
+      </c>
+      <c r="E1151" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1151" t="inlineStr">
+        <is>
+          <t>bì mén zào chē</t>
+        </is>
+      </c>
+      <c r="G1151" t="inlineStr">
+        <is>
+          <t>실제 현실을 고려하지 않고 자기 생각만으로 허황되게 일하다</t>
+        </is>
+      </c>
+      <c r="H1151" t="inlineStr">
+        <is>
+          <t>推进环保和畜禽养殖治理工作要实地考察，绝不能闭门造车。</t>
+        </is>
+      </c>
+      <c r="I1151" t="inlineStr">
+        <is>
+          <t>做市场调研必须要深入消费者群体，待在办公室里闭门造车是没有前途的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>CHI-20260917-007</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1152" t="inlineStr">
+        <is>
+          <t>莫逆之交</t>
+        </is>
+      </c>
+      <c r="E1152" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1152" t="inlineStr">
+        <is>
+          <t>mò nì zhī jiāo</t>
+        </is>
+      </c>
+      <c r="G1152" t="inlineStr">
+        <is>
+          <t>서로 허물이 없고 뜻이 아주 잘 통하는 막역한 친구 사이</t>
+        </is>
+      </c>
+      <c r="H1152" t="inlineStr">
+        <is>
+          <t>两家友好单位通过多年的深度合作，如今已经成为了莫逆之交。</t>
+        </is>
+      </c>
+      <c r="I1152" t="inlineStr">
+        <is>
+          <t>他们俩在大学时期就一同创业，经历重重风雨，早已是莫逆之交。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-18 | 1155/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1152"/>
+  <dimension ref="A1:I1156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54560,6 +54560,194 @@
         </is>
       </c>
     </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>CHI-20260918-001</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1153" t="inlineStr">
+        <is>
+          <t>卷走</t>
+        </is>
+      </c>
+      <c r="E1153" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1153" t="inlineStr">
+        <is>
+          <t>juǎn zǒu</t>
+        </is>
+      </c>
+      <c r="G1153" t="inlineStr">
+        <is>
+          <t>돈이나 물건을 몽땅 챙겨 달아나다, 먹튀하다</t>
+        </is>
+      </c>
+      <c r="H1153" t="inlineStr">
+        <is>
+          <t>高考报名头部主播卷走700名家长近2000万元学费，引发社会广泛关注。</t>
+        </is>
+      </c>
+      <c r="I1153" t="inlineStr">
+        <is>
+          <t>那个合伙人卷走公司账上所有的流动资金后就失联了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>CHI-20260918-002</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1154" t="inlineStr">
+        <is>
+          <t>拉后腿</t>
+        </is>
+      </c>
+      <c r="E1154" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1154" t="inlineStr">
+        <is>
+          <t>lā hòu tuǐ</t>
+        </is>
+      </c>
+      <c r="G1154" t="inlineStr">
+        <is>
+          <t>발목을 잡다, 지장을 주다</t>
+        </is>
+      </c>
+      <c r="H1154" t="inlineStr">
+        <is>
+          <t>全员全力治污攻坚，决不允许任何部门在落实环保责任时拉后腿。</t>
+        </is>
+      </c>
+      <c r="I1154" t="inlineStr">
+        <is>
+          <t>大家都在加班加点赶进度，你可千万不要在这个时候拉后腿。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>CHI-20260918-003</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1155" t="inlineStr">
+        <is>
+          <t>打掩护</t>
+        </is>
+      </c>
+      <c r="E1155" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1155" t="inlineStr">
+        <is>
+          <t>dǎ yǎn hù</t>
+        </is>
+      </c>
+      <c r="G1155" t="inlineStr">
+        <is>
+          <t>엄호하다, 둘러대어 숨겨주다</t>
+        </is>
+      </c>
+      <c r="H1155" t="inlineStr">
+        <is>
+          <t>某些涉案机构打着高考升学指导的幌子，实际上是为非法集资打掩护。</t>
+        </is>
+      </c>
+      <c r="I1155" t="inlineStr">
+        <is>
+          <t>昨天下午我提前溜出去办私事，全靠小李在主管面前替我打掩护。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>CHI-20260918-004</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1156" t="inlineStr">
+        <is>
+          <t>拿得起放得下</t>
+        </is>
+      </c>
+      <c r="E1156" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1156" t="inlineStr">
+        <is>
+          <t>ná de qǐ fàng de xià</t>
+        </is>
+      </c>
+      <c r="G1156" t="inlineStr">
+        <is>
+          <t>대범하고 결단력 있다, 집착하지 않고 초연하게 대처하다</t>
+        </is>
+      </c>
+      <c r="H1156" t="inlineStr">
+        <is>
+          <t>面对高考失利，这位年轻的学子展现出了拿得起放得下的开阔胸怀。</t>
+        </is>
+      </c>
+      <c r="I1156" t="inlineStr">
+        <is>
+          <t>做生意有输有赢，我们要拿得起放得下，才能走得更远。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-21 | 1164/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1156"/>
+  <dimension ref="A1:I1165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54748,6 +54748,429 @@
         </is>
       </c>
     </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>CHI-20260921-001</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1157" t="inlineStr">
+        <is>
+          <t>扬帆起航</t>
+        </is>
+      </c>
+      <c r="E1157" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1157" t="inlineStr">
+        <is>
+          <t>yáng fān qǐ háng</t>
+        </is>
+      </c>
+      <c r="G1157" t="inlineStr">
+        <is>
+          <t>돛을 올리고 출항하다, 새로운 목표나 여정을 향해 힘차게 출발하다</t>
+        </is>
+      </c>
+      <c r="H1157" t="inlineStr">
+        <is>
+          <t>上海市城管执法系统扬帆起航正当时，共绘城管新篇章。</t>
+        </is>
+      </c>
+      <c r="I1157" t="inlineStr">
+        <is>
+          <t>新项目正式启动，大家准备好扬帆起航了吗？</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>CHI-20260921-002</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1158" t="inlineStr">
+        <is>
+          <t>划得来</t>
+        </is>
+      </c>
+      <c r="E1158" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1158" t="inlineStr">
+        <is>
+          <t>huá de lái</t>
+        </is>
+      </c>
+      <c r="G1158" t="inlineStr">
+        <is>
+          <t>수지가 맞다, 이득이다, 해볼 만하다</t>
+        </is>
+      </c>
+      <c r="H1158" t="inlineStr">
+        <is>
+          <t>鸡腿才1元一个，9.5元能吃三个菜，怎么算都划得来。</t>
+        </is>
+      </c>
+      <c r="I1158" t="inlineStr">
+        <is>
+          <t>买打折年卡每天只要两块钱，划得来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>CHI-20260921-003</t>
+        </is>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1159" t="inlineStr">
+        <is>
+          <t>划不来</t>
+        </is>
+      </c>
+      <c r="E1159" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1159" t="inlineStr">
+        <is>
+          <t>huá bu lái</t>
+        </is>
+      </c>
+      <c r="G1159" t="inlineStr">
+        <is>
+          <t>손해다, 수지가 안 맞다, 밑지는 장사다</t>
+        </is>
+      </c>
+      <c r="H1159" t="inlineStr">
+        <is>
+          <t>为了一点补贴跑那么远办手续，真划不来。</t>
+        </is>
+      </c>
+      <c r="I1159" t="inlineStr">
+        <is>
+          <t>为了省几块钱排队两小时，实在划不来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>CHI-20260921-004</t>
+        </is>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1160" t="inlineStr">
+        <is>
+          <t>互学互鉴</t>
+        </is>
+      </c>
+      <c r="E1160" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1160" t="inlineStr">
+        <is>
+          <t>hù xué hù jiàn</t>
+        </is>
+      </c>
+      <c r="G1160" t="inlineStr">
+        <is>
+          <t>서로 배우고 참고하다, 상호 벤치마킹하다</t>
+        </is>
+      </c>
+      <c r="H1160" t="inlineStr">
+        <is>
+          <t>在滇台企代表走进国企交流，互学互鉴共寻合作新空间。</t>
+        </is>
+      </c>
+      <c r="I1160" t="inlineStr">
+        <is>
+          <t>两个研发团队定期交流技术，互学互鉴共同进步。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>CHI-20260921-005</t>
+        </is>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1161" t="inlineStr">
+        <is>
+          <t>咬咬牙</t>
+        </is>
+      </c>
+      <c r="E1161" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1161" t="inlineStr">
+        <is>
+          <t>yǎo yǎo yá</t>
+        </is>
+      </c>
+      <c r="G1161" t="inlineStr">
+        <is>
+          <t>이를 악물다, 꾹 참고 버티다</t>
+        </is>
+      </c>
+      <c r="H1161" t="inlineStr">
+        <is>
+          <t>课业压力虽然大，但只要咬咬牙，难关总会过去的。</t>
+        </is>
+      </c>
+      <c r="I1161" t="inlineStr">
+        <is>
+          <t>再咬咬牙坚持最后半个小时，我们就能交差了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>CHI-20260921-006</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1162" t="inlineStr">
+        <is>
+          <t>摸得着</t>
+        </is>
+      </c>
+      <c r="E1162" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1162" t="inlineStr">
+        <is>
+          <t>mō de zháo</t>
+        </is>
+      </c>
+      <c r="G1162" t="inlineStr">
+        <is>
+          <t>손에 닿다, 피부로 체감할 수 있다, 실질적이다</t>
+        </is>
+      </c>
+      <c r="H1162" t="inlineStr">
+        <is>
+          <t>城市治理不仅要有力度，更要让市民感受到看得见、摸得着的温度。</t>
+        </is>
+      </c>
+      <c r="I1162" t="inlineStr">
+        <is>
+          <t>提高员工福利必须是摸得着的实惠，而不是空头支票。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>CHI-20260921-007</t>
+        </is>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1163" t="inlineStr">
+        <is>
+          <t>见成效</t>
+        </is>
+      </c>
+      <c r="E1163" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1163" t="inlineStr">
+        <is>
+          <t>jiàn chéng xiào</t>
+        </is>
+      </c>
+      <c r="G1163" t="inlineStr">
+        <is>
+          <t>성과를 거두다, 효과를 보다</t>
+        </is>
+      </c>
+      <c r="H1163" t="inlineStr">
+        <is>
+          <t>智慧监管上线几个月就初见成效，食品安全投诉大幅下降。</t>
+        </is>
+      </c>
+      <c r="I1163" t="inlineStr">
+        <is>
+          <t>新政策推行不久便初见成效，市民纷纷点赞。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>CHI-20260921-008</t>
+        </is>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1164" t="inlineStr">
+        <is>
+          <t>打基础</t>
+        </is>
+      </c>
+      <c r="E1164" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1164" t="inlineStr">
+        <is>
+          <t>dǎ jī chǔ</t>
+        </is>
+      </c>
+      <c r="G1164" t="inlineStr">
+        <is>
+          <t>기반을 다지다, 기초를 놓다</t>
+        </is>
+      </c>
+      <c r="H1164" t="inlineStr">
+        <is>
+          <t>开学的军事训练和德育课，正是给年轻人踏入社会打基础。</t>
+        </is>
+      </c>
+      <c r="I1164" t="inlineStr">
+        <is>
+          <t>大学本科阶段主要任务就是把专业知识打好基础。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="inlineStr">
+        <is>
+          <t>CHI-20260921-009</t>
+        </is>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1165" t="inlineStr">
+        <is>
+          <t>放宽心</t>
+        </is>
+      </c>
+      <c r="E1165" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1165" t="inlineStr">
+        <is>
+          <t>fàng kuān xīn</t>
+        </is>
+      </c>
+      <c r="G1165" t="inlineStr">
+        <is>
+          <t>안심하다, 마음을 푹 놓다</t>
+        </is>
+      </c>
+      <c r="H1165" t="inlineStr">
+        <is>
+          <t>食堂采购全程有智慧监管追溯，家长们尽管放宽心。</t>
+        </is>
+      </c>
+      <c r="I1165" t="inlineStr">
+        <is>
+          <t>手术很顺利，医生说恢复得好，你就放宽心吧。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-22 | 1174/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1165"/>
+  <dimension ref="A1:I1175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55171,6 +55171,476 @@
         </is>
       </c>
     </row>
+    <row r="1166">
+      <c r="A1166" t="inlineStr">
+        <is>
+          <t>CHI-20260922-001</t>
+        </is>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1166" t="inlineStr">
+        <is>
+          <t>投简历</t>
+        </is>
+      </c>
+      <c r="E1166" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1166" t="inlineStr">
+        <is>
+          <t>tóu jiǎn lì</t>
+        </is>
+      </c>
+      <c r="G1166" t="inlineStr">
+        <is>
+          <t>이력서를 제출하다, 지원서를 넣다</t>
+        </is>
+      </c>
+      <c r="H1166" t="inlineStr">
+        <is>
+          <t>秋招开始了，大批应届毕业生开始在各个招聘会上投简历。</t>
+        </is>
+      </c>
+      <c r="I1166" t="inlineStr">
+        <is>
+          <t>为了早点拿到录取通知，我昨天在网上投了十几份简历。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="inlineStr">
+        <is>
+          <t>CHI-20260922-002</t>
+        </is>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1167" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1167" t="inlineStr">
+        <is>
+          <t>合胃口</t>
+        </is>
+      </c>
+      <c r="E1167" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1167" t="inlineStr">
+        <is>
+          <t>hé wèi kǒu</t>
+        </is>
+      </c>
+      <c r="G1167" t="inlineStr">
+        <is>
+          <t>입맛에 맞다, (일, 사람 등이) 취향에 맞다</t>
+        </is>
+      </c>
+      <c r="H1167" t="inlineStr">
+        <is>
+          <t>学校食堂推出的一元鸡腿和特惠菜，非常合学生的胃口。</t>
+        </is>
+      </c>
+      <c r="I1167" t="inlineStr">
+        <is>
+          <t>这家川菜馆的味道非常合我的胃口，我每个周末都来吃。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" t="inlineStr">
+        <is>
+          <t>CHI-20260922-003</t>
+        </is>
+      </c>
+      <c r="B1168" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1168" t="inlineStr">
+        <is>
+          <t>赶时髦</t>
+        </is>
+      </c>
+      <c r="E1168" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1168" t="inlineStr">
+        <is>
+          <t>gǎn shí máo</t>
+        </is>
+      </c>
+      <c r="G1168" t="inlineStr">
+        <is>
+          <t>유행을 좇다, 트렌드를 따르다</t>
+        </is>
+      </c>
+      <c r="H1168" t="inlineStr">
+        <is>
+          <t>现在年轻人都喜欢赶时髦，追求新潮的生活方式。</t>
+        </is>
+      </c>
+      <c r="I1168" t="inlineStr">
+        <is>
+          <t>现在的智能手机功能都差不多，没必要为了赶时髦年年换新。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" t="inlineStr">
+        <is>
+          <t>CHI-20260922-004</t>
+        </is>
+      </c>
+      <c r="B1169" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1169" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1169" t="inlineStr">
+        <is>
+          <t>丢面子</t>
+        </is>
+      </c>
+      <c r="E1169" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1169" t="inlineStr">
+        <is>
+          <t>diū miàn zi</t>
+        </is>
+      </c>
+      <c r="G1169" t="inlineStr">
+        <is>
+          <t>체면을 구기다, 창피를 당하다</t>
+        </is>
+      </c>
+      <c r="H1169" t="inlineStr">
+        <is>
+          <t>在公开场合做错事，觉得很丢面子。</t>
+        </is>
+      </c>
+      <c r="I1169" t="inlineStr">
+        <is>
+          <t>输掉比赛固然难过，但只要尽力了，就一点也不丢面子。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" t="inlineStr">
+        <is>
+          <t>CHI-20260922-005</t>
+        </is>
+      </c>
+      <c r="B1170" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1170" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1170" t="inlineStr">
+        <is>
+          <t>意气风发</t>
+        </is>
+      </c>
+      <c r="E1170" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1170" t="inlineStr">
+        <is>
+          <t>yì qì fēng fā</t>
+        </is>
+      </c>
+      <c r="G1170" t="inlineStr">
+        <is>
+          <t>의기양양하다, 활기가 넘치다, 기세가 드높다</t>
+        </is>
+      </c>
+      <c r="H1170" t="inlineStr">
+        <is>
+          <t>校园里满是意气风发的新生，朝气蓬勃。</t>
+        </is>
+      </c>
+      <c r="I1170" t="inlineStr">
+        <is>
+          <t>看着那些意气风发的大学毕业生，我仿佛看到了当年的自己。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" t="inlineStr">
+        <is>
+          <t>CHI-20260922-006</t>
+        </is>
+      </c>
+      <c r="B1171" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1171" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1171" t="inlineStr">
+        <is>
+          <t>根深蒂固</t>
+        </is>
+      </c>
+      <c r="E1171" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1171" t="inlineStr">
+        <is>
+          <t>gēn shēn dì gù</t>
+        </is>
+      </c>
+      <c r="G1171" t="inlineStr">
+        <is>
+          <t>뿌리가 깊어 쉽게 흔들리지 않다, 뿌리 깊다</t>
+        </is>
+      </c>
+      <c r="H1171" t="inlineStr">
+        <is>
+          <t>环保理念要在大家心中根深蒂固，需要长期的宣传。</t>
+        </is>
+      </c>
+      <c r="I1171" t="inlineStr">
+        <is>
+          <t>这种重男轻女的陈旧观念在一些地区仍然根深蒂固。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" t="inlineStr">
+        <is>
+          <t>CHI-20260922-007</t>
+        </is>
+      </c>
+      <c r="B1172" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1172" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1172" t="inlineStr">
+        <is>
+          <t>互惠互利</t>
+        </is>
+      </c>
+      <c r="E1172" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1172" t="inlineStr">
+        <is>
+          <t>hù huì hù lì</t>
+        </is>
+      </c>
+      <c r="G1172" t="inlineStr">
+        <is>
+          <t>상호 혜택과 이익을 나누다, 상호 호혜적이다</t>
+        </is>
+      </c>
+      <c r="H1172" t="inlineStr">
+        <is>
+          <t>双方本着互惠互利的原则，达成了长期合作。</t>
+        </is>
+      </c>
+      <c r="I1172" t="inlineStr">
+        <is>
+          <t>国际贸易的本质应该是互惠互利，而不是单方面受损。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" t="inlineStr">
+        <is>
+          <t>CHI-20260922-008</t>
+        </is>
+      </c>
+      <c r="B1173" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1173" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1173" t="inlineStr">
+        <is>
+          <t>畅所欲言</t>
+        </is>
+      </c>
+      <c r="E1173" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1173" t="inlineStr">
+        <is>
+          <t>chàng suǒ yù yán</t>
+        </is>
+      </c>
+      <c r="G1173" t="inlineStr">
+        <is>
+          <t>마음껏 의견을 개진하다, 하고 싶은 말을 다 하다</t>
+        </is>
+      </c>
+      <c r="H1173" t="inlineStr">
+        <is>
+          <t>在这次座谈会上，大家可以畅所欲言，提出宝贵意见。</t>
+        </is>
+      </c>
+      <c r="I1173" t="inlineStr">
+        <is>
+          <t>今天的讨论会气氛很轻松，大家都可以畅所欲言，不用有什么顾虑。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" t="inlineStr">
+        <is>
+          <t>CHI-20260922-009</t>
+        </is>
+      </c>
+      <c r="B1174" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1174" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1174" t="inlineStr">
+        <is>
+          <t>顾全大局</t>
+        </is>
+      </c>
+      <c r="E1174" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1174" t="inlineStr">
+        <is>
+          <t>gù quán dà jù</t>
+        </is>
+      </c>
+      <c r="G1174" t="inlineStr">
+        <is>
+          <t>전체적인 대세를 고려하다, 큰 대국을 위해 양보하다</t>
+        </is>
+      </c>
+      <c r="H1174" t="inlineStr">
+        <is>
+          <t>面对突发状况，我们要顾全大局，听从统一指挥。</t>
+        </is>
+      </c>
+      <c r="I1174" t="inlineStr">
+        <is>
+          <t>关键时刻，他决定牺牲个人利益，以顾全大局。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" t="inlineStr">
+        <is>
+          <t>CHI-20260922-010</t>
+        </is>
+      </c>
+      <c r="B1175" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1175" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1175" t="inlineStr">
+        <is>
+          <t>乱成一团</t>
+        </is>
+      </c>
+      <c r="E1175" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1175" t="inlineStr">
+        <is>
+          <t>luàn chéng yī tuán</t>
+        </is>
+      </c>
+      <c r="G1175" t="inlineStr">
+        <is>
+          <t>아수라장이 되다, 엉망진창이 되다, 발칵 뒤집히다</t>
+        </is>
+      </c>
+      <c r="H1175" t="inlineStr">
+        <is>
+          <t>突如其来的大雨让现场乱成一团，交通也瘫痪了。</t>
+        </is>
+      </c>
+      <c r="I1175" t="inlineStr">
+        <is>
+          <t>妈妈一出门，家里的两个小家伙就把客厅闹得乱成一团。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-23 | 1182/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1175"/>
+  <dimension ref="A1:I1183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55641,6 +55641,382 @@
         </is>
       </c>
     </row>
+    <row r="1176">
+      <c r="A1176" t="inlineStr">
+        <is>
+          <t>CHI-20260923-001</t>
+        </is>
+      </c>
+      <c r="B1176" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C1176" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1176" t="inlineStr">
+        <is>
+          <t>眼见为实</t>
+        </is>
+      </c>
+      <c r="E1176" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1176" t="inlineStr">
+        <is>
+          <t>yǎn jiàn wéi shí</t>
+        </is>
+      </c>
+      <c r="G1176" t="inlineStr">
+        <is>
+          <t>백문이 불여일견, 직접 봐야 믿을 수 있다</t>
+        </is>
+      </c>
+      <c r="H1176" t="inlineStr">
+        <is>
+          <t>자선단체들이 사용 내역을 투명하게 플랫폼에 공시함으로써, 기부자들이 직접 눈으로 투명성을 확인하게 해야 신뢰를 얻습니다.</t>
+        </is>
+      </c>
+      <c r="I1176" t="inlineStr">
+        <is>
+          <t>光听他说没用，咱们还是眼见为实吧。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" t="inlineStr">
+        <is>
+          <t>CHI-20260923-002</t>
+        </is>
+      </c>
+      <c r="B1177" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C1177" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1177" t="inlineStr">
+        <is>
+          <t>必修课</t>
+        </is>
+      </c>
+      <c r="E1177" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1177" t="inlineStr">
+        <is>
+          <t>bì xiū kè</t>
+        </is>
+      </c>
+      <c r="G1177" t="inlineStr">
+        <is>
+          <t>필수 코스, 인생이나 사회생활에서 반드시 거치고 배워야 할 것</t>
+        </is>
+      </c>
+      <c r="H1177" t="inlineStr">
+        <is>
+          <t>学会如何面对人生的挫折，是每个年轻人的必修课。</t>
+        </is>
+      </c>
+      <c r="I1177" t="inlineStr">
+        <is>
+          <t>对于创业者来说，如何合理控制财务风险是一门必修课。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" t="inlineStr">
+        <is>
+          <t>CHI-20260923-003</t>
+        </is>
+      </c>
+      <c r="B1178" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C1178" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1178" t="inlineStr">
+        <is>
+          <t>招工</t>
+        </is>
+      </c>
+      <c r="E1178" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1178" t="inlineStr">
+        <is>
+          <t>zhāo gōng</t>
+        </is>
+      </c>
+      <c r="G1178" t="inlineStr">
+        <is>
+          <t>일꾼(직원)을 모집하다, 구인하다</t>
+        </is>
+      </c>
+      <c r="H1178" t="inlineStr">
+        <is>
+          <t>人社部近期启动了秋季联合招聘，很多企业都在积极招工。</t>
+        </is>
+      </c>
+      <c r="I1178" t="inlineStr">
+        <is>
+          <t>这家工厂由于业务量剧增，最近急需在当地招工。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" t="inlineStr">
+        <is>
+          <t>CHI-20260923-004</t>
+        </is>
+      </c>
+      <c r="B1179" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C1179" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1179" t="inlineStr">
+        <is>
+          <t>避嫌</t>
+        </is>
+      </c>
+      <c r="E1179" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1179" t="inlineStr">
+        <is>
+          <t>bì xián</t>
+        </is>
+      </c>
+      <c r="G1179" t="inlineStr">
+        <is>
+          <t>혐의를 피하다, 오해 살 만한 일을 피하다</t>
+        </is>
+      </c>
+      <c r="H1179" t="inlineStr">
+        <is>
+          <t>为了在慈善监管中避嫌，他主动退出了这次的善款审核工作。</t>
+        </is>
+      </c>
+      <c r="I1179" t="inlineStr">
+        <is>
+          <t>在这个敏感时期，他作为项目负责人选择主动避嫌是不无道理的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" t="inlineStr">
+        <is>
+          <t>CHI-20260923-005</t>
+        </is>
+      </c>
+      <c r="B1180" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C1180" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1180" t="inlineStr">
+        <is>
+          <t>露面</t>
+        </is>
+      </c>
+      <c r="E1180" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1180" t="inlineStr">
+        <is>
+          <t>lòu miàn</t>
+        </is>
+      </c>
+      <c r="G1180" t="inlineStr">
+        <is>
+          <t>얼굴을 드러내다, 공식 석상에 나타나다</t>
+        </is>
+      </c>
+      <c r="H1180" t="inlineStr">
+        <is>
+          <t>因为身体原因，他最近很少在公开活动中露面。</t>
+        </is>
+      </c>
+      <c r="I1180" t="inlineStr">
+        <is>
+          <t>在这次重要的新品发布会上，公司新聘任的CEO终于露了面。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" t="inlineStr">
+        <is>
+          <t>CHI-20260923-006</t>
+        </is>
+      </c>
+      <c r="B1181" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C1181" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1181" t="inlineStr">
+        <is>
+          <t>看好</t>
+        </is>
+      </c>
+      <c r="E1181" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1181" t="inlineStr">
+        <is>
+          <t>kàn hǎo</t>
+        </is>
+      </c>
+      <c r="G1181" t="inlineStr">
+        <is>
+          <t>유망하게 보다, 좋게 평가하다, 낙관하다</t>
+        </is>
+      </c>
+      <c r="H1181" t="inlineStr">
+        <is>
+          <t>发改委这次向民营企业推介的几十个项目，被业内专家普遍看好。</t>
+        </is>
+      </c>
+      <c r="I1181" t="inlineStr">
+        <is>
+          <t>尽管他现在遇到了挫折，但我依然非常看好他未来的职业发展。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" t="inlineStr">
+        <is>
+          <t>CHI-20260923-007</t>
+        </is>
+      </c>
+      <c r="B1182" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C1182" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1182" t="inlineStr">
+        <is>
+          <t>出面</t>
+        </is>
+      </c>
+      <c r="E1182" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1182" t="inlineStr">
+        <is>
+          <t>chū miàn</t>
+        </is>
+      </c>
+      <c r="G1182" t="inlineStr">
+        <is>
+          <t>나서다, 직접 주선하다 (중재나 문제 해결을 위해)</t>
+        </is>
+      </c>
+      <c r="H1182" t="inlineStr">
+        <is>
+          <t>邻里之间如果有了纠纷，往往需要城管或居委会出面协调。</t>
+        </is>
+      </c>
+      <c r="I1182" t="inlineStr">
+        <is>
+          <t>这件事情影响很大，必须得由我们总经理亲自出面才能摆平。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" t="inlineStr">
+        <is>
+          <t>CHI-20260923-008</t>
+        </is>
+      </c>
+      <c r="B1183" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C1183" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1183" t="inlineStr">
+        <is>
+          <t>迫在眉睫</t>
+        </is>
+      </c>
+      <c r="E1183" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1183" t="inlineStr">
+        <is>
+          <t>pò zài méi jié</t>
+        </is>
+      </c>
+      <c r="G1183" t="inlineStr">
+        <is>
+          <t>눈앞에 닥치다, 매우 시급하다</t>
+        </is>
+      </c>
+      <c r="H1183" t="inlineStr">
+        <is>
+          <t>随着人口快速老龄化，推动养老机构护理型床位建设已经迫在眉睫。</t>
+        </is>
+      </c>
+      <c r="I1183" t="inlineStr">
+        <is>
+          <t>这个项目的截止日期快到了，寻找合适的合作伙伴已经是迫在眉睫的事情。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-24 | 1185/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1183"/>
+  <dimension ref="A1:I1186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -56017,6 +56017,147 @@
         </is>
       </c>
     </row>
+    <row r="1184">
+      <c r="A1184" t="inlineStr">
+        <is>
+          <t>CHI-20260924-001</t>
+        </is>
+      </c>
+      <c r="B1184" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C1184" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1184" t="inlineStr">
+        <is>
+          <t>泼脏水</t>
+        </is>
+      </c>
+      <c r="E1184" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1184" t="inlineStr">
+        <is>
+          <t>pō zāng shuǐ</t>
+        </is>
+      </c>
+      <c r="G1184" t="inlineStr">
+        <is>
+          <t>터무니없이 모함하다, 오명을 씌우다, 흙탕물을 끼얹다</t>
+        </is>
+      </c>
+      <c r="H1184" t="inlineStr">
+        <is>
+          <t>针对某些国家有关机构故意散布谎言、抹黑中国形象的行为，外交部发言人严正敦促其立即停止这种恶意泼脏水的行径。</t>
+        </is>
+      </c>
+      <c r="I1184" t="inlineStr">
+        <is>
+          <t>对手故意在网上给我们公司泼脏水，抹黑我们的环保品牌。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" t="inlineStr">
+        <is>
+          <t>CHI-20260924-002</t>
+        </is>
+      </c>
+      <c r="B1185" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C1185" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1185" t="inlineStr">
+        <is>
+          <t>捞一把</t>
+        </is>
+      </c>
+      <c r="E1185" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1185" t="inlineStr">
+        <is>
+          <t>lāo yī bǎ</t>
+        </is>
+      </c>
+      <c r="G1185" t="inlineStr">
+        <is>
+          <t>한몫 챙기다, 부당하게 이득을 취하다</t>
+        </is>
+      </c>
+      <c r="H1185" t="inlineStr">
+        <is>
+          <t>为了打造公开透明的“阳光慈善”，民政部出台了更严格的监管政策，绝不给企图利用慈善募捐捞一把的人任何机会。</t>
+        </is>
+      </c>
+      <c r="I1185" t="inlineStr">
+        <is>
+          <t>慈善基金是为了帮助弱势群体的，决不允许任何人借机捞一把。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" t="inlineStr">
+        <is>
+          <t>CHI-20260924-003</t>
+        </is>
+      </c>
+      <c r="B1186" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C1186" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1186" t="inlineStr">
+        <is>
+          <t>不着调</t>
+        </is>
+      </c>
+      <c r="E1186" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1186" t="inlineStr">
+        <is>
+          <t>bù zháo diào</t>
+        </is>
+      </c>
+      <c r="G1186" t="inlineStr">
+        <is>
+          <t>터무니없다, 믿음직스럽지 못하다, 종잡을 수 없다</t>
+        </is>
+      </c>
+      <c r="H1186" t="inlineStr">
+        <is>
+          <t>环保床垫怎么挑？三步看穿不着调的“伪环保”陷阱。</t>
+        </is>
+      </c>
+      <c r="I1186" t="inlineStr">
+        <is>
+          <t>他这个人说话办事总是不着调，大家都不怎么信任他。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-25 | 1197/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1186"/>
+  <dimension ref="A1:I1198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -56158,6 +56158,570 @@
         </is>
       </c>
     </row>
+    <row r="1187">
+      <c r="A1187" t="inlineStr">
+        <is>
+          <t>CHI-20260925-001</t>
+        </is>
+      </c>
+      <c r="B1187" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C1187" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1187" t="inlineStr">
+        <is>
+          <t>过紧日子</t>
+        </is>
+      </c>
+      <c r="E1187" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1187" t="inlineStr">
+        <is>
+          <t>guò jǐn rì zi</t>
+        </is>
+      </c>
+      <c r="G1187" t="inlineStr">
+        <is>
+          <t>예산을 절약하다, 허리띠를 졸라매다</t>
+        </is>
+      </c>
+      <c r="H1187" t="inlineStr">
+        <is>
+          <t>경제 상황이 어려워지자 회사와 공공기관들이 예산을 대폭 줄이고 알뜰하게 운영해야 하는 상황</t>
+        </is>
+      </c>
+      <c r="I1187" t="inlineStr">
+        <is>
+          <t>现在公司项目预算缩减，大家都要学会过紧日子。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" t="inlineStr">
+        <is>
+          <t>CHI-20260925-002</t>
+        </is>
+      </c>
+      <c r="B1188" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C1188" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1188" t="inlineStr">
+        <is>
+          <t>颜值</t>
+        </is>
+      </c>
+      <c r="E1188" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1188" t="inlineStr">
+        <is>
+          <t>yán zhí</t>
+        </is>
+      </c>
+      <c r="G1188" t="inlineStr">
+        <is>
+          <t>외모 수준, 비주얼</t>
+        </is>
+      </c>
+      <c r="H1188" t="inlineStr">
+        <is>
+          <t>도시의 환경 정비나 물건의 디자인이 얼마나 보기 좋고 아름다운지 평가할 때</t>
+        </is>
+      </c>
+      <c r="I1188" t="inlineStr">
+        <is>
+          <t>这家咖啡店的颜值很高，非常适合打卡拍照。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" t="inlineStr">
+        <is>
+          <t>CHI-20260925-003</t>
+        </is>
+      </c>
+      <c r="B1189" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C1189" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1189" t="inlineStr">
+        <is>
+          <t>良方</t>
+        </is>
+      </c>
+      <c r="E1189" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1189" t="inlineStr">
+        <is>
+          <t>liáng fāng</t>
+        </is>
+      </c>
+      <c r="G1189" t="inlineStr">
+        <is>
+          <t>좋은 해결책, 묘책</t>
+        </is>
+      </c>
+      <c r="H1189" t="inlineStr">
+        <is>
+          <t>복잡한 도시 문제나 사회적 난제를 해결하기 위한 효과적인 정책이나 아이디어</t>
+        </is>
+      </c>
+      <c r="I1189" t="inlineStr">
+        <is>
+          <t>这是解决交通拥堵问题的良方，建议大家参考。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" t="inlineStr">
+        <is>
+          <t>CHI-20260925-004</t>
+        </is>
+      </c>
+      <c r="B1190" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C1190" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1190" t="inlineStr">
+        <is>
+          <t>扰民</t>
+        </is>
+      </c>
+      <c r="E1190" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1190" t="inlineStr">
+        <is>
+          <t>rǎo mín</t>
+        </is>
+      </c>
+      <c r="G1190" t="inlineStr">
+        <is>
+          <t>주민에게 피해(소음 등)를 끼치다</t>
+        </is>
+      </c>
+      <c r="H1190" t="inlineStr">
+        <is>
+          <t>학교 종소리나 공사 소음 등이 인근 주민들의 평온한 생활을 방해할 때</t>
+        </is>
+      </c>
+      <c r="I1190" t="inlineStr">
+        <is>
+          <t>深夜在小区里大声喧哗，实在是太扰民了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" t="inlineStr">
+        <is>
+          <t>CHI-20260925-005</t>
+        </is>
+      </c>
+      <c r="B1191" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C1191" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1191" t="inlineStr">
+        <is>
+          <t>生根</t>
+        </is>
+      </c>
+      <c r="E1191" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1191" t="inlineStr">
+        <is>
+          <t>shēng gēn</t>
+        </is>
+      </c>
+      <c r="G1191" t="inlineStr">
+        <is>
+          <t>뿌리를 내리다, 정착하다</t>
+        </is>
+      </c>
+      <c r="H1191" t="inlineStr">
+        <is>
+          <t>좋은 문화나 지식이 특정 지역에 완전히 자리 잡고 확산될 때</t>
+        </is>
+      </c>
+      <c r="I1191" t="inlineStr">
+        <is>
+          <t>阅读文化需要时间在基层社区慢慢生根发芽。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" t="inlineStr">
+        <is>
+          <t>CHI-20260925-006</t>
+        </is>
+      </c>
+      <c r="B1192" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C1192" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1192" t="inlineStr">
+        <is>
+          <t>全方位</t>
+        </is>
+      </c>
+      <c r="E1192" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1192" t="inlineStr">
+        <is>
+          <t>quán fāng wèi</t>
+        </is>
+      </c>
+      <c r="G1192" t="inlineStr">
+        <is>
+          <t>전방위적으로, 모든 방면에서</t>
+        </is>
+      </c>
+      <c r="H1192" t="inlineStr">
+        <is>
+          <t>도시 환경 개선이나 업무 보고 등에서 빈틈없이 모든 부분을 관리할 때</t>
+        </is>
+      </c>
+      <c r="I1192" t="inlineStr">
+        <is>
+          <t>我们需要进行全方位的市场调研才能做出决策。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="inlineStr">
+        <is>
+          <t>CHI-20260925-007</t>
+        </is>
+      </c>
+      <c r="B1193" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1193" t="inlineStr">
+        <is>
+          <t>当面一套背后一套</t>
+        </is>
+      </c>
+      <c r="E1193" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1193" t="inlineStr">
+        <is>
+          <t>dāng miàn yī tào bèi hòu yī tào</t>
+        </is>
+      </c>
+      <c r="G1193" t="inlineStr">
+        <is>
+          <t>표리부동하다, 앞뒤가 다르다</t>
+        </is>
+      </c>
+      <c r="H1193" t="inlineStr">
+        <is>
+          <t>직장 내에서 동료의 태도가 사람 앞과 뒤에서 다를 때 비판하는 표현</t>
+        </is>
+      </c>
+      <c r="I1193" t="inlineStr">
+        <is>
+          <t>我最讨厌那种当面一套背后一套的人，很不真诚。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" t="inlineStr">
+        <is>
+          <t>CHI-20260925-008</t>
+        </is>
+      </c>
+      <c r="B1194" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1194" t="inlineStr">
+        <is>
+          <t>心头好</t>
+        </is>
+      </c>
+      <c r="E1194" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1194" t="inlineStr">
+        <is>
+          <t>xīn tóu hǎo</t>
+        </is>
+      </c>
+      <c r="G1194" t="inlineStr">
+        <is>
+          <t>가장 아끼는 것, 최애</t>
+        </is>
+      </c>
+      <c r="H1194" t="inlineStr">
+        <is>
+          <t>개인이 평소에 정말 좋아하고 소중하게 여기는 아이템이나 대상을 지칭할 때</t>
+        </is>
+      </c>
+      <c r="I1194" t="inlineStr">
+        <is>
+          <t>这款新款手机是我的心头好，用了就再也回不去了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="inlineStr">
+        <is>
+          <t>CHI-20260925-009</t>
+        </is>
+      </c>
+      <c r="B1195" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1195" t="inlineStr">
+        <is>
+          <t>动不动</t>
+        </is>
+      </c>
+      <c r="E1195" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1195" t="inlineStr">
+        <is>
+          <t>dòng bu dòng</t>
+        </is>
+      </c>
+      <c r="G1195" t="inlineStr">
+        <is>
+          <t>툭하면, 틈만 나면</t>
+        </is>
+      </c>
+      <c r="H1195" t="inlineStr">
+        <is>
+          <t>부정적인 행동이 습관적으로 자주 발생할 때 쓰는 강조 표현</t>
+        </is>
+      </c>
+      <c r="I1195" t="inlineStr">
+        <is>
+          <t>他动不动就发脾气，大家都很怕他。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="inlineStr">
+        <is>
+          <t>CHI-20260925-010</t>
+        </is>
+      </c>
+      <c r="B1196" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1196" t="inlineStr">
+        <is>
+          <t>拿捏</t>
+        </is>
+      </c>
+      <c r="E1196" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1196" t="inlineStr">
+        <is>
+          <t>ná niē</t>
+        </is>
+      </c>
+      <c r="G1196" t="inlineStr">
+        <is>
+          <t>능숙하게 다루다, 요령을 잘 알다</t>
+        </is>
+      </c>
+      <c r="H1196" t="inlineStr">
+        <is>
+          <t>城市治理需要精准拿捏管理的力度与温度.</t>
+        </is>
+      </c>
+      <c r="I1196" t="inlineStr">
+        <is>
+          <t>他处理这种突发状况非常有一套，火候拿捏得刚好。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" t="inlineStr">
+        <is>
+          <t>CHI-20260925-011</t>
+        </is>
+      </c>
+      <c r="B1197" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C1197" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1197" t="inlineStr">
+        <is>
+          <t>撒手锏</t>
+        </is>
+      </c>
+      <c r="E1197" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1197" t="inlineStr">
+        <is>
+          <t>sā shǒu jiàn</t>
+        </is>
+      </c>
+      <c r="G1197" t="inlineStr">
+        <is>
+          <t>필살기, 결정적인 수단</t>
+        </is>
+      </c>
+      <c r="H1197" t="inlineStr">
+        <is>
+          <t>这是我们提升城市治理品质的撒手锏.</t>
+        </is>
+      </c>
+      <c r="I1197" t="inlineStr">
+        <is>
+          <t>技术创新是这家企业在市场上立足的撒手锏。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" t="inlineStr">
+        <is>
+          <t>CHI-20260925-012</t>
+        </is>
+      </c>
+      <c r="B1198" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C1198" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1198" t="inlineStr">
+        <is>
+          <t>心知肚明</t>
+        </is>
+      </c>
+      <c r="E1198" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1198" t="inlineStr">
+        <is>
+          <t>xīn zhī dù míng</t>
+        </is>
+      </c>
+      <c r="G1198" t="inlineStr">
+        <is>
+          <t>속으로 뻔히 알다, 다 알고 있다</t>
+        </is>
+      </c>
+      <c r="H1198" t="inlineStr">
+        <is>
+          <t>大家对项目的失败原因都心知肚明.</t>
+        </is>
+      </c>
+      <c r="I1198" t="inlineStr">
+        <is>
+          <t>虽然大家没说出来，但对这次人事变动都心知肚明。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-28 | 1203/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1198"/>
+  <dimension ref="A1:I1204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -56722,6 +56722,288 @@
         </is>
       </c>
     </row>
+    <row r="1199">
+      <c r="A1199" t="inlineStr">
+        <is>
+          <t>CHI-20260928-001</t>
+        </is>
+      </c>
+      <c r="B1199" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C1199" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1199" t="inlineStr">
+        <is>
+          <t>大白话</t>
+        </is>
+      </c>
+      <c r="E1199" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1199" t="inlineStr">
+        <is>
+          <t>dà bái huà</t>
+        </is>
+      </c>
+      <c r="G1199" t="inlineStr">
+        <is>
+          <t>알기 쉬운 말, 평이한 말</t>
+        </is>
+      </c>
+      <c r="H1199" t="inlineStr">
+        <is>
+          <t>어려운 용어 없이 누구나 알아들을 수 있게 말할 때</t>
+        </is>
+      </c>
+      <c r="I1199" t="inlineStr">
+        <is>
+          <t>能不能用大白话解释一下这个政策？</t>
+        </is>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" t="inlineStr">
+        <is>
+          <t>CHI-20260928-002</t>
+        </is>
+      </c>
+      <c r="B1200" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C1200" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1200" t="inlineStr">
+        <is>
+          <t>翻白眼</t>
+        </is>
+      </c>
+      <c r="E1200" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1200" t="inlineStr">
+        <is>
+          <t>fān bái yǎn</t>
+        </is>
+      </c>
+      <c r="G1200" t="inlineStr">
+        <is>
+          <t>눈을 흘기다, 어이없다는 듯 쳐다보다</t>
+        </is>
+      </c>
+      <c r="H1200" t="inlineStr">
+        <is>
+          <t>상대방의 말이 마음에 안 들거나 어이없을 때 하는 무언의 행동</t>
+        </is>
+      </c>
+      <c r="I1200" t="inlineStr">
+        <is>
+          <t>听到这个笑话，她忍不住翻了个白眼。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" t="inlineStr">
+        <is>
+          <t>CHI-20260928-003</t>
+        </is>
+      </c>
+      <c r="B1201" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C1201" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1201" t="inlineStr">
+        <is>
+          <t>露两手</t>
+        </is>
+      </c>
+      <c r="E1201" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1201" t="inlineStr">
+        <is>
+          <t>lòu liǎng shǒu</t>
+        </is>
+      </c>
+      <c r="G1201" t="inlineStr">
+        <is>
+          <t>실력을 보여주다, 솜씨를 발휘하다</t>
+        </is>
+      </c>
+      <c r="H1201" t="inlineStr">
+        <is>
+          <t>자신의 뛰어난 기술이나 능력을 남에게 뽐낼 때</t>
+        </is>
+      </c>
+      <c r="I1201" t="inlineStr">
+        <is>
+          <t>既然来了，你就给大家露两手吧！</t>
+        </is>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" t="inlineStr">
+        <is>
+          <t>CHI-20260928-004</t>
+        </is>
+      </c>
+      <c r="B1202" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C1202" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1202" t="inlineStr">
+        <is>
+          <t>过意不去</t>
+        </is>
+      </c>
+      <c r="E1202" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1202" t="inlineStr">
+        <is>
+          <t>guò yì bù qù</t>
+        </is>
+      </c>
+      <c r="G1202" t="inlineStr">
+        <is>
+          <t>미안하다, 마음이 편치 않다</t>
+        </is>
+      </c>
+      <c r="H1202" t="inlineStr">
+        <is>
+          <t>상대방의 호의를 받아 빚을 진 느낌이 들 때</t>
+        </is>
+      </c>
+      <c r="I1202" t="inlineStr">
+        <is>
+          <t>让你破费了，真让我过意不去。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" t="inlineStr">
+        <is>
+          <t>CHI-20260928-005</t>
+        </is>
+      </c>
+      <c r="B1203" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C1203" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1203" t="inlineStr">
+        <is>
+          <t>耍脾气</t>
+        </is>
+      </c>
+      <c r="E1203" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1203" t="inlineStr">
+        <is>
+          <t>shuǎ pí qi</t>
+        </is>
+      </c>
+      <c r="G1203" t="inlineStr">
+        <is>
+          <t>성질을 부리다, 투정을 부리다</t>
+        </is>
+      </c>
+      <c r="H1203" t="inlineStr">
+        <is>
+          <t>자신의 뜻대로 되지 않아 짜증을 내는 상황</t>
+        </is>
+      </c>
+      <c r="I1203" t="inlineStr">
+        <is>
+          <t>已经是成年人了，别动不动就耍脾气。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" t="inlineStr">
+        <is>
+          <t>CHI-20260928-006</t>
+        </is>
+      </c>
+      <c r="B1204" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C1204" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1204" t="inlineStr">
+        <is>
+          <t>冷处理</t>
+        </is>
+      </c>
+      <c r="E1204" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1204" t="inlineStr">
+        <is>
+          <t>lěng chǔ lǐ</t>
+        </is>
+      </c>
+      <c r="G1204" t="inlineStr">
+        <is>
+          <t>조용히 처리하다, 시간을 두고 해결하다</t>
+        </is>
+      </c>
+      <c r="H1204" t="inlineStr">
+        <is>
+          <t>문제가 생겼을 때 즉각 대응하지 않고 상황이 진정되길 기다릴 때</t>
+        </is>
+      </c>
+      <c r="I1204" t="inlineStr">
+        <is>
+          <t>这件事情太敏感了，先冷处理一段时间吧。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-29 | 1218/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1204"/>
+  <dimension ref="A1:I1219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -57004,6 +57004,711 @@
         </is>
       </c>
     </row>
+    <row r="1205">
+      <c r="A1205" t="inlineStr">
+        <is>
+          <t>CHI-20260929-001</t>
+        </is>
+      </c>
+      <c r="B1205" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1205" t="inlineStr">
+        <is>
+          <t>玻璃心</t>
+        </is>
+      </c>
+      <c r="E1205" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1205" t="inlineStr">
+        <is>
+          <t>bō li xīn</t>
+        </is>
+      </c>
+      <c r="G1205" t="inlineStr">
+        <is>
+          <t>유리 멘탈, 쿠쿠다스 심장 (쉽게 상처받는 약한 마음)</t>
+        </is>
+      </c>
+      <c r="H1205" t="inlineStr">
+        <is>
+          <t>온라인상에서 쏟아지는 악성 댓글이나 비난을 견디지 못하고 쉽게 좌절하는 사람들의 연약한 멘탈을 비유하는 단어이다.</t>
+        </is>
+      </c>
+      <c r="I1205" t="inlineStr">
+        <is>
+          <t>做自媒体工作就不能有玻璃心，必须要能承受各种各样的评价。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="inlineStr">
+        <is>
+          <t>CHI-20260929-002</t>
+        </is>
+      </c>
+      <c r="B1206" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1206" t="inlineStr">
+        <is>
+          <t>烧脑</t>
+        </is>
+      </c>
+      <c r="E1206" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1206" t="inlineStr">
+        <is>
+          <t>shāo nǎo</t>
+        </is>
+      </c>
+      <c r="G1206" t="inlineStr">
+        <is>
+          <t>머리를 많이 써야 하는, 지적으로 복잡하고 흥미진진한</t>
+        </is>
+      </c>
+      <c r="H1206" t="inlineStr">
+        <is>
+          <t>단순한 오락거리를 넘어, 복잡한 인과관계나 치밀한 지적 논리를 요구하는 콘텐츠나 경제 구조를 묘사한다.</t>
+        </is>
+      </c>
+      <c r="I1206" t="inlineStr">
+        <is>
+          <t>这部悬疑电影剧情环环相扣，实在太烧脑了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" t="inlineStr">
+        <is>
+          <t>CHI-20260929-003</t>
+        </is>
+      </c>
+      <c r="B1207" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C1207" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1207" t="inlineStr">
+        <is>
+          <t>冤枉钱</t>
+        </is>
+      </c>
+      <c r="E1207" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1207" t="inlineStr">
+        <is>
+          <t>yuān wang qián</t>
+        </is>
+      </c>
+      <c r="G1207" t="inlineStr">
+        <is>
+          <t>아깝게 낭비한 돈, 안 써도 될 곳에 쓴 돈</t>
+        </is>
+      </c>
+      <c r="H1207" t="inlineStr">
+        <is>
+          <t>허위 친환경 마케팅이나 과장된 광고에 속아 정가보다 훨씬 높은 비용을 지불하는 어리석은 소비를 의미한다.</t>
+        </is>
+      </c>
+      <c r="I1207" t="inlineStr">
+        <is>
+          <t>买东西前要做足功课，免得花冤枉钱买到假货。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="inlineStr">
+        <is>
+          <t>CHI-20260929-004</t>
+        </is>
+      </c>
+      <c r="B1208" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C1208" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1208" t="inlineStr">
+        <is>
+          <t>华而不实</t>
+        </is>
+      </c>
+      <c r="E1208" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1208" t="inlineStr">
+        <is>
+          <t>huá ér bù shí</t>
+        </is>
+      </c>
+      <c r="G1208" t="inlineStr">
+        <is>
+          <t>빛 좋은 개살구, 겉만 번지르르하고 실속이 없다</t>
+        </is>
+      </c>
+      <c r="H1208" t="inlineStr">
+        <is>
+          <t>디자인만 그럴듯하고 실제 내구성이나 친환경 실용성은 전혀 고려되지 않은 가구 등의 겉모습을 풍자하는 성어이다.</t>
+        </is>
+      </c>
+      <c r="I1208" t="inlineStr">
+        <is>
+          <t>买家具不能只看外观，华而不实的产品用不了多久就会坏。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="inlineStr">
+        <is>
+          <t>CHI-20260929-005</t>
+        </is>
+      </c>
+      <c r="B1209" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C1209" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1209" t="inlineStr">
+        <is>
+          <t>出力</t>
+        </is>
+      </c>
+      <c r="E1209" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1209" t="inlineStr">
+        <is>
+          <t>chū lì</t>
+        </is>
+      </c>
+      <c r="G1209" t="inlineStr">
+        <is>
+          <t>힘을 쓰다, 공을 들이다</t>
+        </is>
+      </c>
+      <c r="H1209" t="inlineStr">
+        <is>
+          <t>环保不仅需要政策，更需要每个人为城市治理出力。</t>
+        </is>
+      </c>
+      <c r="I1209" t="inlineStr">
+        <is>
+          <t>为了这次项目能顺利上线，大家都出了不少力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="inlineStr">
+        <is>
+          <t>CHI-20260929-006</t>
+        </is>
+      </c>
+      <c r="B1210" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1210" t="inlineStr">
+        <is>
+          <t>做主</t>
+        </is>
+      </c>
+      <c r="E1210" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1210" t="inlineStr">
+        <is>
+          <t>zuò zhǔ</t>
+        </is>
+      </c>
+      <c r="G1210" t="inlineStr">
+        <is>
+          <t>결정권을 갖다, 주관하다</t>
+        </is>
+      </c>
+      <c r="H1210" t="inlineStr">
+        <is>
+          <t>在学生实践活动的安排上，老师不能完全替学生做主。</t>
+        </is>
+      </c>
+      <c r="I1210" t="inlineStr">
+        <is>
+          <t>这件事情你还是自己做主吧，毕竟是你自己的职业规划。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="inlineStr">
+        <is>
+          <t>CHI-20260929-007</t>
+        </is>
+      </c>
+      <c r="B1211" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1211" t="inlineStr">
+        <is>
+          <t>变脸</t>
+        </is>
+      </c>
+      <c r="E1211" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1211" t="inlineStr">
+        <is>
+          <t>biàn liǎn</t>
+        </is>
+      </c>
+      <c r="G1211" t="inlineStr">
+        <is>
+          <t>태도를 갑자기 바꾸다</t>
+        </is>
+      </c>
+      <c r="H1211" t="inlineStr">
+        <is>
+          <t>有些人面对质量投诉时立刻变脸，完全不负责任。</t>
+        </is>
+      </c>
+      <c r="I1211" t="inlineStr">
+        <is>
+          <t>刚才还谈笑风生，怎么提起赔偿问题就变脸了？</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="inlineStr">
+        <is>
+          <t>CHI-20260929-008</t>
+        </is>
+      </c>
+      <c r="B1212" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1212" t="inlineStr">
+        <is>
+          <t>下场</t>
+        </is>
+      </c>
+      <c r="E1212" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1212" t="inlineStr">
+        <is>
+          <t>xià chǎng</t>
+        </is>
+      </c>
+      <c r="G1212" t="inlineStr">
+        <is>
+          <t>결말(주로 나쁜 상황)</t>
+        </is>
+      </c>
+      <c r="H1212" t="inlineStr">
+        <is>
+          <t>忽视质量问题的商家，最终的下场只有被市场淘汰。</t>
+        </is>
+      </c>
+      <c r="I1212" t="inlineStr">
+        <is>
+          <t>如果不遵守规则，这就是他迟早要面临的下场。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="inlineStr">
+        <is>
+          <t>CHI-20260929-009</t>
+        </is>
+      </c>
+      <c r="B1213" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1213" t="inlineStr">
+        <is>
+          <t>入坑</t>
+        </is>
+      </c>
+      <c r="E1213" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1213" t="inlineStr">
+        <is>
+          <t>rù kēng</t>
+        </is>
+      </c>
+      <c r="G1213" t="inlineStr">
+        <is>
+          <t>좋아하게 되다, 취미에 빠지다</t>
+        </is>
+      </c>
+      <c r="H1213" t="inlineStr">
+        <is>
+          <t>很多年轻人因为养多肉而入坑，从此一发不可收拾。</t>
+        </is>
+      </c>
+      <c r="I1213" t="inlineStr">
+        <is>
+          <t>朋友送了我一本小说，结果我彻底入坑了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="inlineStr">
+        <is>
+          <t>CHI-20260929-010</t>
+        </is>
+      </c>
+      <c r="B1214" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1214" t="inlineStr">
+        <is>
+          <t>站位</t>
+        </is>
+      </c>
+      <c r="E1214" t="inlineStr">
+        <is>
+          <t>오피스 표현</t>
+        </is>
+      </c>
+      <c r="F1214" t="inlineStr">
+        <is>
+          <t>zhàn wèi</t>
+        </is>
+      </c>
+      <c r="G1214" t="inlineStr">
+        <is>
+          <t>입장, 위치 선정</t>
+        </is>
+      </c>
+      <c r="H1214" t="inlineStr">
+        <is>
+          <t>企业在谈环保时，必须具备全局站位。</t>
+        </is>
+      </c>
+      <c r="I1214" t="inlineStr">
+        <is>
+          <t>我们需要从更高的站位来审视这个战略方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="inlineStr">
+        <is>
+          <t>CHI-20260929-011</t>
+        </is>
+      </c>
+      <c r="B1215" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1215" t="inlineStr">
+        <is>
+          <t>共生</t>
+        </is>
+      </c>
+      <c r="E1215" t="inlineStr">
+        <is>
+          <t>오피스 표현</t>
+        </is>
+      </c>
+      <c r="F1215" t="inlineStr">
+        <is>
+          <t>gòng shēng</t>
+        </is>
+      </c>
+      <c r="G1215" t="inlineStr">
+        <is>
+          <t>상생, 공생</t>
+        </is>
+      </c>
+      <c r="H1215" t="inlineStr">
+        <is>
+          <t>城校共生，是推动大学城发展的关键。</t>
+        </is>
+      </c>
+      <c r="I1215" t="inlineStr">
+        <is>
+          <t>我们追求的是企业与环境之间的良性共生。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="inlineStr">
+        <is>
+          <t>CHI-20260929-012</t>
+        </is>
+      </c>
+      <c r="B1216" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1216" t="inlineStr">
+        <is>
+          <t>量力而行</t>
+        </is>
+      </c>
+      <c r="E1216" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1216" t="inlineStr">
+        <is>
+          <t>liàng lì ér xíng</t>
+        </is>
+      </c>
+      <c r="G1216" t="inlineStr">
+        <is>
+          <t>자신의 능력에 맞게 행동하다</t>
+        </is>
+      </c>
+      <c r="H1216" t="inlineStr">
+        <is>
+          <t>参与实践活动应量力而行，不要给学生太大压力。</t>
+        </is>
+      </c>
+      <c r="I1216" t="inlineStr">
+        <is>
+          <t>无论工作还是生活，都要学会量力而行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="inlineStr">
+        <is>
+          <t>CHI-20260929-013</t>
+        </is>
+      </c>
+      <c r="B1217" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1217" t="inlineStr">
+        <is>
+          <t>免疫</t>
+        </is>
+      </c>
+      <c r="E1217" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1217" t="inlineStr">
+        <is>
+          <t>miǎn yì</t>
+        </is>
+      </c>
+      <c r="G1217" t="inlineStr">
+        <is>
+          <t>(유혹에) 무뎌지다, 초연해지다</t>
+        </is>
+      </c>
+      <c r="H1217" t="inlineStr">
+        <is>
+          <t>孩子对零食突然免疫，让家长省心不少。</t>
+        </is>
+      </c>
+      <c r="I1217" t="inlineStr">
+        <is>
+          <t>听多了这种场面话，我都产生免疫力了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="inlineStr">
+        <is>
+          <t>CHI-20260929-014</t>
+        </is>
+      </c>
+      <c r="B1218" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1218" t="inlineStr">
+        <is>
+          <t>盘点</t>
+        </is>
+      </c>
+      <c r="E1218" t="inlineStr">
+        <is>
+          <t>오피스 표현</t>
+        </is>
+      </c>
+      <c r="F1218" t="inlineStr">
+        <is>
+          <t>pán diǎn</t>
+        </is>
+      </c>
+      <c r="G1218" t="inlineStr">
+        <is>
+          <t>정리하다, 총괄하다</t>
+        </is>
+      </c>
+      <c r="H1218" t="inlineStr">
+        <is>
+          <t>各大高校借华诞之机，盘点过去的发展成就。</t>
+        </is>
+      </c>
+      <c r="I1218" t="inlineStr">
+        <is>
+          <t>年末了，我们来盘点一下今年的工作成果。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="inlineStr">
+        <is>
+          <t>CHI-20260929-015</t>
+        </is>
+      </c>
+      <c r="B1219" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1219" t="inlineStr">
+        <is>
+          <t>靠山</t>
+        </is>
+      </c>
+      <c r="E1219" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1219" t="inlineStr">
+        <is>
+          <t>kào shān</t>
+        </is>
+      </c>
+      <c r="G1219" t="inlineStr">
+        <is>
+          <t>든든한 배경, 의지할 곳</t>
+        </is>
+      </c>
+      <c r="H1219" t="inlineStr">
+        <is>
+          <t>对于民企来说，完善的制度就是最好的靠山。</t>
+        </is>
+      </c>
+      <c r="I1219" t="inlineStr">
+        <is>
+          <t>靠山山倒，靠人人跑，最后还是得靠自己。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-30 | 1232/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1219"/>
+  <dimension ref="A1:I1233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -57709,6 +57709,664 @@
         </is>
       </c>
     </row>
+    <row r="1220">
+      <c r="A1220" t="inlineStr">
+        <is>
+          <t>CHI-20260930-001</t>
+        </is>
+      </c>
+      <c r="B1220" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1220" t="inlineStr">
+        <is>
+          <t>民生福祉</t>
+        </is>
+      </c>
+      <c r="E1220" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1220" t="inlineStr">
+        <is>
+          <t>mín shēng fú zhǐ</t>
+        </is>
+      </c>
+      <c r="G1220" t="inlineStr">
+        <is>
+          <t>국민의 실질적인 삶의 질과 행복</t>
+        </is>
+      </c>
+      <c r="H1220" t="inlineStr">
+        <is>
+          <t>정부 정책이나 공공 사업이 국민의 실제 생활과 행복에 미치는 영향력을 강조할 때</t>
+        </is>
+      </c>
+      <c r="I1220" t="inlineStr">
+        <is>
+          <t>我们要把民生福祉放在首位，切实解决老百姓的急难愁盼问题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="inlineStr">
+        <is>
+          <t>CHI-20260930-002</t>
+        </is>
+      </c>
+      <c r="B1221" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1221" t="inlineStr">
+        <is>
+          <t>烟火气</t>
+        </is>
+      </c>
+      <c r="E1221" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1221" t="inlineStr">
+        <is>
+          <t>yān huǒ qì</t>
+        </is>
+      </c>
+      <c r="G1221" t="inlineStr">
+        <is>
+          <t>사람 사는 냄새, 소소하고 활기찬 일상의 정취</t>
+        </is>
+      </c>
+      <c r="H1221" t="inlineStr">
+        <is>
+          <t>도시의 활기찬 거리, 야시장, 식당 등 인간미 넘치는 공간을 묘사할 때</t>
+        </is>
+      </c>
+      <c r="I1221" t="inlineStr">
+        <is>
+          <t>这条老街改造得很好，既保留了浓浓的烟火气，又显得非常整洁。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr">
+        <is>
+          <t>CHI-20260930-003</t>
+        </is>
+      </c>
+      <c r="B1222" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1222" t="inlineStr">
+        <is>
+          <t>不让...等</t>
+        </is>
+      </c>
+      <c r="E1222" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1222" t="inlineStr">
+        <is>
+          <t>bù ràng ... děng</t>
+        </is>
+      </c>
+      <c r="G1222" t="inlineStr">
+        <is>
+          <t>기다리게 하지 않다(효율적인 업무 처리 강조)</t>
+        </is>
+      </c>
+      <c r="H1222" t="inlineStr">
+        <is>
+          <t>프로젝트나 자금 집행이 지체 없이 즉각적으로 이루어져야 함을 강조할 때</t>
+        </is>
+      </c>
+      <c r="I1222" t="inlineStr">
+        <is>
+          <t>我们要提高审批效率，真正做到不让项目等资金，不让企业等政策。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="inlineStr">
+        <is>
+          <t>CHI-20260930-004</t>
+        </is>
+      </c>
+      <c r="B1223" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1223" t="inlineStr">
+        <is>
+          <t>入脑入心</t>
+        </is>
+      </c>
+      <c r="E1223" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1223" t="inlineStr">
+        <is>
+          <t>rù nǎo rù xīn</t>
+        </is>
+      </c>
+      <c r="G1223" t="inlineStr">
+        <is>
+          <t>완전히 이해하고 마음 깊이 새기다</t>
+        </is>
+      </c>
+      <c r="H1223" t="inlineStr">
+        <is>
+          <t>교육이나 사상 전달이 형식적이지 않고 개인의 가치관에 실질적인 변화를 줄 때</t>
+        </is>
+      </c>
+      <c r="I1223" t="inlineStr">
+        <is>
+          <t>这次环保宣讲活动非常生动，真正做到了让绿色理念入脑入心。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="inlineStr">
+        <is>
+          <t>CHI-20260930-005</t>
+        </is>
+      </c>
+      <c r="B1224" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1224" t="inlineStr">
+        <is>
+          <t>两高项目</t>
+        </is>
+      </c>
+      <c r="E1224" t="inlineStr">
+        <is>
+          <t>오피스 표현</t>
+        </is>
+      </c>
+      <c r="F1224" t="inlineStr">
+        <is>
+          <t>liǎng gāo xiàng mù</t>
+        </is>
+      </c>
+      <c r="G1224" t="inlineStr">
+        <is>
+          <t>고에너지 소비 및 고오염 배출 프로젝트</t>
+        </is>
+      </c>
+      <c r="H1224" t="inlineStr">
+        <is>
+          <t>환경 규제 대상이 되는 산업 시설이나 개발 사업을 지칭할 때</t>
+        </is>
+      </c>
+      <c r="I1224" t="inlineStr">
+        <is>
+          <t>政府明确要求严控两高项目，加快推动产业结构绿色转型。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="inlineStr">
+        <is>
+          <t>CHI-20260930-006</t>
+        </is>
+      </c>
+      <c r="B1225" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1225" t="inlineStr">
+        <is>
+          <t>一站式</t>
+        </is>
+      </c>
+      <c r="E1225" t="inlineStr">
+        <is>
+          <t>오피스 표현</t>
+        </is>
+      </c>
+      <c r="F1225" t="inlineStr">
+        <is>
+          <t>yī zhàn shì</t>
+        </is>
+      </c>
+      <c r="G1225" t="inlineStr">
+        <is>
+          <t>원스톱 서비스, 통합 처리</t>
+        </is>
+      </c>
+      <c r="H1225" t="inlineStr">
+        <is>
+          <t>고객의 번거로움을 줄이기 위해 여러 과정을 한곳에서 해결하는 비즈니스 모델</t>
+        </is>
+      </c>
+      <c r="I1225" t="inlineStr">
+        <is>
+          <t>我们提供装修一站式服务，从设计到材料配送全部包办。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="inlineStr">
+        <is>
+          <t>CHI-20260930-007</t>
+        </is>
+      </c>
+      <c r="B1226" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1226" t="inlineStr">
+        <is>
+          <t>伪环保</t>
+        </is>
+      </c>
+      <c r="E1226" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1226" t="inlineStr">
+        <is>
+          <t>wěi huán bǎo</t>
+        </is>
+      </c>
+      <c r="G1226" t="inlineStr">
+        <is>
+          <t>가짜 친환경, 그린워싱</t>
+        </is>
+      </c>
+      <c r="H1226" t="inlineStr">
+        <is>
+          <t>친환경을 마케팅 수단으로만 이용하고 실제로는 효과가 없는 제품이나 기업을 비판할 때</t>
+        </is>
+      </c>
+      <c r="I1226" t="inlineStr">
+        <is>
+          <t>很多商家打着伪环保的旗号欺骗消费者，必须加强监管。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="inlineStr">
+        <is>
+          <t>CHI-20260930-008</t>
+        </is>
+      </c>
+      <c r="B1227" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1227" t="inlineStr">
+        <is>
+          <t>看穿</t>
+        </is>
+      </c>
+      <c r="E1227" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1227" t="inlineStr">
+        <is>
+          <t>kàn chuān</t>
+        </is>
+      </c>
+      <c r="G1227" t="inlineStr">
+        <is>
+          <t>꿰뚫어 보다, 진실을 간파하다</t>
+        </is>
+      </c>
+      <c r="H1227" t="inlineStr">
+        <is>
+          <t>겉모습에 속지 않고 본질이나 의도를 정확히 파악할 때</t>
+        </is>
+      </c>
+      <c r="I1227" t="inlineStr">
+        <is>
+          <t>无论他怎么掩饰，我一眼就看穿了他的真实意图。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="inlineStr">
+        <is>
+          <t>CHI-20260930-009</t>
+        </is>
+      </c>
+      <c r="B1228" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1228" t="inlineStr">
+        <is>
+          <t>保研</t>
+        </is>
+      </c>
+      <c r="E1228" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1228" t="inlineStr">
+        <is>
+          <t>bǎo yán</t>
+        </is>
+      </c>
+      <c r="G1228" t="inlineStr">
+        <is>
+          <t>대학원 무시험 입학(추천 전형)</t>
+        </is>
+      </c>
+      <c r="H1228" t="inlineStr">
+        <is>
+          <t>우수한 성적으로 시험을 보지 않고 대학원에 진학하는 상황을 말할 때</t>
+        </is>
+      </c>
+      <c r="I1228" t="inlineStr">
+        <is>
+          <t>她凭借优异的科研表现，大四那年成功获得了保研资格。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="inlineStr">
+        <is>
+          <t>CHI-20260930-010</t>
+        </is>
+      </c>
+      <c r="B1229" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1229" t="inlineStr">
+        <is>
+          <t>敲门砖</t>
+        </is>
+      </c>
+      <c r="E1229" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1229" t="inlineStr">
+        <is>
+          <t>qiāo mén zhuān</t>
+        </is>
+      </c>
+      <c r="G1229" t="inlineStr">
+        <is>
+          <t>성공으로 가는 발판, 입구에서 문을 두드리는 도구(수단)</t>
+        </is>
+      </c>
+      <c r="H1229" t="inlineStr">
+        <is>
+          <t>취업이나 성공을 위해 필요한 자격증, 학위, 경력 등을 비유할 때</t>
+        </is>
+      </c>
+      <c r="I1229" t="inlineStr">
+        <is>
+          <t>这份实习经验是他进入顶级外企的一块敲门砖。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="inlineStr">
+        <is>
+          <t>CHI-20260930-011</t>
+        </is>
+      </c>
+      <c r="B1230" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1230" t="inlineStr">
+        <is>
+          <t>多点攻坚</t>
+        </is>
+      </c>
+      <c r="E1230" t="inlineStr">
+        <is>
+          <t>오피스 표현</t>
+        </is>
+      </c>
+      <c r="F1230" t="inlineStr">
+        <is>
+          <t>duō diǎn gōng jiān</t>
+        </is>
+      </c>
+      <c r="G1230" t="inlineStr">
+        <is>
+          <t>다방면에서 난제를 돌파하다</t>
+        </is>
+      </c>
+      <c r="H1230" t="inlineStr">
+        <is>
+          <t>기업이나 정부가 여러 핵심 과제를 동시에 해결해 나갈 때</t>
+        </is>
+      </c>
+      <c r="I1230" t="inlineStr">
+        <is>
+          <t>公司通过多点攻坚，终于在核心技术领域取得了重大突破。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="inlineStr">
+        <is>
+          <t>CHI-20260930-012</t>
+        </is>
+      </c>
+      <c r="B1231" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C1231" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1231" t="inlineStr">
+        <is>
+          <t>零时差</t>
+        </is>
+      </c>
+      <c r="E1231" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1231" t="inlineStr">
+        <is>
+          <t>líng shí chā</t>
+        </is>
+      </c>
+      <c r="G1231" t="inlineStr">
+        <is>
+          <t>실시간의, 지체 없는</t>
+        </is>
+      </c>
+      <c r="H1231" t="inlineStr">
+        <is>
+          <t>정보 전달이나 업무 처리가 즉각적임을 강조할 때</t>
+        </is>
+      </c>
+      <c r="I1231" t="inlineStr">
+        <is>
+          <t>通过这款软件，你可以零时差获取最新的市场资讯。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="inlineStr">
+        <is>
+          <t>CHI-20260930-013</t>
+        </is>
+      </c>
+      <c r="B1232" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C1232" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1232" t="inlineStr">
+        <is>
+          <t>抱大腿</t>
+        </is>
+      </c>
+      <c r="E1232" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1232" t="inlineStr">
+        <is>
+          <t>bào dà tuǐ</t>
+        </is>
+      </c>
+      <c r="G1232" t="inlineStr">
+        <is>
+          <t>유력자에게 빌붙다, 강자의 도움을 받으려 하다</t>
+        </is>
+      </c>
+      <c r="H1232" t="inlineStr">
+        <is>
+          <t>힘 있는 사람이나 기업의 도움으로 이득을 보려 할 때(약간의 비꼬는 어조)</t>
+        </is>
+      </c>
+      <c r="I1232" t="inlineStr">
+        <is>
+          <t>他为了拿到项目，到处找机会去抱大腿。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="inlineStr">
+        <is>
+          <t>CHI-20260930-014</t>
+        </is>
+      </c>
+      <c r="B1233" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C1233" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1233" t="inlineStr">
+        <is>
+          <t>断崖式</t>
+        </is>
+      </c>
+      <c r="E1233" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1233" t="inlineStr">
+        <is>
+          <t>duàn yá shì</t>
+        </is>
+      </c>
+      <c r="G1233" t="inlineStr">
+        <is>
+          <t>급격한, 절벽처럼 뚝 떨어진</t>
+        </is>
+      </c>
+      <c r="H1233" t="inlineStr">
+        <is>
+          <t>수치나 상태가 순식간에 크게 변화했을 때</t>
+        </is>
+      </c>
+      <c r="I1233" t="inlineStr">
+        <is>
+          <t>由于管理不善，公司业绩出现了断崖式下跌。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-10-01 | 1245/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1233"/>
+  <dimension ref="A1:I1246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -58367,6 +58367,617 @@
         </is>
       </c>
     </row>
+    <row r="1234">
+      <c r="A1234" t="inlineStr">
+        <is>
+          <t>CHI-20261001-001</t>
+        </is>
+      </c>
+      <c r="B1234" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C1234" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1234" t="inlineStr">
+        <is>
+          <t>键盘侠</t>
+        </is>
+      </c>
+      <c r="E1234" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1234" t="inlineStr">
+        <is>
+          <t>jiàn pán xiá</t>
+        </is>
+      </c>
+      <c r="G1234" t="inlineStr">
+        <is>
+          <t>키보드 워리어 (인터넷에서 무책임하게 비난을 퍼붓는 사람들)</t>
+        </is>
+      </c>
+      <c r="H1234" t="inlineStr">
+        <is>
+          <t>现在网上的键盘侠太多了，那个高考誓师被网暴的女孩心理承受力真的很强。</t>
+        </is>
+      </c>
+      <c r="I1234" t="inlineStr">
+        <is>
+          <t>我们别理那些键盘侠，做好自己的事情就行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="inlineStr">
+        <is>
+          <t>CHI-20261001-002</t>
+        </is>
+      </c>
+      <c r="B1235" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C1235" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1235" t="inlineStr">
+        <is>
+          <t>大惊小怪</t>
+        </is>
+      </c>
+      <c r="E1235" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1235" t="inlineStr">
+        <is>
+          <t>dài jīng xiǎo guài</t>
+        </is>
+      </c>
+      <c r="G1235" t="inlineStr">
+        <is>
+          <t>사소한 일에 호들갑을 떨다 (별것 아닌 일에 크게 놀라다)</t>
+        </is>
+      </c>
+      <c r="H1235" t="inlineStr">
+        <is>
+          <t>孩子一开学感冒发烧是常有的事，家长不用大惊小怪，做好防护就行。</t>
+        </is>
+      </c>
+      <c r="I1235" t="inlineStr">
+        <is>
+          <t>他不过是换了个发型，大家没必要大惊小怪的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="inlineStr">
+        <is>
+          <t>CHI-20261001-003</t>
+        </is>
+      </c>
+      <c r="B1236" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C1236" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1236" t="inlineStr">
+        <is>
+          <t>舍得</t>
+        </is>
+      </c>
+      <c r="E1236" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1236" t="inlineStr">
+        <is>
+          <t>shě de</t>
+        </is>
+      </c>
+      <c r="G1236" t="inlineStr">
+        <is>
+          <t>기꺼이 쓰다 (돈, 시간, 감정 등을 아까워하지 않다)</t>
+        </is>
+      </c>
+      <c r="H1236" t="inlineStr">
+        <is>
+          <t>现在的家长为了孩子的教育真的很舍得花钱，但报班不如把钱花在刀刃上。</t>
+        </is>
+      </c>
+      <c r="I1236" t="inlineStr">
+        <is>
+          <t>只要能提升专业技能，他花多少学费都舍得。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" t="inlineStr">
+        <is>
+          <t>CHI-20261001-004</t>
+        </is>
+      </c>
+      <c r="B1237" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C1237" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1237" t="inlineStr">
+        <is>
+          <t>格局</t>
+        </is>
+      </c>
+      <c r="E1237" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1237" t="inlineStr">
+        <is>
+          <t>gé jú</t>
+        </is>
+      </c>
+      <c r="G1237" t="inlineStr">
+        <is>
+          <t>그릇, 안목 (생각의 크기나 시야의 넓이)</t>
+        </is>
+      </c>
+      <c r="H1237" t="inlineStr">
+        <is>
+          <t>始终把自身发展放在全球坐标系中，体现了大国的外交格局和担当。</t>
+        </is>
+      </c>
+      <c r="I1237" t="inlineStr">
+        <is>
+          <t>做生意要有大格局，不能光盯着眼前的这一点小利益。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" t="inlineStr">
+        <is>
+          <t>CHI-20261001-005</t>
+        </is>
+      </c>
+      <c r="B1238" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C1238" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1238" t="inlineStr">
+        <is>
+          <t>放眼未来</t>
+        </is>
+      </c>
+      <c r="E1238" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1238" t="inlineStr">
+        <is>
+          <t>fàng yǎn wèi lái</t>
+        </is>
+      </c>
+      <c r="G1238" t="inlineStr">
+        <is>
+          <t>미래를 내다보다 (먼 앞날을 향해 시선을 돌리다)</t>
+        </is>
+      </c>
+      <c r="H1238" t="inlineStr">
+        <is>
+          <t>中俄两国关系的发展不仅要立足当下，更要放眼未来，实现深层合作。</t>
+        </is>
+      </c>
+      <c r="I1238" t="inlineStr">
+        <is>
+          <t>我们在规划职业生涯时，应该放眼未来，多储备一些核心技能。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" t="inlineStr">
+        <is>
+          <t>CHI-20261001-006</t>
+        </is>
+      </c>
+      <c r="B1239" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C1239" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1239" t="inlineStr">
+        <is>
+          <t>自食其果</t>
+        </is>
+      </c>
+      <c r="E1239" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1239" t="inlineStr">
+        <is>
+          <t>zì shí qí guǒ</t>
+        </is>
+      </c>
+      <c r="G1239" t="inlineStr">
+        <is>
+          <t>자업자득 (스스로 저지른 잘못으로 인해 나쁜 결과를 얻다)</t>
+        </is>
+      </c>
+      <c r="H1239" t="inlineStr">
+        <is>
+          <t>有些国家用环保法搞贸易壁垒，最后很可能会自食其果，伤害自己的产业。</t>
+        </is>
+      </c>
+      <c r="I1239" t="inlineStr">
+        <is>
+          <t>他在工作中总是弄虚作假，这次被公司开除纯属自食其果。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" t="inlineStr">
+        <is>
+          <t>CHI-20261001-007</t>
+        </is>
+      </c>
+      <c r="B1240" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C1240" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1240" t="inlineStr">
+        <is>
+          <t>拔苗助长</t>
+        </is>
+      </c>
+      <c r="E1240" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1240" t="inlineStr">
+        <is>
+          <t>bá miáo zhù zhǎng</t>
+        </is>
+      </c>
+      <c r="G1240" t="inlineStr">
+        <is>
+          <t>급하게 서두르다 도리어 일을 그르치다</t>
+        </is>
+      </c>
+      <c r="H1240" t="inlineStr">
+        <is>
+          <t>辅导班不是万能药，家长如果盲目拔苗助长，反而会消磨孩子的学习兴趣。</t>
+        </is>
+      </c>
+      <c r="I1240" t="inlineStr">
+        <is>
+          <t>培养新员工要循序渐进，过度施压只会拔苗助长，让他们产生抗拒。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" t="inlineStr">
+        <is>
+          <t>CHI-20261001-008</t>
+        </is>
+      </c>
+      <c r="B1241" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C1241" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1241" t="inlineStr">
+        <is>
+          <t>说一套，做一套</t>
+        </is>
+      </c>
+      <c r="E1241" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1241" t="inlineStr">
+        <is>
+          <t>shuō yī tào, zuò yī tào</t>
+        </is>
+      </c>
+      <c r="G1241" t="inlineStr">
+        <is>
+          <t>말과 행동이 전혀 다르다 (언행불일치)</t>
+        </is>
+      </c>
+      <c r="H1241" t="inlineStr">
+        <is>
+          <t>某些国家表面上呼吁和平解决国际争端，背地里却说一套做一套，暗中挑拨。</t>
+        </is>
+      </c>
+      <c r="I1241" t="inlineStr">
+        <is>
+          <t>我最讨厌那种说一套做一套的人，跟他们合作一点安全感都没有。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" t="inlineStr">
+        <is>
+          <t>CHI-20261001-009</t>
+        </is>
+      </c>
+      <c r="B1242" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C1242" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1242" t="inlineStr">
+        <is>
+          <t>想不开</t>
+        </is>
+      </c>
+      <c r="E1242" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1242" t="inlineStr">
+        <is>
+          <t>xiǎng bù kāi</t>
+        </is>
+      </c>
+      <c r="G1242" t="inlineStr">
+        <is>
+          <t>마음을 열지 못하고 비관하다 (스스로 갇혀 부정적인 생각을 고수하다)</t>
+        </is>
+      </c>
+      <c r="H1242" t="inlineStr">
+        <is>
+          <t>面对网络暴力，很多年轻人心理脆弱容易想不开，这时候需要及时疏导。</t>
+        </is>
+      </c>
+      <c r="I1242" t="inlineStr">
+        <is>
+          <t>考试没考好没关系，你可千万别想不开，下次再努力就是了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="inlineStr">
+        <is>
+          <t>CHI-20261001-010</t>
+        </is>
+      </c>
+      <c r="B1243" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C1243" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1243" t="inlineStr">
+        <is>
+          <t>眼光</t>
+        </is>
+      </c>
+      <c r="E1243" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1243" t="inlineStr">
+        <is>
+          <t>yǎn guāng</t>
+        </is>
+      </c>
+      <c r="G1243" t="inlineStr">
+        <is>
+          <t>트렌드나 가치를 꿰뚫어 보는 안목</t>
+        </is>
+      </c>
+      <c r="H1243" t="inlineStr">
+        <is>
+          <t>优秀的投资机构往往有独到的眼光，能提前布局具有潜力的绿色低碳场景。</t>
+        </is>
+      </c>
+      <c r="I1243" t="inlineStr">
+        <is>
+          <t>他的投资眼光真的很毒辣，几年前买的那几只股票现在都翻倍了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="inlineStr">
+        <is>
+          <t>CHI-20261001-011</t>
+        </is>
+      </c>
+      <c r="B1244" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C1244" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1244" t="inlineStr">
+        <is>
+          <t>对胃口</t>
+        </is>
+      </c>
+      <c r="E1244" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1244" t="inlineStr">
+        <is>
+          <t>duì wèi kǒu</t>
+        </is>
+      </c>
+      <c r="G1244" t="inlineStr">
+        <is>
+          <t>취향이나 마음에 딱 들어맞다 (입맛에 맞다)</t>
+        </is>
+      </c>
+      <c r="H1244" t="inlineStr">
+        <is>
+          <t>这种简单、标准化的智能家装方案非常对年轻人的胃口，市场反应很好。</t>
+        </is>
+      </c>
+      <c r="I1244" t="inlineStr">
+        <is>
+          <t>这部职场剧的剧情非常对我的胃口，节奏紧凑而且一点也不狗血。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" t="inlineStr">
+        <is>
+          <t>CHI-20261001-012</t>
+        </is>
+      </c>
+      <c r="B1245" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C1245" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1245" t="inlineStr">
+        <is>
+          <t>诉苦</t>
+        </is>
+      </c>
+      <c r="E1245" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1245" t="inlineStr">
+        <is>
+          <t>sù kǔ</t>
+        </is>
+      </c>
+      <c r="G1245" t="inlineStr">
+        <is>
+          <t>고충을 털어놓다, 하소연하다, 푸념하다</t>
+        </is>
+      </c>
+      <c r="H1245" t="inlineStr">
+        <is>
+          <t>面对高强度的备考压力，很多考生会选择向朋友或老师诉苦来释放情绪。</t>
+        </is>
+      </c>
+      <c r="I1245" t="inlineStr">
+        <is>
+          <t>遇到困难时，与其坐在这里诉苦，不如起而行之去寻找解决方案。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="inlineStr">
+        <is>
+          <t>CHI-20261001-013</t>
+        </is>
+      </c>
+      <c r="B1246" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C1246" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1246" t="inlineStr">
+        <is>
+          <t>分心</t>
+        </is>
+      </c>
+      <c r="E1246" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1246" t="inlineStr">
+        <is>
+          <t>fēn xīn</t>
+        </is>
+      </c>
+      <c r="G1246" t="inlineStr">
+        <is>
+          <t>정신을 팔다, 한눈을 팔다, 신경이 분산되다</t>
+        </is>
+      </c>
+      <c r="H1246" t="inlineStr">
+        <is>
+          <t>在关键的冲刺阶段，考生们千万不要因为网络上的杂音而分心。</t>
+        </is>
+      </c>
+      <c r="I1246" t="inlineStr">
+        <is>
+          <t>边开车边看手机极易分心，为了安全起见，千万不可尝试。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-10-02 | 1250/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1246"/>
+  <dimension ref="A1:I1251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -58978,6 +58978,241 @@
         </is>
       </c>
     </row>
+    <row r="1247">
+      <c r="A1247" t="inlineStr">
+        <is>
+          <t>CHI-20261002-001</t>
+        </is>
+      </c>
+      <c r="B1247" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C1247" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1247" t="inlineStr">
+        <is>
+          <t>示弱</t>
+        </is>
+      </c>
+      <c r="E1247" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1247" t="inlineStr">
+        <is>
+          <t>shì ruò</t>
+        </is>
+      </c>
+      <c r="G1247" t="inlineStr">
+        <is>
+          <t>자신의 약함을 보여주다, 져주며 양보하다</t>
+        </is>
+      </c>
+      <c r="H1247" t="inlineStr">
+        <is>
+          <t>有时候，管理班级或团队也需要智慧，适度示弱能让下属或学生更主动地承担责任。</t>
+        </is>
+      </c>
+      <c r="I1247" t="inlineStr">
+        <is>
+          <t>在人际交往中，适当示弱不仅不会丢面子，反而能拉近彼此的距离。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="inlineStr">
+        <is>
+          <t>CHI-20261002-002</t>
+        </is>
+      </c>
+      <c r="B1248" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C1248" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1248" t="inlineStr">
+        <is>
+          <t>报班</t>
+        </is>
+      </c>
+      <c r="E1248" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1248" t="inlineStr">
+        <is>
+          <t>bào bān</t>
+        </is>
+      </c>
+      <c r="G1248" t="inlineStr">
+        <is>
+          <t>학원 반에 등록하다, 사교육 수업을 신청하다</t>
+        </is>
+      </c>
+      <c r="H1248" t="inlineStr">
+        <is>
+          <t>现在的家长总是急着给中学生报班，其实一些陪伴和引导比盲目报辅导班更有价值。</t>
+        </is>
+      </c>
+      <c r="I1248" t="inlineStr">
+        <is>
+          <t>为了下个月的中文口语考试，我特意去报了一个一对一的口语提升班。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="inlineStr">
+        <is>
+          <t>CHI-20261002-003</t>
+        </is>
+      </c>
+      <c r="B1249" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C1249" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1249" t="inlineStr">
+        <is>
+          <t>瞎折腾</t>
+        </is>
+      </c>
+      <c r="E1249" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1249" t="inlineStr">
+        <is>
+          <t>xiā zhē teng</t>
+        </is>
+      </c>
+      <c r="G1249" t="inlineStr">
+        <is>
+          <t>쓸데없이 일을 벌여 고생하다, 부질없는 짓으로 헛수고하다</t>
+        </is>
+      </c>
+      <c r="H1249" t="inlineStr">
+        <is>
+          <t>环保工作不能光在表面上瞎折腾，而要把绿色环保理念真正落实到社区居民的日常生活中。</t>
+        </is>
+      </c>
+      <c r="I1249" t="inlineStr">
+        <is>
+          <t>方案都已经定好了，你就别再瞎折腾改来改去了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="inlineStr">
+        <is>
+          <t>CHI-20261002-004</t>
+        </is>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C1250" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1250" t="inlineStr">
+        <is>
+          <t>风雨无阻</t>
+        </is>
+      </c>
+      <c r="E1250" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1250" t="inlineStr">
+        <is>
+          <t>fēng yǔ wú zǔ</t>
+        </is>
+      </c>
+      <c r="G1250" t="inlineStr">
+        <is>
+          <t>비바람이 불어도 아랑곳하지 않다, 날씨에 상관없이 예정대로 진행하다</t>
+        </is>
+      </c>
+      <c r="H1250" t="inlineStr">
+        <is>
+          <t>国庆假期期间，城管人员风雨无阻地守护着城市秩序。</t>
+        </is>
+      </c>
+      <c r="I1250" t="inlineStr">
+        <is>
+          <t>无论刮风下雨，他都风雨无阻地坚持每天早上跑步。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="inlineStr">
+        <is>
+          <t>CHI-20261002-005</t>
+        </is>
+      </c>
+      <c r="B1251" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C1251" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1251" t="inlineStr">
+        <is>
+          <t>息息相关</t>
+        </is>
+      </c>
+      <c r="E1251" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1251" t="inlineStr">
+        <is>
+          <t>xī xī xiāng guān</t>
+        </is>
+      </c>
+      <c r="G1251" t="inlineStr">
+        <is>
+          <t>밀접한 관계가 있다, 숨결을 같이하다</t>
+        </is>
+      </c>
+      <c r="H1251" t="inlineStr">
+        <is>
+          <t>民生福祉与国家的各项改革政策息息相关。</t>
+        </is>
+      </c>
+      <c r="I1251" t="inlineStr">
+        <is>
+          <t>环境保护与我们每个人的身体健康息息相关。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-10-05 | 1278/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1251"/>
+  <dimension ref="A1:I1279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -59213,6 +59213,1322 @@
         </is>
       </c>
     </row>
+    <row r="1252">
+      <c r="A1252" t="inlineStr">
+        <is>
+          <t>CHI-20261005-001</t>
+        </is>
+      </c>
+      <c r="B1252" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1252" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1252" t="inlineStr">
+        <is>
+          <t>中招</t>
+        </is>
+      </c>
+      <c r="E1252" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1252" t="inlineStr">
+        <is>
+          <t>zhòng zhāo</t>
+        </is>
+      </c>
+      <c r="G1252" t="inlineStr">
+        <is>
+          <t>사기를 당하다, 수법에 걸려들다, (감기/코로나 등에) 걸리다</t>
+        </is>
+      </c>
+      <c r="H1252" t="inlineStr">
+        <is>
+          <t>现在网上有很多虚假的抢票平台，一不小心就会中招，大家一定要提高警惕。</t>
+        </is>
+      </c>
+      <c r="I1252" t="inlineStr">
+        <is>
+          <t>听说最近流行一种新型的电信诈骗，好多人都中招了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="inlineStr">
+        <is>
+          <t>CHI-20261005-002</t>
+        </is>
+      </c>
+      <c r="B1253" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1253" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1253" t="inlineStr">
+        <is>
+          <t>人满为患</t>
+        </is>
+      </c>
+      <c r="E1253" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1253" t="inlineStr">
+        <is>
+          <t>rén mǎn wéi huàn</t>
+        </is>
+      </c>
+      <c r="G1253" t="inlineStr">
+        <is>
+          <t>인산인해를 이루다, 사람들로 미어터지다</t>
+        </is>
+      </c>
+      <c r="H1253" t="inlineStr">
+        <is>
+          <t>国庆假期的西藏博物馆人满为患，每天一开馆排队的队伍就排到了街角。</t>
+        </is>
+      </c>
+      <c r="I1253" t="inlineStr">
+        <is>
+          <t>每逢周末，这家网红餐厅就人满为患，不提前预约根本没有位置。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="inlineStr">
+        <is>
+          <t>CHI-20261005-003</t>
+        </is>
+      </c>
+      <c r="B1254" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1254" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1254" t="inlineStr">
+        <is>
+          <t>计划赶不上变化</t>
+        </is>
+      </c>
+      <c r="E1254" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1254" t="inlineStr">
+        <is>
+          <t>jì huà gǎn bu shàng biàn huà</t>
+        </is>
+      </c>
+      <c r="G1254" t="inlineStr">
+        <is>
+          <t>계획은 변화를 따라갈 수 없다 (세상일은 뜻대로 되지 않는다)</t>
+        </is>
+      </c>
+      <c r="H1254" t="inlineStr">
+        <is>
+          <t>本来计划国庆假期去宁夏看丰收景色的，结果临时接到通知要加班，真是计划赶不上变化。</t>
+        </is>
+      </c>
+      <c r="I1254" t="inlineStr">
+        <is>
+          <t>别把行程安排得太满，计划赶不上变化，我们要留出一些机动时间。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="inlineStr">
+        <is>
+          <t>CHI-20261005-004</t>
+        </is>
+      </c>
+      <c r="B1255" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1255" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1255" t="inlineStr">
+        <is>
+          <t>办喜事</t>
+        </is>
+      </c>
+      <c r="E1255" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1255" t="inlineStr">
+        <is>
+          <t>bàn xǐ shì</t>
+        </is>
+      </c>
+      <c r="G1255" t="inlineStr">
+        <is>
+          <t>혼사를 치르다, 집안에 경사스러운 행사를 열다</t>
+        </is>
+      </c>
+      <c r="H1255" t="inlineStr">
+        <is>
+          <t>桦川县红光村的村民们现在办喜事都倡导简朴风尚，不仅省钱还很有意义。</t>
+        </is>
+      </c>
+      <c r="I1255" t="inlineStr">
+        <is>
+          <t>我们家下个月要办喜事，我哥要结婚了，这几天全家人都在忙着筹备。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" t="inlineStr">
+        <is>
+          <t>CHI-20261005-005</t>
+        </is>
+      </c>
+      <c r="B1256" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1256" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1256" t="inlineStr">
+        <is>
+          <t>讲排场</t>
+        </is>
+      </c>
+      <c r="E1256" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1256" t="inlineStr">
+        <is>
+          <t>jiǎng pái chǎng</t>
+        </is>
+      </c>
+      <c r="G1256" t="inlineStr">
+        <is>
+          <t>체면치레를 하다, 겉치레를 중요시하다</t>
+        </is>
+      </c>
+      <c r="H1256" t="inlineStr">
+        <is>
+          <t>现在的年轻人结婚越来越不讲排场了，他们更喜欢温馨、有个性的草坪婚礼。</t>
+        </is>
+      </c>
+      <c r="I1256" t="inlineStr">
+        <is>
+          <t>请客吃饭最重要的是大家开心，没必要为了讲排场而点一桌子吃不完的菜。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="inlineStr">
+        <is>
+          <t>CHI-20261005-006</t>
+        </is>
+      </c>
+      <c r="B1257" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1257" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1257" t="inlineStr">
+        <is>
+          <t>耍到晚</t>
+        </is>
+      </c>
+      <c r="E1257" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1257" t="inlineStr">
+        <is>
+          <t>shuǎ dào wǎn</t>
+        </is>
+      </c>
+      <c r="G1257" t="inlineStr">
+        <is>
+          <t>밤까지 놀다, 하루 종일 즐겁게 놀다</t>
+        </is>
+      </c>
+      <c r="H1257" t="inlineStr">
+        <is>
+          <t>到成都洛带从早耍到晚.</t>
+        </is>
+      </c>
+      <c r="I1257" t="inlineStr">
+        <is>
+          <t>周末我们约好去游乐场，从早到晚耍到晚，玩得非常开心。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="inlineStr">
+        <is>
+          <t>CHI-20261005-007</t>
+        </is>
+      </c>
+      <c r="B1258" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1258" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1258" t="inlineStr">
+        <is>
+          <t>游人如织</t>
+        </is>
+      </c>
+      <c r="E1258" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1258" t="inlineStr">
+        <is>
+          <t>yóu rén rú zhī</t>
+        </is>
+      </c>
+      <c r="G1258" t="inlineStr">
+        <is>
+          <t>관광객이 베틀의 실처럼 붐비다(인산인해를 이루다)</t>
+        </is>
+      </c>
+      <c r="H1258" t="inlineStr">
+        <is>
+          <t>西藏博物馆国庆假期游人如织.</t>
+        </is>
+      </c>
+      <c r="I1258" t="inlineStr">
+        <is>
+          <t>国庆长假期间，著名的旅游景点到处是游人如织的景象。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="inlineStr">
+        <is>
+          <t>CHI-20261005-008</t>
+        </is>
+      </c>
+      <c r="B1259" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1259" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1259" t="inlineStr">
+        <is>
+          <t>蝶变</t>
+        </is>
+      </c>
+      <c r="E1259" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1259" t="inlineStr">
+        <is>
+          <t>dié biàn</t>
+        </is>
+      </c>
+      <c r="G1259" t="inlineStr">
+        <is>
+          <t>나비가 되듯 극적인 탈바꿈/변화</t>
+        </is>
+      </c>
+      <c r="H1259" t="inlineStr">
+        <is>
+          <t>十年蝶变新丝路.</t>
+        </is>
+      </c>
+      <c r="I1259" t="inlineStr">
+        <is>
+          <t>这片曾经的荒地经过改造，终于迎来了华丽的蝶变。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="inlineStr">
+        <is>
+          <t>CHI-20261005-009</t>
+        </is>
+      </c>
+      <c r="B1260" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1260" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1260" t="inlineStr">
+        <is>
+          <t>提质焕新</t>
+        </is>
+      </c>
+      <c r="E1260" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1260" t="inlineStr">
+        <is>
+          <t>tí zhì huàn xīn</t>
+        </is>
+      </c>
+      <c r="G1260" t="inlineStr">
+        <is>
+          <t>품질을 높이고 새롭게 바꾸다(개보수)</t>
+        </is>
+      </c>
+      <c r="H1260" t="inlineStr">
+        <is>
+          <t>济南黄河大桥大修提质焕新.</t>
+        </is>
+      </c>
+      <c r="I1260" t="inlineStr">
+        <is>
+          <t>老旧社区经过政府的提质焕新工程，环境变得越来越宜居。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="inlineStr">
+        <is>
+          <t>CHI-20261005-010</t>
+        </is>
+      </c>
+      <c r="B1261" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1261" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1261" t="inlineStr">
+        <is>
+          <t>聚木成林</t>
+        </is>
+      </c>
+      <c r="E1261" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F1261" t="inlineStr">
+        <is>
+          <t>jù mù chéng lín</t>
+        </is>
+      </c>
+      <c r="G1261" t="inlineStr">
+        <is>
+          <t>나무를 모아 숲을 이루다(힘을 합쳐 규모를 키우다)</t>
+        </is>
+      </c>
+      <c r="H1261" t="inlineStr">
+        <is>
+          <t>黑龙江智慧农业聚木成林.</t>
+        </is>
+      </c>
+      <c r="I1261" t="inlineStr">
+        <is>
+          <t>我们通过整合各方资源，真正实现了聚木成林，做大产业规模。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" t="inlineStr">
+        <is>
+          <t>CHI-20261005-011</t>
+        </is>
+      </c>
+      <c r="B1262" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1262" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1262" t="inlineStr">
+        <is>
+          <t>开学</t>
+        </is>
+      </c>
+      <c r="E1262" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1262" t="inlineStr">
+        <is>
+          <t>kāi xué</t>
+        </is>
+      </c>
+      <c r="G1262" t="inlineStr">
+        <is>
+          <t>개학하다</t>
+        </is>
+      </c>
+      <c r="H1262" t="inlineStr">
+        <is>
+          <t>格力技工学校开学，董明珠当校长.</t>
+        </is>
+      </c>
+      <c r="I1262" t="inlineStr">
+        <is>
+          <t>下周一就要开学了，我得赶紧把暑假作业补完。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="inlineStr">
+        <is>
+          <t>CHI-20261005-012</t>
+        </is>
+      </c>
+      <c r="B1263" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1263" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1263" t="inlineStr">
+        <is>
+          <t>欢腾</t>
+        </is>
+      </c>
+      <c r="E1263" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1263" t="inlineStr">
+        <is>
+          <t>huān téng</t>
+        </is>
+      </c>
+      <c r="G1263" t="inlineStr">
+        <is>
+          <t>기쁨으로 떠들썩하다, 환호작약하다</t>
+        </is>
+      </c>
+      <c r="H1263" t="inlineStr">
+        <is>
+          <t>来宁夏，看丰收的欢腾.</t>
+        </is>
+      </c>
+      <c r="I1263" t="inlineStr">
+        <is>
+          <t>运动会上，同学们为胜利欢腾雀跃。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" t="inlineStr">
+        <is>
+          <t>CHI-20261005-013</t>
+        </is>
+      </c>
+      <c r="B1264" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1264" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1264" t="inlineStr">
+        <is>
+          <t>不停歇</t>
+        </is>
+      </c>
+      <c r="E1264" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1264" t="inlineStr">
+        <is>
+          <t>bù tíng xiē</t>
+        </is>
+      </c>
+      <c r="G1264" t="inlineStr">
+        <is>
+          <t>쉬지 않고 계속하다</t>
+        </is>
+      </c>
+      <c r="H1264" t="inlineStr">
+        <is>
+          <t>假期不停歇 奋斗在岗位.</t>
+        </is>
+      </c>
+      <c r="I1264" t="inlineStr">
+        <is>
+          <t>为了赶在截止日期前完成项目，团队成员熬夜不停歇地工作。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="inlineStr">
+        <is>
+          <t>CHI-20261005-014</t>
+        </is>
+      </c>
+      <c r="B1265" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1265" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1265" t="inlineStr">
+        <is>
+          <t>圆满落幕</t>
+        </is>
+      </c>
+      <c r="E1265" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1265" t="inlineStr">
+        <is>
+          <t>yuán mǎn luò mù</t>
+        </is>
+      </c>
+      <c r="G1265" t="inlineStr">
+        <is>
+          <t>성공적으로 막을 내리다</t>
+        </is>
+      </c>
+      <c r="H1265" t="inlineStr">
+        <is>
+          <t>剑河昂英2026年开渔系列活动圆满落幕.</t>
+        </is>
+      </c>
+      <c r="I1265" t="inlineStr">
+        <is>
+          <t>经过三天的激烈角逐，本次艺术节圆满落幕。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" t="inlineStr">
+        <is>
+          <t>CHI-20261005-015</t>
+        </is>
+      </c>
+      <c r="B1266" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1266" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1266" t="inlineStr">
+        <is>
+          <t>平稳有序</t>
+        </is>
+      </c>
+      <c r="E1266" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1266" t="inlineStr">
+        <is>
+          <t>píng wěn yǒu xù</t>
+        </is>
+      </c>
+      <c r="G1266" t="inlineStr">
+        <is>
+          <t>안정적이고 질서 정연하다</t>
+        </is>
+      </c>
+      <c r="H1266" t="inlineStr">
+        <is>
+          <t>国庆假期第五天全国道路交通平稳有序.</t>
+        </is>
+      </c>
+      <c r="I1266" t="inlineStr">
+        <is>
+          <t>在老师的组织下，学生们的撤离过程平稳有序。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" t="inlineStr">
+        <is>
+          <t>CHI-20261005-016</t>
+        </is>
+      </c>
+      <c r="B1267" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1267" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1267" t="inlineStr">
+        <is>
+          <t>点燃</t>
+        </is>
+      </c>
+      <c r="E1267" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1267" t="inlineStr">
+        <is>
+          <t>diǎn rán</t>
+        </is>
+      </c>
+      <c r="G1267" t="inlineStr">
+        <is>
+          <t>불을 붙이다, (열기 등을) 고조시키다</t>
+        </is>
+      </c>
+      <c r="H1267" t="inlineStr">
+        <is>
+          <t>山西柳林后冯家沟文旅活动点燃国庆假期.</t>
+        </is>
+      </c>
+      <c r="I1267" t="inlineStr">
+        <is>
+          <t>这场演唱会点燃了全场观众的热情。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" t="inlineStr">
+        <is>
+          <t>CHI-20261005-017</t>
+        </is>
+      </c>
+      <c r="B1268" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1268" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1268" t="inlineStr">
+        <is>
+          <t>遗落</t>
+        </is>
+      </c>
+      <c r="E1268" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1268" t="inlineStr">
+        <is>
+          <t>yí luò</t>
+        </is>
+      </c>
+      <c r="G1268" t="inlineStr">
+        <is>
+          <t>잊어버리고 떨어뜨리다(분실하다)</t>
+        </is>
+      </c>
+      <c r="H1268" t="inlineStr">
+        <is>
+          <t>女子将装有大量现金的挎包遗落站台.</t>
+        </is>
+      </c>
+      <c r="I1268" t="inlineStr">
+        <is>
+          <t>我不小心把钱包遗落在出租车上了，真着急。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" t="inlineStr">
+        <is>
+          <t>CHI-20261005-018</t>
+        </is>
+      </c>
+      <c r="B1269" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1269" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1269" t="inlineStr">
+        <is>
+          <t>抢票</t>
+        </is>
+      </c>
+      <c r="E1269" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1269" t="inlineStr">
+        <is>
+          <t>qiǎng piào</t>
+        </is>
+      </c>
+      <c r="G1269" t="inlineStr">
+        <is>
+          <t>경쟁하며 표를 예매하다(티켓팅)</t>
+        </is>
+      </c>
+      <c r="H1269" t="inlineStr">
+        <is>
+          <t>警惕这些第三方平台“抢票”常见套路.</t>
+        </is>
+      </c>
+      <c r="I1269" t="inlineStr">
+        <is>
+          <t>春运期间，在网上抢票几乎比中彩票还难。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" t="inlineStr">
+        <is>
+          <t>CHI-20261005-019</t>
+        </is>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1270" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1270" t="inlineStr">
+        <is>
+          <t>溯源</t>
+        </is>
+      </c>
+      <c r="E1270" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1270" t="inlineStr">
+        <is>
+          <t>sù yuán</t>
+        </is>
+      </c>
+      <c r="G1270" t="inlineStr">
+        <is>
+          <t>근원을 거슬러 올라가다(추적하다)</t>
+        </is>
+      </c>
+      <c r="H1270" t="inlineStr">
+        <is>
+          <t>在哈留学生溯源中国优质稻米.</t>
+        </is>
+      </c>
+      <c r="I1270" t="inlineStr">
+        <is>
+          <t>我们需要从源头溯源，找出导致产品质量不稳定的根本原因。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="inlineStr">
+        <is>
+          <t>CHI-20261005-020</t>
+        </is>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1271" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1271" t="inlineStr">
+        <is>
+          <t>感知</t>
+        </is>
+      </c>
+      <c r="E1271" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1271" t="inlineStr">
+        <is>
+          <t>gǎn zhī</t>
+        </is>
+      </c>
+      <c r="G1271" t="inlineStr">
+        <is>
+          <t>체감하다, 느끼다</t>
+        </is>
+      </c>
+      <c r="H1271" t="inlineStr">
+        <is>
+          <t>感知“中国饭碗”背后的...</t>
+        </is>
+      </c>
+      <c r="I1271" t="inlineStr">
+        <is>
+          <t>通过这次实习，我更深刻地感知到了职场的压力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="inlineStr">
+        <is>
+          <t>CHI-20261005-021</t>
+        </is>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1272" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1272" t="inlineStr">
+        <is>
+          <t>激昂</t>
+        </is>
+      </c>
+      <c r="E1272" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1272" t="inlineStr">
+        <is>
+          <t>jī áng</t>
+        </is>
+      </c>
+      <c r="G1272" t="inlineStr">
+        <is>
+          <t>(감정 등이) 격앙된, 열정적인</t>
+        </is>
+      </c>
+      <c r="H1272" t="inlineStr">
+        <is>
+          <t>泰晤士小镇英式街区露天舞台鼓点激昂.</t>
+        </is>
+      </c>
+      <c r="I1272" t="inlineStr">
+        <is>
+          <t>听到那首激昂的国歌，大家都感到心潮澎湃。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="inlineStr">
+        <is>
+          <t>CHI-20261005-022</t>
+        </is>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1273" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1273" t="inlineStr">
+        <is>
+          <t>同台</t>
+        </is>
+      </c>
+      <c r="E1273" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1273" t="inlineStr">
+        <is>
+          <t>tóng tái</t>
+        </is>
+      </c>
+      <c r="G1273" t="inlineStr">
+        <is>
+          <t>같은 무대에 서다</t>
+        </is>
+      </c>
+      <c r="H1273" t="inlineStr">
+        <is>
+          <t>南县地花鼓、舞龙同台献...</t>
+        </is>
+      </c>
+      <c r="I1273" t="inlineStr">
+        <is>
+          <t>能和偶像同台表演，对我来说是最大的荣幸。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="inlineStr">
+        <is>
+          <t>CHI-20261005-023</t>
+        </is>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1274" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1274" t="inlineStr">
+        <is>
+          <t>进境</t>
+        </is>
+      </c>
+      <c r="E1274" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1274" t="inlineStr">
+        <is>
+          <t>jìn jìng</t>
+        </is>
+      </c>
+      <c r="G1274" t="inlineStr">
+        <is>
+          <t>입경하다(국경을 넘어 들어오다)</t>
+        </is>
+      </c>
+      <c r="H1274" t="inlineStr">
+        <is>
+          <t>仅0.55克，进境旅客当场被拦.</t>
+        </is>
+      </c>
+      <c r="I1274" t="inlineStr">
+        <is>
+          <t>旅客在进境时必须如实申报所携带的物品。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="inlineStr">
+        <is>
+          <t>CHI-20261005-024</t>
+        </is>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1275" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1275" t="inlineStr">
+        <is>
+          <t>焕新</t>
+        </is>
+      </c>
+      <c r="E1275" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1275" t="inlineStr">
+        <is>
+          <t>huàn xīn</t>
+        </is>
+      </c>
+      <c r="G1275" t="inlineStr">
+        <is>
+          <t>새롭게 바꾸다(리뉴얼)</t>
+        </is>
+      </c>
+      <c r="H1275" t="inlineStr">
+        <is>
+          <t>大修提质焕新.</t>
+        </is>
+      </c>
+      <c r="I1275" t="inlineStr">
+        <is>
+          <t>这个老品牌正在通过设计焕新吸引年轻消费群体。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="inlineStr">
+        <is>
+          <t>CHI-20261005-025</t>
+        </is>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1276" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1276" t="inlineStr">
+        <is>
+          <t>签到</t>
+        </is>
+      </c>
+      <c r="E1276" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1276" t="inlineStr">
+        <is>
+          <t>qiān dào</t>
+        </is>
+      </c>
+      <c r="G1276" t="inlineStr">
+        <is>
+          <t>출석/입장을 등록하다</t>
+        </is>
+      </c>
+      <c r="H1276" t="inlineStr">
+        <is>
+          <t>参赛选手陆续签到就位.</t>
+        </is>
+      </c>
+      <c r="I1276" t="inlineStr">
+        <is>
+          <t>会议开始前，请大家在门口签到并领取资料。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="inlineStr">
+        <is>
+          <t>CHI-20261005-026</t>
+        </is>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1277" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1277" t="inlineStr">
+        <is>
+          <t>拓宽</t>
+        </is>
+      </c>
+      <c r="E1277" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1277" t="inlineStr">
+        <is>
+          <t>tuò kuān</t>
+        </is>
+      </c>
+      <c r="G1277" t="inlineStr">
+        <is>
+          <t>넓히다(길, 지식, 경로 등)</t>
+        </is>
+      </c>
+      <c r="H1277" t="inlineStr">
+        <is>
+          <t>拓宽乡村致富路.</t>
+        </is>
+      </c>
+      <c r="I1277" t="inlineStr">
+        <is>
+          <t>我们要努力拓宽销售渠道，让产品卖得更远。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="inlineStr">
+        <is>
+          <t>CHI-20261005-027</t>
+        </is>
+      </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1278" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1278" t="inlineStr">
+        <is>
+          <t>贯通</t>
+        </is>
+      </c>
+      <c r="E1278" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1278" t="inlineStr">
+        <is>
+          <t>guàn tōng</t>
+        </is>
+      </c>
+      <c r="G1278" t="inlineStr">
+        <is>
+          <t>(터널, 길 등이) 완전히 뚫리다</t>
+        </is>
+      </c>
+      <c r="H1278" t="inlineStr">
+        <is>
+          <t>天陇铁路“第一长隧”安化隧道顺利贯通.</t>
+        </is>
+      </c>
+      <c r="I1278" t="inlineStr">
+        <is>
+          <t>经过五年的挖掘，这条隧道终于贯通了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="inlineStr">
+        <is>
+          <t>CHI-20261005-028</t>
+        </is>
+      </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C1279" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1279" t="inlineStr">
+        <is>
+          <t>民俗</t>
+        </is>
+      </c>
+      <c r="E1279" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1279" t="inlineStr">
+        <is>
+          <t>mín sú</t>
+        </is>
+      </c>
+      <c r="G1279" t="inlineStr">
+        <is>
+          <t>민속, 전통 풍습</t>
+        </is>
+      </c>
+      <c r="H1279" t="inlineStr">
+        <is>
+          <t>国庆悦享民俗.</t>
+        </is>
+      </c>
+      <c r="I1279" t="inlineStr">
+        <is>
+          <t>这个小镇保留了许多有趣的民俗活动，值得一游。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-10-06 | 1300/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1279"/>
+  <dimension ref="A1:I1301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -60529,6 +60529,1040 @@
         </is>
       </c>
     </row>
+    <row r="1280">
+      <c r="A1280" t="inlineStr">
+        <is>
+          <t>CHI-20261006-001</t>
+        </is>
+      </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1280" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1280" t="inlineStr">
+        <is>
+          <t>报批</t>
+        </is>
+      </c>
+      <c r="E1280" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1280" t="inlineStr">
+        <is>
+          <t>bào pī</t>
+        </is>
+      </c>
+      <c r="G1280" t="inlineStr">
+        <is>
+          <t>상부에 보고하여 허가를 받다(공적 절차)</t>
+        </is>
+      </c>
+      <c r="H1280" t="inlineStr">
+        <is>
+          <t>절차를 거치지 않고 일을 진행하려다 제지당했을 때 사용하는 표현</t>
+        </is>
+      </c>
+      <c r="I1280" t="inlineStr">
+        <is>
+          <t>这个项目没经过报批就私自启动了，肯定会被叫停。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="inlineStr">
+        <is>
+          <t>CHI-20261006-002</t>
+        </is>
+      </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1281" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1281" t="inlineStr">
+        <is>
+          <t>归心似箭</t>
+        </is>
+      </c>
+      <c r="E1281" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1281" t="inlineStr">
+        <is>
+          <t>guī xīn sì jiàn</t>
+        </is>
+      </c>
+      <c r="G1281" t="inlineStr">
+        <is>
+          <t>집으로 돌아가고 싶은 마음이 화살같이 간절하다</t>
+        </is>
+      </c>
+      <c r="H1281" t="inlineStr">
+        <is>
+          <t>명절이나 긴 여행 끝에 빨리 집에 가고 싶어 하는 심정을 나타낼 때</t>
+        </is>
+      </c>
+      <c r="I1281" t="inlineStr">
+        <is>
+          <t>假期快结束了，大家都归心似箭，想赶快回家休息。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="inlineStr">
+        <is>
+          <t>CHI-20261006-003</t>
+        </is>
+      </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1282" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1282" t="inlineStr">
+        <is>
+          <t>闹</t>
+        </is>
+      </c>
+      <c r="E1282" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1282" t="inlineStr">
+        <is>
+          <t>nào</t>
+        </is>
+      </c>
+      <c r="G1282" t="inlineStr">
+        <is>
+          <t>(축제 분위기 등을) 떠들썩하게 만들다, 성대하게 벌이다</t>
+        </is>
+      </c>
+      <c r="H1282" t="inlineStr">
+        <is>
+          <t>행사를 활기차게 운영하거나 축제 분위기를 띄울 때</t>
+        </is>
+      </c>
+      <c r="I1282" t="inlineStr">
+        <is>
+          <t>村里的人聚在一起，热热闹闹地闹元宵。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="inlineStr">
+        <is>
+          <t>CHI-20261006-004</t>
+        </is>
+      </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1283" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1283" t="inlineStr">
+        <is>
+          <t>入心</t>
+        </is>
+      </c>
+      <c r="E1283" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1283" t="inlineStr">
+        <is>
+          <t>rù xīn</t>
+        </is>
+      </c>
+      <c r="G1283" t="inlineStr">
+        <is>
+          <t>마음속 깊이 와닿다, 깊이 새겨지다</t>
+        </is>
+      </c>
+      <c r="H1283" t="inlineStr">
+        <is>
+          <t>감동적인 경험이나 가르침이 뇌리에 깊이 남았을 때</t>
+        </is>
+      </c>
+      <c r="I1283" t="inlineStr">
+        <is>
+          <t>这些传统的文化精神，深深地入心入脑。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="inlineStr">
+        <is>
+          <t>CHI-20261006-005</t>
+        </is>
+      </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1284" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1284" t="inlineStr">
+        <is>
+          <t>出片</t>
+        </is>
+      </c>
+      <c r="E1284" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1284" t="inlineStr">
+        <is>
+          <t>chū piàn</t>
+        </is>
+      </c>
+      <c r="G1284" t="inlineStr">
+        <is>
+          <t>(사진이) 아주 잘 나오다, 인생 사진을 건지다</t>
+        </is>
+      </c>
+      <c r="H1284" t="inlineStr">
+        <is>
+          <t>풍경이 좋아 사진 촬영을 하기에 최적일 때</t>
+        </is>
+      </c>
+      <c r="I1284" t="inlineStr">
+        <is>
+          <t>这里的景色非常美，随手拍都很出片。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="inlineStr">
+        <is>
+          <t>CHI-20261006-006</t>
+        </is>
+      </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1285" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1285" t="inlineStr">
+        <is>
+          <t>凉凉</t>
+        </is>
+      </c>
+      <c r="E1285" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1285" t="inlineStr">
+        <is>
+          <t>liáng liáng</t>
+        </is>
+      </c>
+      <c r="G1285" t="inlineStr">
+        <is>
+          <t>끝장나다, 망하다</t>
+        </is>
+      </c>
+      <c r="H1285" t="inlineStr">
+        <is>
+          <t>인기가 떨어지거나 프로젝트가 실패로 돌아갔을 때의 자조적 표현</t>
+        </is>
+      </c>
+      <c r="I1285" t="inlineStr">
+        <is>
+          <t>再这样无视市场需求，这个产品离凉凉就不远了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="inlineStr">
+        <is>
+          <t>CHI-20261006-007</t>
+        </is>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1286" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1286" t="inlineStr">
+        <is>
+          <t>画饼</t>
+        </is>
+      </c>
+      <c r="E1286" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1286" t="inlineStr">
+        <is>
+          <t>huà bǐng</t>
+        </is>
+      </c>
+      <c r="G1286" t="inlineStr">
+        <is>
+          <t>실현 불가능한 공약을 내세우다(헛된 희망)</t>
+        </is>
+      </c>
+      <c r="H1286" t="inlineStr">
+        <is>
+          <t>상사가 실현 안 될 비전을 제시하며 직원들을 달랠 때</t>
+        </is>
+      </c>
+      <c r="I1286" t="inlineStr">
+        <is>
+          <t>老板只会给员工画饼，从来不落实具体的涨薪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="inlineStr">
+        <is>
+          <t>CHI-20261006-008</t>
+        </is>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1287" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1287" t="inlineStr">
+        <is>
+          <t>耍</t>
+        </is>
+      </c>
+      <c r="E1287" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1287" t="inlineStr">
+        <is>
+          <t>shuǎ</t>
+        </is>
+      </c>
+      <c r="G1287" t="inlineStr">
+        <is>
+          <t>놀다, 시간을 보내다</t>
+        </is>
+      </c>
+      <c r="H1287" t="inlineStr">
+        <is>
+          <t>到成都洛带从早耍到晚。</t>
+        </is>
+      </c>
+      <c r="I1287" t="inlineStr">
+        <is>
+          <t>周末我们一起去公园耍吧，别总待在家里。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="inlineStr">
+        <is>
+          <t>CHI-20261006-009</t>
+        </is>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1288" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1288" t="inlineStr">
+        <is>
+          <t>竞驰</t>
+        </is>
+      </c>
+      <c r="E1288" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1288" t="inlineStr">
+        <is>
+          <t>jìng chí</t>
+        </is>
+      </c>
+      <c r="G1288" t="inlineStr">
+        <is>
+          <t>함께 질주하다, 경쟁하며 달리다</t>
+        </is>
+      </c>
+      <c r="H1288" t="inlineStr">
+        <is>
+          <t>骏马竞驰骋！</t>
+        </is>
+      </c>
+      <c r="I1288" t="inlineStr">
+        <is>
+          <t>赛场上，选手们各显神通，竞驰终点。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="inlineStr">
+        <is>
+          <t>CHI-20261006-010</t>
+        </is>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1289" t="inlineStr">
+        <is>
+          <t>接龙</t>
+        </is>
+      </c>
+      <c r="E1289" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1289" t="inlineStr">
+        <is>
+          <t>jiē lóng</t>
+        </is>
+      </c>
+      <c r="G1289" t="inlineStr">
+        <is>
+          <t>(메신저 등에서) 이어달리기 형식으로 명단 등을 작성하다</t>
+        </is>
+      </c>
+      <c r="H1289" t="inlineStr">
+        <is>
+          <t>说是“自愿”却要实名接龙</t>
+        </is>
+      </c>
+      <c r="I1289" t="inlineStr">
+        <is>
+          <t>团购水果的人，请在群里接龙。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="inlineStr">
+        <is>
+          <t>CHI-20261006-011</t>
+        </is>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1290" t="inlineStr">
+        <is>
+          <t>引客</t>
+        </is>
+      </c>
+      <c r="E1290" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1290" t="inlineStr">
+        <is>
+          <t>yǐn kè</t>
+        </is>
+      </c>
+      <c r="G1290" t="inlineStr">
+        <is>
+          <t>손님을 끌어들이다, 유치하다</t>
+        </is>
+      </c>
+      <c r="H1290" t="inlineStr">
+        <is>
+          <t>乡野风光引客来。</t>
+        </is>
+      </c>
+      <c r="I1290" t="inlineStr">
+        <is>
+          <t>这家餐厅最近推出的新菜品非常引客。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="inlineStr">
+        <is>
+          <t>CHI-20261006-012</t>
+        </is>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1291" t="inlineStr">
+        <is>
+          <t>热议</t>
+        </is>
+      </c>
+      <c r="E1291" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1291" t="inlineStr">
+        <is>
+          <t>rè yì</t>
+        </is>
+      </c>
+      <c r="G1291" t="inlineStr">
+        <is>
+          <t>뜨거운 화젯거리, 열띤 토론</t>
+        </is>
+      </c>
+      <c r="H1291" t="inlineStr">
+        <is>
+          <t>引发热议</t>
+        </is>
+      </c>
+      <c r="I1291" t="inlineStr">
+        <is>
+          <t>这个电影的结局在网上引起了热议。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="inlineStr">
+        <is>
+          <t>CHI-20261006-013</t>
+        </is>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1292" t="inlineStr">
+        <is>
+          <t>顺畅</t>
+        </is>
+      </c>
+      <c r="E1292" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1292" t="inlineStr">
+        <is>
+          <t>shùn chàng</t>
+        </is>
+      </c>
+      <c r="G1292" t="inlineStr">
+        <is>
+          <t>막힘없이 원활하다</t>
+        </is>
+      </c>
+      <c r="H1292" t="inlineStr">
+        <is>
+          <t>未来五年，出行更顺畅。</t>
+        </is>
+      </c>
+      <c r="I1292" t="inlineStr">
+        <is>
+          <t>只要避开早高峰，现在的交通顺畅多了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="inlineStr">
+        <is>
+          <t>CHI-20261006-014</t>
+        </is>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1293" t="inlineStr">
+        <is>
+          <t>热度</t>
+        </is>
+      </c>
+      <c r="E1293" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1293" t="inlineStr">
+        <is>
+          <t>rè dù</t>
+        </is>
+      </c>
+      <c r="G1293" t="inlineStr">
+        <is>
+          <t>관심도, 인기</t>
+        </is>
+      </c>
+      <c r="H1293" t="inlineStr">
+        <is>
+          <t>文旅热度不减</t>
+        </is>
+      </c>
+      <c r="I1293" t="inlineStr">
+        <is>
+          <t>这部电视剧刚播出，热度就非常高。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="inlineStr">
+        <is>
+          <t>CHI-20261006-015</t>
+        </is>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1294" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1294" t="inlineStr">
+        <is>
+          <t>客流</t>
+        </is>
+      </c>
+      <c r="E1294" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1294" t="inlineStr">
+        <is>
+          <t>kè liú</t>
+        </is>
+      </c>
+      <c r="G1294" t="inlineStr">
+        <is>
+          <t>승객 흐름, 이용객 수</t>
+        </is>
+      </c>
+      <c r="H1294" t="inlineStr">
+        <is>
+          <t>武汉铁路迎来假期客流高峰</t>
+        </is>
+      </c>
+      <c r="I1294" t="inlineStr">
+        <is>
+          <t>国庆期间火车站的客流非常大。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="inlineStr">
+        <is>
+          <t>CHI-20261006-016</t>
+        </is>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1295" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1295" t="inlineStr">
+        <is>
+          <t>讲方</t>
+        </is>
+      </c>
+      <c r="E1295" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1295" t="inlineStr">
+        <is>
+          <t>jiǎng fāng</t>
+        </is>
+      </c>
+      <c r="G1295" t="inlineStr">
+        <is>
+          <t>방법을 잘 따지다, 요령을 알다</t>
+        </is>
+      </c>
+      <c r="H1295" t="inlineStr">
+        <is>
+          <t>号召捐款得讲方</t>
+        </is>
+      </c>
+      <c r="I1295" t="inlineStr">
+        <is>
+          <t>办事要讲方，不然只会事倍功半。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="inlineStr">
+        <is>
+          <t>CHI-20261006-017</t>
+        </is>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1296" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1296" t="inlineStr">
+        <is>
+          <t>立项</t>
+        </is>
+      </c>
+      <c r="E1296" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1296" t="inlineStr">
+        <is>
+          <t>lì xiàng</t>
+        </is>
+      </c>
+      <c r="G1296" t="inlineStr">
+        <is>
+          <t>프로젝트를 승인하다, 사업을 시작하다</t>
+        </is>
+      </c>
+      <c r="H1296" t="inlineStr">
+        <is>
+          <t>山东拟立法</t>
+        </is>
+      </c>
+      <c r="I1296" t="inlineStr">
+        <is>
+          <t>这个科研项目已经正式立项了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="inlineStr">
+        <is>
+          <t>CHI-20261006-018</t>
+        </is>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1297" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1297" t="inlineStr">
+        <is>
+          <t>露天</t>
+        </is>
+      </c>
+      <c r="E1297" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1297" t="inlineStr">
+        <is>
+          <t>lòu tiān</t>
+        </is>
+      </c>
+      <c r="G1297" t="inlineStr">
+        <is>
+          <t>야외의, 지붕이 없는</t>
+        </is>
+      </c>
+      <c r="H1297" t="inlineStr">
+        <is>
+          <t>英式街区露天舞台</t>
+        </is>
+      </c>
+      <c r="I1297" t="inlineStr">
+        <is>
+          <t>晚上我们在露天咖啡馆喝茶聊天。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr">
+        <is>
+          <t>CHI-20261006-019</t>
+        </is>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1298" t="inlineStr">
+        <is>
+          <t>守护</t>
+        </is>
+      </c>
+      <c r="E1298" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1298" t="inlineStr">
+        <is>
+          <t>shǒu hù</t>
+        </is>
+      </c>
+      <c r="G1298" t="inlineStr">
+        <is>
+          <t>지키다, 수호하다</t>
+        </is>
+      </c>
+      <c r="H1298" t="inlineStr">
+        <is>
+          <t>旅途之中的守护身影</t>
+        </is>
+      </c>
+      <c r="I1298" t="inlineStr">
+        <is>
+          <t>感谢医护人员在疫情期间对我们的守护。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr">
+        <is>
+          <t>CHI-20261006-020</t>
+        </is>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1299" t="inlineStr">
+        <is>
+          <t>快报</t>
+        </is>
+      </c>
+      <c r="E1299" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1299" t="inlineStr">
+        <is>
+          <t>kuài bào</t>
+        </is>
+      </c>
+      <c r="G1299" t="inlineStr">
+        <is>
+          <t>속보, 요약 보고</t>
+        </is>
+      </c>
+      <c r="H1299" t="inlineStr">
+        <is>
+          <t>国庆文旅快报</t>
+        </is>
+      </c>
+      <c r="I1299" t="inlineStr">
+        <is>
+          <t>请看最新的股市快报。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>CHI-20261006-021</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1300" t="inlineStr">
+        <is>
+          <t>返程</t>
+        </is>
+      </c>
+      <c r="E1300" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1300" t="inlineStr">
+        <is>
+          <t>fǎn chéng</t>
+        </is>
+      </c>
+      <c r="G1300" t="inlineStr">
+        <is>
+          <t>귀경하다, 돌아오는 길에 오르다</t>
+        </is>
+      </c>
+      <c r="H1300" t="inlineStr">
+        <is>
+          <t>铁路迎来返程客流高峰</t>
+        </is>
+      </c>
+      <c r="I1300" t="inlineStr">
+        <is>
+          <t>假期快结束了，今天开始返程。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="inlineStr">
+        <is>
+          <t>CHI-20261006-022</t>
+        </is>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C1301" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1301" t="inlineStr">
+        <is>
+          <t>就位</t>
+        </is>
+      </c>
+      <c r="E1301" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1301" t="inlineStr">
+        <is>
+          <t>jiù wèi</t>
+        </is>
+      </c>
+      <c r="G1301" t="inlineStr">
+        <is>
+          <t>제자리에 앉다, 자리를 잡다</t>
+        </is>
+      </c>
+      <c r="H1301" t="inlineStr">
+        <is>
+          <t>参赛选手陆续签到就位</t>
+        </is>
+      </c>
+      <c r="I1301" t="inlineStr">
+        <is>
+          <t>全员就位，演出马上就要开始了。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-10-08 | 1304/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1301"/>
+  <dimension ref="A1:I1305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61563,6 +61563,194 @@
         </is>
       </c>
     </row>
+    <row r="1302">
+      <c r="A1302" t="inlineStr">
+        <is>
+          <t>CHI-20261008-001</t>
+        </is>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="C1302" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1302" t="inlineStr">
+        <is>
+          <t>假期余额</t>
+        </is>
+      </c>
+      <c r="E1302" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1302" t="inlineStr">
+        <is>
+          <t>jià qī yú é</t>
+        </is>
+      </c>
+      <c r="G1302" t="inlineStr">
+        <is>
+          <t>남은 연휴 기간</t>
+        </is>
+      </c>
+      <c r="H1302" t="inlineStr">
+        <is>
+          <t>국경절 연휴가 끝나가면서 많은 사람들이 '남은 휴일이 며칠 없다'며 아쉬워하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="I1302" t="inlineStr">
+        <is>
+          <t>假期余额已不足，大家得赶紧调整作息准备上班了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="inlineStr">
+        <is>
+          <t>CHI-20261008-002</t>
+        </is>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="C1303" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1303" t="inlineStr">
+        <is>
+          <t>雷厉风行</t>
+        </is>
+      </c>
+      <c r="E1303" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1303" t="inlineStr">
+        <is>
+          <t>léi lì fēng xíng</t>
+        </is>
+      </c>
+      <c r="G1303" t="inlineStr">
+        <is>
+          <t>전광석화처럼 신속하게 일을 처리하다</t>
+        </is>
+      </c>
+      <c r="H1303" t="inlineStr">
+        <is>
+          <t>창구 직원이 막힘없이 신속하게 행정 처리를 완료하여 단 5분 만에 일을 끝낼 수 있었습니다.</t>
+        </is>
+      </c>
+      <c r="I1303" t="inlineStr">
+        <is>
+          <t>新上任的经理做事雷厉风行，很快就解决了堆积已久的问题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="inlineStr">
+        <is>
+          <t>CHI-20261008-003</t>
+        </is>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="C1304" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1304" t="inlineStr">
+        <is>
+          <t>从娃娃抓起</t>
+        </is>
+      </c>
+      <c r="E1304" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1304" t="inlineStr">
+        <is>
+          <t>cóng wáwa zhuā qǐ</t>
+        </is>
+      </c>
+      <c r="G1304" t="inlineStr">
+        <is>
+          <t>어릴 때부터 철저히 가르치고 준비하다 (조기 교육/기초 육성)</t>
+        </is>
+      </c>
+      <c r="H1304" t="inlineStr">
+        <is>
+          <t>“三大球”等体育教育需要从娃娃抓起，全面提升学生体质。</t>
+        </is>
+      </c>
+      <c r="I1304" t="inlineStr">
+        <is>
+          <t>语言学习要从娃娃抓起，这时候孩子的模仿能力和记忆力最强。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="inlineStr">
+        <is>
+          <t>CHI-20261008-004</t>
+        </is>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="C1305" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1305" t="inlineStr">
+        <is>
+          <t>有备无患</t>
+        </is>
+      </c>
+      <c r="E1305" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F1305" t="inlineStr">
+        <is>
+          <t>yǒu bèi wú huàn</t>
+        </is>
+      </c>
+      <c r="G1305" t="inlineStr">
+        <is>
+          <t>유비무환 (준비가 있으면 걱정이 없다)</t>
+        </is>
+      </c>
+      <c r="H1305" t="inlineStr">
+        <is>
+          <t>面对国庆返程高峰，各交通部门提前做好了客流应急方案，有备无患。</t>
+        </is>
+      </c>
+      <c r="I1305" t="inlineStr">
+        <is>
+          <t>出门旅行前，在包里多带点常用药，有备无患总是好的。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-10-09 | 1317/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1305"/>
+  <dimension ref="A1:I1318"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61751,6 +61751,617 @@
         </is>
       </c>
     </row>
+    <row r="1306">
+      <c r="A1306" t="inlineStr">
+        <is>
+          <t>CHI-20261009-001</t>
+        </is>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C1306" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1306" t="inlineStr">
+        <is>
+          <t>松弛感</t>
+        </is>
+      </c>
+      <c r="E1306" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1306" t="inlineStr">
+        <is>
+          <t>sōng chí gǎn</t>
+        </is>
+      </c>
+      <c r="G1306" t="inlineStr">
+        <is>
+          <t>어떤 상황에서도 초조해하지 않고 여유를 잃지 않는 태도나 멘탈</t>
+        </is>
+      </c>
+      <c r="H1306" t="inlineStr">
+        <is>
+          <t>在这么重大的庆功宴上，他还能表现得这么淡定，松弛感简直拉满了。</t>
+        </is>
+      </c>
+      <c r="I1306" t="inlineStr">
+        <is>
+          <t>面试时别太紧绷，适当展现出一些松弛感反而更容易给考官留下好印象。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="inlineStr">
+        <is>
+          <t>CHI-20261009-002</t>
+        </is>
+      </c>
+      <c r="B1307" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C1307" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1307" t="inlineStr">
+        <is>
+          <t>探店</t>
+        </is>
+      </c>
+      <c r="E1307" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1307" t="inlineStr">
+        <is>
+          <t>tàn diàn</t>
+        </is>
+      </c>
+      <c r="G1307" t="inlineStr">
+        <is>
+          <t>(SNS에서 핫한) 맛집이나 명소를 직접 방문해 체험하다</t>
+        </is>
+      </c>
+      <c r="H1307" t="inlineStr">
+        <is>
+          <t>现在不少人挑选餐厅前，都喜欢先刷一刷网红探店视频来当参考。</t>
+        </is>
+      </c>
+      <c r="I1307" t="inlineStr">
+        <is>
+          <t>周末要是没事，我们一起去新开的那家创意咖啡馆探店吧。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="inlineStr">
+        <is>
+          <t>CHI-20261009-003</t>
+        </is>
+      </c>
+      <c r="B1308" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C1308" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1308" t="inlineStr">
+        <is>
+          <t>动心</t>
+        </is>
+      </c>
+      <c r="E1308" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1308" t="inlineStr">
+        <is>
+          <t>dòng xīn</t>
+        </is>
+      </c>
+      <c r="G1308" t="inlineStr">
+        <is>
+          <t>마음이 혹하다, 솔깃해지다</t>
+        </is>
+      </c>
+      <c r="H1308" t="inlineStr">
+        <is>
+          <t>博主镜头里那些价格诱人的高端海鲜套餐，换作是谁都难免会动心。</t>
+        </is>
+      </c>
+      <c r="I1308" t="inlineStr">
+        <is>
+          <t>虽然对方开出的薪资条件让我很动心，但综合考虑通勤成本后我还是拒绝了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="inlineStr">
+        <is>
+          <t>CHI-20261009-004</t>
+        </is>
+      </c>
+      <c r="B1309" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C1309" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1309" t="inlineStr">
+        <is>
+          <t>张冠李戴</t>
+        </is>
+      </c>
+      <c r="E1309" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1309" t="inlineStr">
+        <is>
+          <t>zhāng guān lǐ dài</t>
+        </is>
+      </c>
+      <c r="G1309" t="inlineStr">
+        <is>
+          <t>엉뚱한 대상을 잘못 연결해 혼동하거나 속이다</t>
+        </is>
+      </c>
+      <c r="H1309" t="inlineStr">
+        <is>
+          <t>有些商家抓住外行人难分辨的空子，玩起食材张冠李戴的把戏，说好的帝王蟹却端上了廉价蟹。</t>
+        </is>
+      </c>
+      <c r="I1309" t="inlineStr">
+        <is>
+          <t>做数据汇报一定要核对清楚，千万别张冠李戴，把两家客户的预算搞混了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="inlineStr">
+        <is>
+          <t>CHI-20261009-005</t>
+        </is>
+      </c>
+      <c r="B1310" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C1310" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1310" t="inlineStr">
+        <is>
+          <t>门道</t>
+        </is>
+      </c>
+      <c r="E1310" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1310" t="inlineStr">
+        <is>
+          <t>mén dao</t>
+        </is>
+      </c>
+      <c r="G1310" t="inlineStr">
+        <is>
+          <t>(특정 분야의) 요령, 비결, 내막</t>
+        </is>
+      </c>
+      <c r="H1310" t="inlineStr">
+        <is>
+          <t>看似普通的海鲜采购，外行人看热闹，懂行的人才知道里面的门道有多深。</t>
+        </is>
+      </c>
+      <c r="I1310" t="inlineStr">
+        <is>
+          <t>跟这种老资格的客户谈合作，你必须摸清其中的门道，不然很容易吃亏。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="inlineStr">
+        <is>
+          <t>CHI-20261009-006</t>
+        </is>
+      </c>
+      <c r="B1311" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C1311" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1311" t="inlineStr">
+        <is>
+          <t>较真</t>
+        </is>
+      </c>
+      <c r="E1311" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1311" t="inlineStr">
+        <is>
+          <t>jiào zhēn</t>
+        </is>
+      </c>
+      <c r="G1311" t="inlineStr">
+        <is>
+          <t>지나치게 따지다, 융통성 없이 꼬치꼬치 캐묻다</t>
+        </is>
+      </c>
+      <c r="H1311" t="inlineStr">
+        <is>
+          <t>邻里之间如果凡事都太较真，一点动静就闹得不可开交，日子就会过得很累。</t>
+        </is>
+      </c>
+      <c r="I1311" t="inlineStr">
+        <is>
+          <t>大家只是在开玩笑而已，你何必这么较真，弄得场面这么尴尬呢？</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="inlineStr">
+        <is>
+          <t>CHI-20261009-007</t>
+        </is>
+      </c>
+      <c r="B1312" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C1312" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1312" t="inlineStr">
+        <is>
+          <t>补觉</t>
+        </is>
+      </c>
+      <c r="E1312" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1312" t="inlineStr">
+        <is>
+          <t>bǔ jiào</t>
+        </is>
+      </c>
+      <c r="G1312" t="inlineStr">
+        <is>
+          <t>부족했던 잠을 몰아서 보충하다</t>
+        </is>
+      </c>
+      <c r="H1312" t="inlineStr">
+        <is>
+          <t>隔壁一直吵闹到后半夜，搞得我第二天根本没办法正常工作，周末必须好好补觉。</t>
+        </is>
+      </c>
+      <c r="I1312" t="inlineStr">
+        <is>
+          <t>连续熬夜加班赶方案，今天一整天我什么都不想干，只想躺平补觉。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="inlineStr">
+        <is>
+          <t>CHI-20261009-008</t>
+        </is>
+      </c>
+      <c r="B1313" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C1313" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1313" t="inlineStr">
+        <is>
+          <t>吃得消</t>
+        </is>
+      </c>
+      <c r="E1313" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1313" t="inlineStr">
+        <is>
+          <t>chī de xiāo</t>
+        </is>
+      </c>
+      <c r="G1313" t="inlineStr">
+        <is>
+          <t>(육체적, 정신적 부담을) 견뎌내다, 감당하다</t>
+        </is>
+      </c>
+      <c r="H1313" t="inlineStr">
+        <is>
+          <t>每天从早忙到晚还要应对各种突发投诉，身体和精神真有点吃不消了。</t>
+        </is>
+      </c>
+      <c r="I1313" t="inlineStr">
+        <is>
+          <t>这么高强度的出差频率，就算年轻人底子好，长期下来也未必吃得消。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="inlineStr">
+        <is>
+          <t>CHI-20261009-009</t>
+        </is>
+      </c>
+      <c r="B1314" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C1314" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1314" t="inlineStr">
+        <is>
+          <t>敷衍</t>
+        </is>
+      </c>
+      <c r="E1314" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1314" t="inlineStr">
+        <is>
+          <t>fū yan</t>
+        </is>
+      </c>
+      <c r="G1314" t="inlineStr">
+        <is>
+          <t>대충 일 처리하다, 얼렁뚱땅 넘어가다</t>
+        </is>
+      </c>
+      <c r="H1314" t="inlineStr">
+        <is>
+          <t>教辅打印到底是学校还是家长的事？可不能敷衍了事，得先把‘打印边界’理清楚。</t>
+        </is>
+      </c>
+      <c r="I1314" t="inlineStr">
+        <is>
+          <t>工作态度不能这么敷衍，出了问题谁来负责？</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="inlineStr">
+        <is>
+          <t>CHI-20261009-010</t>
+        </is>
+      </c>
+      <c r="B1315" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C1315" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1315" t="inlineStr">
+        <is>
+          <t>做东</t>
+        </is>
+      </c>
+      <c r="E1315" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1315" t="inlineStr">
+        <is>
+          <t>zuò dōng</t>
+        </is>
+      </c>
+      <c r="G1315" t="inlineStr">
+        <is>
+          <t>한턱내다, 대접하다</t>
+        </is>
+      </c>
+      <c r="H1315" t="inlineStr">
+        <is>
+          <t>今天项目顺利通过了，晚上我做东，请大家去吃帝王蟹套餐。</t>
+        </is>
+      </c>
+      <c r="I1315" t="inlineStr">
+        <is>
+          <t>难得你来北京，今天中午必须由我来做东。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" t="inlineStr">
+        <is>
+          <t>CHI-20261009-011</t>
+        </is>
+      </c>
+      <c r="B1316" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C1316" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1316" t="inlineStr">
+        <is>
+          <t>不以为然</t>
+        </is>
+      </c>
+      <c r="E1316" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1316" t="inlineStr">
+        <is>
+          <t>bù yǐ wéi rán</t>
+        </is>
+      </c>
+      <c r="G1316" t="inlineStr">
+        <is>
+          <t>그렇게 생각하지 않다, 대수롭지 않게 여기다</t>
+        </is>
+      </c>
+      <c r="H1316" t="inlineStr">
+        <is>
+          <t>起初，家长对合并办学的决定不以为然，觉得只是挂了个名牌。</t>
+        </is>
+      </c>
+      <c r="I1316" t="inlineStr">
+        <is>
+          <t>大家都觉得这个问题很严重，他却不以为然。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="inlineStr">
+        <is>
+          <t>CHI-20261009-012</t>
+        </is>
+      </c>
+      <c r="B1317" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C1317" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1317" t="inlineStr">
+        <is>
+          <t>兜风</t>
+        </is>
+      </c>
+      <c r="E1317" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1317" t="inlineStr">
+        <is>
+          <t>dōu fēng</t>
+        </is>
+      </c>
+      <c r="G1317" t="inlineStr">
+        <is>
+          <t>드라이브하다, 바람을 쐬다</t>
+        </is>
+      </c>
+      <c r="H1317" t="inlineStr">
+        <is>
+          <t>国庆假期，他开着私家车带着家人去郊外兜风。</t>
+        </is>
+      </c>
+      <c r="I1317" t="inlineStr">
+        <is>
+          <t>周末天气这么好，我们开车去海边兜风吧。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" t="inlineStr">
+        <is>
+          <t>CHI-20261009-013</t>
+        </is>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C1318" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1318" t="inlineStr">
+        <is>
+          <t>留面子</t>
+        </is>
+      </c>
+      <c r="E1318" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1318" t="inlineStr">
+        <is>
+          <t>liú miàn zi</t>
+        </is>
+      </c>
+      <c r="G1318" t="inlineStr">
+        <is>
+          <t>체면을 세워주다, 낯을 세워주다</t>
+        </is>
+      </c>
+      <c r="H1318" t="inlineStr">
+        <is>
+          <t>就算下属工作出了差错，领导在公开场合也应该给他们留面子。</t>
+        </is>
+      </c>
+      <c r="I1318" t="inlineStr">
+        <is>
+          <t>我知道是我错了，但你在外人面前好歹给我留点面子吧。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-10-12 | 1320/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1318"/>
+  <dimension ref="A1:I1321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -62362,6 +62362,147 @@
         </is>
       </c>
     </row>
+    <row r="1319">
+      <c r="A1319" t="inlineStr">
+        <is>
+          <t>CHI-20261012-001</t>
+        </is>
+      </c>
+      <c r="B1319" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C1319" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1319" t="inlineStr">
+        <is>
+          <t>迎刃而解</t>
+        </is>
+      </c>
+      <c r="E1319" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1319" t="inlineStr">
+        <is>
+          <t>yíng rèn ér jiě</t>
+        </is>
+      </c>
+      <c r="G1319" t="inlineStr">
+        <is>
+          <t>문제가 술술 풀리다, 쉽게 해결되다</t>
+        </is>
+      </c>
+      <c r="H1319" t="inlineStr">
+        <is>
+          <t>只要把核心技术突破了，后续的生产难题就会迎刃而解。</t>
+        </is>
+      </c>
+      <c r="I1319" t="inlineStr">
+        <is>
+          <t>理清了沟通流程后，部门之间原本复杂的协作矛盾迎刃而解。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" t="inlineStr">
+        <is>
+          <t>CHI-20261012-002</t>
+        </is>
+      </c>
+      <c r="B1320" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C1320" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1320" t="inlineStr">
+        <is>
+          <t>打破僵局</t>
+        </is>
+      </c>
+      <c r="E1320" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1320" t="inlineStr">
+        <is>
+          <t>dǎ pò jiāng jú</t>
+        </is>
+      </c>
+      <c r="G1320" t="inlineStr">
+        <is>
+          <t>교착 상태를 타개하다, 막힌 국면을 풀다</t>
+        </is>
+      </c>
+      <c r="H1320" t="inlineStr">
+        <is>
+          <t>双方谈判陷入停滞，需要提出一个折中方案来打破僵局。</t>
+        </is>
+      </c>
+      <c r="I1320" t="inlineStr">
+        <is>
+          <t>他在会议上的幽默发言瞬间缓和了气氛，打破了原有的僵局。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="inlineStr">
+        <is>
+          <t>CHI-20261012-003</t>
+        </is>
+      </c>
+      <c r="B1321" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C1321" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1321" t="inlineStr">
+        <is>
+          <t>讨价还价</t>
+        </is>
+      </c>
+      <c r="E1321" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1321" t="inlineStr">
+        <is>
+          <t>tǎo jià huán jià</t>
+        </is>
+      </c>
+      <c r="G1321" t="inlineStr">
+        <is>
+          <t>흥정하다, 조건을 두고 왈가왈부하다</t>
+        </is>
+      </c>
+      <c r="H1321" t="inlineStr">
+        <is>
+          <t>安全红线是原则问题，没有任何讨价还价的余地。</t>
+        </is>
+      </c>
+      <c r="I1321" t="inlineStr">
+        <is>
+          <t>采购部正就设备保养周期的补充条款和厂家进行讨价还价。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-10-13 | 1333/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1321"/>
+  <dimension ref="A1:I1334"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -62503,6 +62503,617 @@
         </is>
       </c>
     </row>
+    <row r="1322">
+      <c r="A1322" t="inlineStr">
+        <is>
+          <t>CHI-20261013-001</t>
+        </is>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C1322" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1322" t="inlineStr">
+        <is>
+          <t>洗白</t>
+        </is>
+      </c>
+      <c r="E1322" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1322" t="inlineStr">
+        <is>
+          <t>xǐ bái</t>
+        </is>
+      </c>
+      <c r="G1322" t="inlineStr">
+        <is>
+          <t>이미지를 세탁하다, 오명을 벗다</t>
+        </is>
+      </c>
+      <c r="H1322" t="inlineStr">
+        <is>
+          <t>기업이나 개인이 부정적인 여론을 돌리기 위해 긍정적인 홍보를 하는 상황</t>
+        </is>
+      </c>
+      <c r="I1322" t="inlineStr">
+        <is>
+          <t>出了这么大的公关危机，想靠发几条微博就洗白是不可能的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="inlineStr">
+        <is>
+          <t>CHI-20261013-002</t>
+        </is>
+      </c>
+      <c r="B1323" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C1323" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1323" t="inlineStr">
+        <is>
+          <t>起劲</t>
+        </is>
+      </c>
+      <c r="E1323" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1323" t="inlineStr">
+        <is>
+          <t>qǐ jìn</t>
+        </is>
+      </c>
+      <c r="G1323" t="inlineStr">
+        <is>
+          <t>신나다, 열의를 보이다</t>
+        </is>
+      </c>
+      <c r="H1323" t="inlineStr">
+        <is>
+          <t>어떤 일에 흥미를 느끼고 열심히 달려들 때</t>
+        </is>
+      </c>
+      <c r="I1323" t="inlineStr">
+        <is>
+          <t>大家谈起未来的职业规划时，都特别起劲。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="inlineStr">
+        <is>
+          <t>CHI-20261013-003</t>
+        </is>
+      </c>
+      <c r="B1324" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C1324" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1324" t="inlineStr">
+        <is>
+          <t>没准</t>
+        </is>
+      </c>
+      <c r="E1324" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1324" t="inlineStr">
+        <is>
+          <t>méi zhǔn</t>
+        </is>
+      </c>
+      <c r="G1324" t="inlineStr">
+        <is>
+          <t>어쩌면, 확실치 않다, 그럴지도 모른다</t>
+        </is>
+      </c>
+      <c r="H1324" t="inlineStr">
+        <is>
+          <t>어떤 결과가 나올지 불확실함을 나타낼 때</t>
+        </is>
+      </c>
+      <c r="I1324" t="inlineStr">
+        <is>
+          <t>没准他今天加班，我们还是先别去打扰他了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="inlineStr">
+        <is>
+          <t>CHI-20261013-004</t>
+        </is>
+      </c>
+      <c r="B1325" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C1325" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1325" t="inlineStr">
+        <is>
+          <t>给面子</t>
+        </is>
+      </c>
+      <c r="E1325" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1325" t="inlineStr">
+        <is>
+          <t>gěi miàn zi</t>
+        </is>
+      </c>
+      <c r="G1325" t="inlineStr">
+        <is>
+          <t>체면을 세워주다, 기분을 맞춰주다</t>
+        </is>
+      </c>
+      <c r="H1325" t="inlineStr">
+        <is>
+          <t>상대방의 입장을 고려해 요청을 들어주거나 친절하게 대할 때</t>
+        </is>
+      </c>
+      <c r="I1325" t="inlineStr">
+        <is>
+          <t>他今天特意推掉会议来参加聚会，真的很给面子。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="inlineStr">
+        <is>
+          <t>CHI-20261013-005</t>
+        </is>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C1326" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1326" t="inlineStr">
+        <is>
+          <t>没辙</t>
+        </is>
+      </c>
+      <c r="E1326" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1326" t="inlineStr">
+        <is>
+          <t>méi zhé</t>
+        </is>
+      </c>
+      <c r="G1326" t="inlineStr">
+        <is>
+          <t>방법이 없다, 속수무책이다</t>
+        </is>
+      </c>
+      <c r="H1326" t="inlineStr">
+        <is>
+          <t>상황이 해결되지 않아 어쩔 도리가 없을 때</t>
+        </is>
+      </c>
+      <c r="I1326" t="inlineStr">
+        <is>
+          <t>客户坚持要退货，我也没辙，只能按规定处理。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="inlineStr">
+        <is>
+          <t>CHI-20261013-006</t>
+        </is>
+      </c>
+      <c r="B1327" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C1327" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1327" t="inlineStr">
+        <is>
+          <t>说曹操曹操到</t>
+        </is>
+      </c>
+      <c r="E1327" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1327" t="inlineStr">
+        <is>
+          <t>shuō cáo cāo cáo cāo dào</t>
+        </is>
+      </c>
+      <c r="G1327" t="inlineStr">
+        <is>
+          <t>호랑이도 제 말 하면 온다</t>
+        </is>
+      </c>
+      <c r="H1327" t="inlineStr">
+        <is>
+          <t>이야기하던 사람이 마침 그 자리에 나타났을 때</t>
+        </is>
+      </c>
+      <c r="I1327" t="inlineStr">
+        <is>
+          <t>我们正谈论你呢，说曹操曹操到，你这就来了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" t="inlineStr">
+        <is>
+          <t>CHI-20261013-007</t>
+        </is>
+      </c>
+      <c r="B1328" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C1328" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1328" t="inlineStr">
+        <is>
+          <t>有门儿</t>
+        </is>
+      </c>
+      <c r="E1328" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1328" t="inlineStr">
+        <is>
+          <t>yǒu mén r</t>
+        </is>
+      </c>
+      <c r="G1328" t="inlineStr">
+        <is>
+          <t>가망이 있다, 길이 보이다</t>
+        </is>
+      </c>
+      <c r="H1328" t="inlineStr">
+        <is>
+          <t>어려운 일에 실마리가 풀릴 기미가 보일 때</t>
+        </is>
+      </c>
+      <c r="I1328" t="inlineStr">
+        <is>
+          <t>刚才和客户聊得不错，看来这个合作项目有门儿。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" t="inlineStr">
+        <is>
+          <t>CHI-20261013-008</t>
+        </is>
+      </c>
+      <c r="B1329" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C1329" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1329" t="inlineStr">
+        <is>
+          <t>不松懈</t>
+        </is>
+      </c>
+      <c r="E1329" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1329" t="inlineStr">
+        <is>
+          <t>bù sōng xiè</t>
+        </is>
+      </c>
+      <c r="G1329" t="inlineStr">
+        <is>
+          <t>긴장을 늦추지 않다, 방심하지 않다</t>
+        </is>
+      </c>
+      <c r="H1329" t="inlineStr">
+        <is>
+          <t>国庆在岗不松懈，全力守护城市市容秩序</t>
+        </is>
+      </c>
+      <c r="I1329" t="inlineStr">
+        <is>
+          <t>临近考试，大家复习的状态一点也不松懈。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" t="inlineStr">
+        <is>
+          <t>CHI-20261013-009</t>
+        </is>
+      </c>
+      <c r="B1330" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C1330" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1330" t="inlineStr">
+        <is>
+          <t>重头戏</t>
+        </is>
+      </c>
+      <c r="E1330" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1330" t="inlineStr">
+        <is>
+          <t>zhòng tóu xì</t>
+        </is>
+      </c>
+      <c r="G1330" t="inlineStr">
+        <is>
+          <t>가장 중요한 부분, 하이라이트</t>
+        </is>
+      </c>
+      <c r="H1330" t="inlineStr">
+        <is>
+          <t>洞见｜对话童彬原：对标国际健康建筑标准，国潮7...</t>
+        </is>
+      </c>
+      <c r="I1330" t="inlineStr">
+        <is>
+          <t>本次发布会的重头戏是新款人工智能产品的演示。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" t="inlineStr">
+        <is>
+          <t>CHI-20261013-010</t>
+        </is>
+      </c>
+      <c r="B1331" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C1331" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1331" t="inlineStr">
+        <is>
+          <t>跟不上</t>
+        </is>
+      </c>
+      <c r="E1331" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1331" t="inlineStr">
+        <is>
+          <t>gēn bu shàng</t>
+        </is>
+      </c>
+      <c r="G1331" t="inlineStr">
+        <is>
+          <t>따라가지 못하다, 뒤처지다</t>
+        </is>
+      </c>
+      <c r="H1331" t="inlineStr">
+        <is>
+          <t>人社部：破解结构性就业矛盾</t>
+        </is>
+      </c>
+      <c r="I1331" t="inlineStr">
+        <is>
+          <t>现在的技术更新太快，老员工怕跟不上时代。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" t="inlineStr">
+        <is>
+          <t>CHI-20261013-011</t>
+        </is>
+      </c>
+      <c r="B1332" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C1332" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1332" t="inlineStr">
+        <is>
+          <t>不折腾</t>
+        </is>
+      </c>
+      <c r="E1332" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1332" t="inlineStr">
+        <is>
+          <t>bù zhē teng</t>
+        </is>
+      </c>
+      <c r="G1332" t="inlineStr">
+        <is>
+          <t>괜히 고생하지 않다, 문제를 일으키지 않다</t>
+        </is>
+      </c>
+      <c r="H1332" t="inlineStr">
+        <is>
+          <t>面对繁琐的换届手续，大家希望过程能精简、不折腾。</t>
+        </is>
+      </c>
+      <c r="I1332" t="inlineStr">
+        <is>
+          <t>我们还是走直达航班吧，为了省钱转机太折腾了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" t="inlineStr">
+        <is>
+          <t>CHI-20261013-012</t>
+        </is>
+      </c>
+      <c r="B1333" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C1333" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1333" t="inlineStr">
+        <is>
+          <t>大实话</t>
+        </is>
+      </c>
+      <c r="E1333" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1333" t="inlineStr">
+        <is>
+          <t>dà shí huà</t>
+        </is>
+      </c>
+      <c r="G1333" t="inlineStr">
+        <is>
+          <t>솔직한 말, 팩트 폭격</t>
+        </is>
+      </c>
+      <c r="H1333" t="inlineStr">
+        <is>
+          <t>听了专家的建议，大家都觉得这是大实话。</t>
+        </is>
+      </c>
+      <c r="I1333" t="inlineStr">
+        <is>
+          <t>他虽然说话直，但说的都是大实话。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" t="inlineStr">
+        <is>
+          <t>CHI-20261013-013</t>
+        </is>
+      </c>
+      <c r="B1334" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C1334" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1334" t="inlineStr">
+        <is>
+          <t>有失偏颇</t>
+        </is>
+      </c>
+      <c r="E1334" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1334" t="inlineStr">
+        <is>
+          <t>yǒu shī piān pō</t>
+        </is>
+      </c>
+      <c r="G1334" t="inlineStr">
+        <is>
+          <t>치우치다, 공정하지 못하다</t>
+        </is>
+      </c>
+      <c r="H1334" t="inlineStr">
+        <is>
+          <t>对单一指标评价就业市场容易有失偏颇。</t>
+        </is>
+      </c>
+      <c r="I1334" t="inlineStr">
+        <is>
+          <t>只看分数来评价一个学生的发展潜力，显然有失偏颇。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-10-15 | 1342/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1334"/>
+  <dimension ref="A1:I1343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63114,6 +63114,429 @@
         </is>
       </c>
     </row>
+    <row r="1335">
+      <c r="A1335" t="inlineStr">
+        <is>
+          <t>CHI-20261015-001</t>
+        </is>
+      </c>
+      <c r="B1335" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C1335" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1335" t="inlineStr">
+        <is>
+          <t>翘尾巴</t>
+        </is>
+      </c>
+      <c r="E1335" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1335" t="inlineStr">
+        <is>
+          <t>qiào wěi ba</t>
+        </is>
+      </c>
+      <c r="G1335" t="inlineStr">
+        <is>
+          <t>자만하다, 우쭐대다</t>
+        </is>
+      </c>
+      <c r="H1335" t="inlineStr">
+        <is>
+          <t>这次运动会虽然包揽了前几名，但也千万不能翘尾巴。</t>
+        </is>
+      </c>
+      <c r="I1335" t="inlineStr">
+        <is>
+          <t>刚取得一点小成绩就开始翘尾巴，往往很快就会摔跟头。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="inlineStr">
+        <is>
+          <t>CHI-20261015-002</t>
+        </is>
+      </c>
+      <c r="B1336" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C1336" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1336" t="inlineStr">
+        <is>
+          <t>走下坡路</t>
+        </is>
+      </c>
+      <c r="E1336" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1336" t="inlineStr">
+        <is>
+          <t>zǒu xià pō lù</t>
+        </is>
+      </c>
+      <c r="G1336" t="inlineStr">
+        <is>
+          <t>내리막길을 걷다, 쇠퇴하다</t>
+        </is>
+      </c>
+      <c r="H1336" t="inlineStr">
+        <is>
+          <t>如果产品不持续研发创新，品牌口碑很快就会走下坡路。</t>
+        </is>
+      </c>
+      <c r="I1336" t="inlineStr">
+        <is>
+          <t>那家老牌连锁餐饮自更换管理层之后，业绩就一直在走下坡路。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="inlineStr">
+        <is>
+          <t>CHI-20261015-003</t>
+        </is>
+      </c>
+      <c r="B1337" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C1337" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1337" t="inlineStr">
+        <is>
+          <t>尝甜头</t>
+        </is>
+      </c>
+      <c r="E1337" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1337" t="inlineStr">
+        <is>
+          <t>cháng tián tou</t>
+        </is>
+      </c>
+      <c r="G1337" t="inlineStr">
+        <is>
+          <t>재미를 보다, 혜택이나 단맛을 보다</t>
+        </is>
+      </c>
+      <c r="H1337" t="inlineStr">
+        <is>
+          <t>自从尝试了数字化教学模式，学校教师们确实尝到了不少甜头。</t>
+        </is>
+      </c>
+      <c r="I1337" t="inlineStr">
+        <is>
+          <t>初期投资尝到甜头之后，他开始考虑进一步扩大店面规模。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" t="inlineStr">
+        <is>
+          <t>CHI-20261015-004</t>
+        </is>
+      </c>
+      <c r="B1338" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C1338" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1338" t="inlineStr">
+        <is>
+          <t>找茬儿</t>
+        </is>
+      </c>
+      <c r="E1338" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1338" t="inlineStr">
+        <is>
+          <t>zhǎo chár</t>
+        </is>
+      </c>
+      <c r="G1338" t="inlineStr">
+        <is>
+          <t>트집을 잡다, 시비를 걸다</t>
+        </is>
+      </c>
+      <c r="H1338" t="inlineStr">
+        <is>
+          <t>他今天心情不好，开会时鸡蛋里挑骨头，纯粹是故意找茬儿。</t>
+        </is>
+      </c>
+      <c r="I1338" t="inlineStr">
+        <is>
+          <t>我们服务流程完全符合规范，顾客要是无理找茬儿我们也不必退缩。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" t="inlineStr">
+        <is>
+          <t>CHI-20261015-005</t>
+        </is>
+      </c>
+      <c r="B1339" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C1339" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1339" t="inlineStr">
+        <is>
+          <t>打小报告</t>
+        </is>
+      </c>
+      <c r="E1339" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1339" t="inlineStr">
+        <is>
+          <t>dǎ xiǎo bào gào</t>
+        </is>
+      </c>
+      <c r="G1339" t="inlineStr">
+        <is>
+          <t>은밀히 고자질하다</t>
+        </is>
+      </c>
+      <c r="H1339" t="inlineStr">
+        <is>
+          <t>在团队里最让人反感的行为，就是背着同事在领导面前打小报告。</t>
+        </is>
+      </c>
+      <c r="I1339" t="inlineStr">
+        <is>
+          <t>有什么问题当面沟通就好，千万别背地里去打小报告。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" t="inlineStr">
+        <is>
+          <t>CHI-20261015-006</t>
+        </is>
+      </c>
+      <c r="B1340" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C1340" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1340" t="inlineStr">
+        <is>
+          <t>包揽</t>
+        </is>
+      </c>
+      <c r="E1340" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1340" t="inlineStr">
+        <is>
+          <t>bāo lǎn</t>
+        </is>
+      </c>
+      <c r="G1340" t="inlineStr">
+        <is>
+          <t>독차지하다, 싹쓸이하다, 도맡다</t>
+        </is>
+      </c>
+      <c r="H1340" t="inlineStr">
+        <is>
+          <t>这次比赛的冠亚军被我们团队完全包揽了。</t>
+        </is>
+      </c>
+      <c r="I1340" t="inlineStr">
+        <is>
+          <t>这个项目的策划和落地基本上都是小李一人包揽的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" t="inlineStr">
+        <is>
+          <t>CHI-20261015-007</t>
+        </is>
+      </c>
+      <c r="B1341" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C1341" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1341" t="inlineStr">
+        <is>
+          <t>对标</t>
+        </is>
+      </c>
+      <c r="E1341" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1341" t="inlineStr">
+        <is>
+          <t>duì biāo</t>
+        </is>
+      </c>
+      <c r="G1341" t="inlineStr">
+        <is>
+          <t>벤치마킹하다, 기준에 맞추다</t>
+        </is>
+      </c>
+      <c r="H1341" t="inlineStr">
+        <is>
+          <t>我们的新产品必须全面对标行业领先标准。</t>
+        </is>
+      </c>
+      <c r="I1341" t="inlineStr">
+        <is>
+          <t>公司计划对标行业龙头企业，全面优化内部管理流程。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" t="inlineStr">
+        <is>
+          <t>CHI-20261015-008</t>
+        </is>
+      </c>
+      <c r="B1342" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C1342" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1342" t="inlineStr">
+        <is>
+          <t>化害为利</t>
+        </is>
+      </c>
+      <c r="E1342" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1342" t="inlineStr">
+        <is>
+          <t>huà hài wéi lì</t>
+        </is>
+      </c>
+      <c r="G1342" t="inlineStr">
+        <is>
+          <t>해로운 것을 이롭게 바꾸다, 위기를 기회로 삼다</t>
+        </is>
+      </c>
+      <c r="H1342" t="inlineStr">
+        <is>
+          <t>面对危机我们要学会调整策略，争取化害为利。</t>
+        </is>
+      </c>
+      <c r="I1342" t="inlineStr">
+        <is>
+          <t>通过资源循环利用，这家化工厂化害为利，降低了排污成本。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" t="inlineStr">
+        <is>
+          <t>CHI-20261015-009</t>
+        </is>
+      </c>
+      <c r="B1343" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C1343" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1343" t="inlineStr">
+        <is>
+          <t>领头羊</t>
+        </is>
+      </c>
+      <c r="E1343" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1343" t="inlineStr">
+        <is>
+          <t>lǐng tóu yáng</t>
+        </is>
+      </c>
+      <c r="G1343" t="inlineStr">
+        <is>
+          <t>선두주자, 리더, 견인차</t>
+        </is>
+      </c>
+      <c r="H1343" t="inlineStr">
+        <is>
+          <t>作为新能源行业的领头羊，这家公司一直注重技术创新。</t>
+        </is>
+      </c>
+      <c r="I1343" t="inlineStr">
+        <is>
+          <t>王总是我们部门的领头羊，总是能带领团队攻克业务难关。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-10-16 | 1348/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1343"/>
+  <dimension ref="A1:I1349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63537,6 +63537,288 @@
         </is>
       </c>
     </row>
+    <row r="1344">
+      <c r="A1344" t="inlineStr">
+        <is>
+          <t>CHI-20261016-001</t>
+        </is>
+      </c>
+      <c r="B1344" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C1344" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1344" t="inlineStr">
+        <is>
+          <t>做表面文章</t>
+        </is>
+      </c>
+      <c r="E1344" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1344" t="inlineStr">
+        <is>
+          <t>zuò biǎomiàn wénzhāng</t>
+        </is>
+      </c>
+      <c r="G1344" t="inlineStr">
+        <is>
+          <t>실속 없이 겉치레만 하다, 눈가리고 아웅하다</t>
+        </is>
+      </c>
+      <c r="H1344" t="inlineStr">
+        <is>
+          <t>企业搞环保不能只停留在口头上做表面文章，消费者看重的是实质行动。</t>
+        </is>
+      </c>
+      <c r="I1344" t="inlineStr">
+        <is>
+          <t>领导最反感下属做表面文章，报告写得再天花乱坠，没有实际业绩也免谈。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" t="inlineStr">
+        <is>
+          <t>CHI-20261016-002</t>
+        </is>
+      </c>
+      <c r="B1345" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C1345" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1345" t="inlineStr">
+        <is>
+          <t>动真格</t>
+        </is>
+      </c>
+      <c r="E1345" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1345" t="inlineStr">
+        <is>
+          <t>dòng zhēn gé</t>
+        </is>
+      </c>
+      <c r="G1345" t="inlineStr">
+        <is>
+          <t>형식적이 아니라 각잡고 본격적으로 나서다, 본때를 보이다</t>
+        </is>
+      </c>
+      <c r="H1345" t="inlineStr">
+        <is>
+          <t>这次纪委连打两虎，说明上面反腐是真的动真格了，绝不姑息迁就。</t>
+        </is>
+      </c>
+      <c r="I1345" t="inlineStr">
+        <is>
+          <t>公司下个月起要动真格推行末位淘汰制，大家私底下都紧张起来了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" t="inlineStr">
+        <is>
+          <t>CHI-20261016-003</t>
+        </is>
+      </c>
+      <c r="B1346" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C1346" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1346" t="inlineStr">
+        <is>
+          <t>缓不过来</t>
+        </is>
+      </c>
+      <c r="E1346" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1346" t="inlineStr">
+        <is>
+          <t>huǎn bu guò lái</t>
+        </is>
+      </c>
+      <c r="G1346" t="inlineStr">
+        <is>
+          <t>충격이나 과로, 긴 연휴의 후유증에서 쉽게 회복되지 못하다</t>
+        </is>
+      </c>
+      <c r="H1346" t="inlineStr">
+        <is>
+          <t>长假都结束一个月了，不少孩子在课堂上还是缓不过来，注意力很难集中。</t>
+        </is>
+      </c>
+      <c r="I1346" t="inlineStr">
+        <is>
+          <t>连轴转熬夜加班了整整一周，我现在整个人浑浑噩噩，完全缓不过来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" t="inlineStr">
+        <is>
+          <t>CHI-20261016-004</t>
+        </is>
+      </c>
+      <c r="B1347" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C1347" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1347" t="inlineStr">
+        <is>
+          <t>压舱石</t>
+        </is>
+      </c>
+      <c r="E1347" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1347" t="inlineStr">
+        <is>
+          <t>yā cāng shí</t>
+        </is>
+      </c>
+      <c r="G1347" t="inlineStr">
+        <is>
+          <t>흔들리지 않게 든든히 중심을 잡아주는 핵심 버팀목</t>
+        </is>
+      </c>
+      <c r="H1347" t="inlineStr">
+        <is>
+          <t>无论国际风云如何变幻，实体经济的基本盘始终是国家繁荣稳定的压舱石。</t>
+        </is>
+      </c>
+      <c r="I1347" t="inlineStr">
+        <is>
+          <t>在瞬息万变的快消行业里，持续稳定的供应链能力就是品牌抵御风险的压舱石。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" t="inlineStr">
+        <is>
+          <t>CHI-20261016-005</t>
+        </is>
+      </c>
+      <c r="B1348" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C1348" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1348" t="inlineStr">
+        <is>
+          <t>扯后腿</t>
+        </is>
+      </c>
+      <c r="E1348" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1348" t="inlineStr">
+        <is>
+          <t>chě hòu tuǐ</t>
+        </is>
+      </c>
+      <c r="G1348" t="inlineStr">
+        <is>
+          <t>뒤에서 훼방을 놓다, 발목을 잡다</t>
+        </is>
+      </c>
+      <c r="H1348" t="inlineStr">
+        <is>
+          <t>大家要心往一处想，千万别在团队关键时刻扯后腿。</t>
+        </is>
+      </c>
+      <c r="I1348" t="inlineStr">
+        <is>
+          <t>如果后勤保障跟不上，就会扯整个前线销售团队的后腿。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" t="inlineStr">
+        <is>
+          <t>CHI-20261016-006</t>
+        </is>
+      </c>
+      <c r="B1349" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C1349" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1349" t="inlineStr">
+        <is>
+          <t>抓把柄</t>
+        </is>
+      </c>
+      <c r="E1349" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1349" t="inlineStr">
+        <is>
+          <t>zhuā bǎ bǐng</t>
+        </is>
+      </c>
+      <c r="G1349" t="inlineStr">
+        <is>
+          <t>약점이나 트집거리를 쥐다</t>
+        </is>
+      </c>
+      <c r="H1349" t="inlineStr">
+        <is>
+          <t>公职人员日常用权必须公私分明，万万不可被居心不良的人抓到把柄。</t>
+        </is>
+      </c>
+      <c r="I1349" t="inlineStr">
+        <is>
+          <t>我们在书面邮件里措辞要严谨，免得被竞争对手抓了把柄。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-10-19 | 1351/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1349"/>
+  <dimension ref="A1:I1352"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63819,6 +63819,147 @@
         </is>
       </c>
     </row>
+    <row r="1350">
+      <c r="A1350" t="inlineStr">
+        <is>
+          <t>CHI-20261019-001</t>
+        </is>
+      </c>
+      <c r="B1350" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C1350" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1350" t="inlineStr">
+        <is>
+          <t>紧锣密鼓</t>
+        </is>
+      </c>
+      <c r="E1350" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F1350" t="inlineStr">
+        <is>
+          <t>jǐn luó mì gǔ</t>
+        </is>
+      </c>
+      <c r="G1350" t="inlineStr">
+        <is>
+          <t>대대적으로 준비하다, 긴박하게 추진하다</t>
+        </is>
+      </c>
+      <c r="H1350" t="inlineStr">
+        <is>
+          <t>APEC工商领导人峰会迎来倒计时1个月，各项筹备工作正在紧锣密鼓地进行。</t>
+        </is>
+      </c>
+      <c r="I1350" t="inlineStr">
+        <is>
+          <t>为了下周的发布会，全公司都在紧锣密鼓地筹备着。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" t="inlineStr">
+        <is>
+          <t>CHI-20261019-002</t>
+        </is>
+      </c>
+      <c r="B1351" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C1351" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1351" t="inlineStr">
+        <is>
+          <t>扯大旗</t>
+        </is>
+      </c>
+      <c r="E1351" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1351" t="inlineStr">
+        <is>
+          <t>chě dà qí</t>
+        </is>
+      </c>
+      <c r="G1351" t="inlineStr">
+        <is>
+          <t>명분을 내세우다, 핑계를 대다</t>
+        </is>
+      </c>
+      <c r="H1351" t="inlineStr">
+        <is>
+          <t>不能借着环保的幌子扯大旗，却在私底下乱扔垃圾。</t>
+        </is>
+      </c>
+      <c r="I1351" t="inlineStr">
+        <is>
+          <t>他总是扯着为公司着想的大旗，实际上全是个人私利。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" t="inlineStr">
+        <is>
+          <t>CHI-20261019-003</t>
+        </is>
+      </c>
+      <c r="B1352" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C1352" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1352" t="inlineStr">
+        <is>
+          <t>打比方</t>
+        </is>
+      </c>
+      <c r="E1352" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1352" t="inlineStr">
+        <is>
+          <t>dǎ bǐ fang</t>
+        </is>
+      </c>
+      <c r="G1352" t="inlineStr">
+        <is>
+          <t>비유를 들다, 예를 들어 설명하다</t>
+        </is>
+      </c>
+      <c r="H1352" t="inlineStr">
+        <is>
+          <t>用打比方的方式解读政策图表，能让普通群众一目了然。</t>
+        </is>
+      </c>
+      <c r="I1352" t="inlineStr">
+        <is>
+          <t>老师打了个很生动的比方，大家立刻就听懂了这个概念。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-10-21 | 1358/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1352"/>
+  <dimension ref="A1:I1359"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63960,6 +63960,335 @@
         </is>
       </c>
     </row>
+    <row r="1353">
+      <c r="A1353" t="inlineStr">
+        <is>
+          <t>CHI-20261021-001</t>
+        </is>
+      </c>
+      <c r="B1353" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C1353" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1353" t="inlineStr">
+        <is>
+          <t>放烟雾弹</t>
+        </is>
+      </c>
+      <c r="E1353" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1353" t="inlineStr">
+        <is>
+          <t>fàng yān wù dàn</t>
+        </is>
+      </c>
+      <c r="G1353" t="inlineStr">
+        <is>
+          <t>연막을 치다, 교란 작전을 펴다</t>
+        </is>
+      </c>
+      <c r="H1353" t="inlineStr">
+        <is>
+          <t>部分企业一边宣传所谓的环保理念，一边偷偷排污，分明是在放烟雾弹。</t>
+        </is>
+      </c>
+      <c r="I1353" t="inlineStr">
+        <is>
+          <t>竞品公司频繁发布新功能预告，很有可能只是在放烟雾弹。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" t="inlineStr">
+        <is>
+          <t>CHI-20261021-002</t>
+        </is>
+      </c>
+      <c r="B1354" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C1354" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1354" t="inlineStr">
+        <is>
+          <t>答卷</t>
+        </is>
+      </c>
+      <c r="E1354" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1354" t="inlineStr">
+        <is>
+          <t>dá juàn</t>
+        </is>
+      </c>
+      <c r="G1354" t="inlineStr">
+        <is>
+          <t>답안지, 성과나 결과물</t>
+        </is>
+      </c>
+      <c r="H1354" t="inlineStr">
+        <is>
+          <t>全链路落实环保，天然之扉书写洗护品牌的生态责任答卷。</t>
+        </is>
+      </c>
+      <c r="I1354" t="inlineStr">
+        <is>
+          <t>新任经理上任三个月，交出了一份令人满意的销售答卷。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" t="inlineStr">
+        <is>
+          <t>CHI-20261021-003</t>
+        </is>
+      </c>
+      <c r="B1355" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C1355" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1355" t="inlineStr">
+        <is>
+          <t>下沉</t>
+        </is>
+      </c>
+      <c r="E1355" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1355" t="inlineStr">
+        <is>
+          <t>xià chén</t>
+        </is>
+      </c>
+      <c r="G1355" t="inlineStr">
+        <is>
+          <t>일선 현장으로 내려가다, 침투하다</t>
+        </is>
+      </c>
+      <c r="H1355" t="inlineStr">
+        <is>
+          <t>面对面听诉求丨香坊城管下沉社区，把服务送到居民家门口。</t>
+        </is>
+      </c>
+      <c r="I1355" t="inlineStr">
+        <is>
+          <t>公司高管团队决定下沉到一线门店，实地考察顾客体验。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" t="inlineStr">
+        <is>
+          <t>CHI-20261021-004</t>
+        </is>
+      </c>
+      <c r="B1356" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C1356" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1356" t="inlineStr">
+        <is>
+          <t>摸脉</t>
+        </is>
+      </c>
+      <c r="E1356" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1356" t="inlineStr">
+        <is>
+          <t>mō mài</t>
+        </is>
+      </c>
+      <c r="G1356" t="inlineStr">
+        <is>
+          <t>맥을 짚다, 트렌드나 핵심 흐름을 파악하다</t>
+        </is>
+      </c>
+      <c r="H1356" t="inlineStr">
+        <is>
+          <t>在这里，最先触摸全球制造升级脉搏。</t>
+        </is>
+      </c>
+      <c r="I1356" t="inlineStr">
+        <is>
+          <t>在制定营销策略之前，我们要先摸清消费者的心理脉搏。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" t="inlineStr">
+        <is>
+          <t>CHI-20261021-005</t>
+        </is>
+      </c>
+      <c r="B1357" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C1357" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1357" t="inlineStr">
+        <is>
+          <t>绊脚石</t>
+        </is>
+      </c>
+      <c r="E1357" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1357" t="inlineStr">
+        <is>
+          <t>bàn jiǎo shí</t>
+        </is>
+      </c>
+      <c r="G1357" t="inlineStr">
+        <is>
+          <t>걸림돌, 장애물</t>
+        </is>
+      </c>
+      <c r="H1357" t="inlineStr">
+        <is>
+          <t>唯分数论已经成为制约学生综合素养全面发展的绊脚石。</t>
+        </is>
+      </c>
+      <c r="I1357" t="inlineStr">
+        <is>
+          <t>畏惧失败的心态往往是个人职业成长道路上的绊脚石。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" t="inlineStr">
+        <is>
+          <t>CHI-20261021-006</t>
+        </is>
+      </c>
+      <c r="B1358" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C1358" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1358" t="inlineStr">
+        <is>
+          <t>找差距</t>
+        </is>
+      </c>
+      <c r="E1358" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1358" t="inlineStr">
+        <is>
+          <t>zhǎo chā jù</t>
+        </is>
+      </c>
+      <c r="G1358" t="inlineStr">
+        <is>
+          <t>격차/미흡한 점을 점검하다, 벤치마킹하여 반성하다</t>
+        </is>
+      </c>
+      <c r="H1358" t="inlineStr">
+        <is>
+          <t>通过对标标杆学校，大家认真找差距、补短板。</t>
+        </is>
+      </c>
+      <c r="I1358" t="inlineStr">
+        <is>
+          <t>年终总结不仅要汇报成绩，更重要的是找差距和不足。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" t="inlineStr">
+        <is>
+          <t>CHI-20261021-007</t>
+        </is>
+      </c>
+      <c r="B1359" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C1359" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1359" t="inlineStr">
+        <is>
+          <t>搭平台</t>
+        </is>
+      </c>
+      <c r="E1359" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1359" t="inlineStr">
+        <is>
+          <t>dā píng tái</t>
+        </is>
+      </c>
+      <c r="G1359" t="inlineStr">
+        <is>
+          <t>발판을 마련하다, 네트워크/플랫폼을 구축하다</t>
+        </is>
+      </c>
+      <c r="H1359" t="inlineStr">
+        <is>
+          <t>栏目正式开播，旨在为本土优秀企业家搭建交流合作的平台。</t>
+        </is>
+      </c>
+      <c r="I1359" t="inlineStr">
+        <is>
+          <t>学校积极搭平台、引资源，为毕业生创造更多的实习机会。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-10-22 | 1361/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1359"/>
+  <dimension ref="A1:I1362"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64289,6 +64289,147 @@
         </is>
       </c>
     </row>
+    <row r="1360">
+      <c r="A1360" t="inlineStr">
+        <is>
+          <t>CHI-20261022-001</t>
+        </is>
+      </c>
+      <c r="B1360" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C1360" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1360" t="inlineStr">
+        <is>
+          <t>碰运气</t>
+        </is>
+      </c>
+      <c r="E1360" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1360" t="inlineStr">
+        <is>
+          <t>pèng yùn qì</t>
+        </is>
+      </c>
+      <c r="G1360" t="inlineStr">
+        <is>
+          <t>운을 시험하다, 요행을 바라다</t>
+        </is>
+      </c>
+      <c r="H1360" t="inlineStr">
+        <is>
+          <t>找工作要靠真本事，不能只抱着碰运气的心理。</t>
+        </is>
+      </c>
+      <c r="I1360" t="inlineStr">
+        <is>
+          <t>他去参加大型招聘会，主要是想碰运气找个好岗位。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" t="inlineStr">
+        <is>
+          <t>CHI-20261022-002</t>
+        </is>
+      </c>
+      <c r="B1361" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C1361" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1361" t="inlineStr">
+        <is>
+          <t>唱红脸</t>
+        </is>
+      </c>
+      <c r="E1361" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1361" t="inlineStr">
+        <is>
+          <t>chàng hóng liǎn</t>
+        </is>
+      </c>
+      <c r="G1361" t="inlineStr">
+        <is>
+          <t>착한 사람 역할을 하다, 달래는 역을 맡다</t>
+        </is>
+      </c>
+      <c r="H1361" t="inlineStr">
+        <is>
+          <t>谈判时经理唱白脸施压，我负责唱红脸缓和气氛。</t>
+        </is>
+      </c>
+      <c r="I1361" t="inlineStr">
+        <is>
+          <t>教育孩子时，父母一个唱红脸一个唱白脸更有效。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" t="inlineStr">
+        <is>
+          <t>CHI-20261022-003</t>
+        </is>
+      </c>
+      <c r="B1362" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C1362" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1362" t="inlineStr">
+        <is>
+          <t>下血本</t>
+        </is>
+      </c>
+      <c r="E1362" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1362" t="inlineStr">
+        <is>
+          <t>xià xuè běn</t>
+        </is>
+      </c>
+      <c r="G1362" t="inlineStr">
+        <is>
+          <t>큰돈을 쏟아붓다, 거금을 들이다</t>
+        </is>
+      </c>
+      <c r="H1362" t="inlineStr">
+        <is>
+          <t>公司为了研发新一代环保材料，这次可是下了血本。</t>
+        </is>
+      </c>
+      <c r="I1362" t="inlineStr">
+        <is>
+          <t>他下了血本升级生产线，终于将产品次品率降到了最低。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-10-26 | 1370/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1362"/>
+  <dimension ref="A1:I1371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64430,6 +64430,429 @@
         </is>
       </c>
     </row>
+    <row r="1363">
+      <c r="A1363" t="inlineStr">
+        <is>
+          <t>CHI-20261026-001</t>
+        </is>
+      </c>
+      <c r="B1363" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C1363" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1363" t="inlineStr">
+        <is>
+          <t>帮大忙</t>
+        </is>
+      </c>
+      <c r="E1363" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1363" t="inlineStr">
+        <is>
+          <t>bāng dà máng</t>
+        </is>
+      </c>
+      <c r="G1363" t="inlineStr">
+        <is>
+          <t>큰 도움이 되다</t>
+        </is>
+      </c>
+      <c r="H1363" t="inlineStr">
+        <is>
+          <t>社区工作人员进驻后，帮了居民不少大忙。</t>
+        </is>
+      </c>
+      <c r="I1363" t="inlineStr">
+        <is>
+          <t>你这次给我提供的资料真是帮了大忙。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" t="inlineStr">
+        <is>
+          <t>CHI-20261026-002</t>
+        </is>
+      </c>
+      <c r="B1364" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C1364" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1364" t="inlineStr">
+        <is>
+          <t>压马路</t>
+        </is>
+      </c>
+      <c r="E1364" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1364" t="inlineStr">
+        <is>
+          <t>yā mǎ lù</t>
+        </is>
+      </c>
+      <c r="G1364" t="inlineStr">
+        <is>
+          <t>(거리/길을) 한가롭게 거닐다, 데이트하며 산책하다</t>
+        </is>
+      </c>
+      <c r="H1364" t="inlineStr">
+        <is>
+          <t>周末大家不去商圈购物，反而喜欢沿着新开通的街道压压马路。</t>
+        </is>
+      </c>
+      <c r="I1364" t="inlineStr">
+        <is>
+          <t>吃完晚饭后，我和家人一起去公园附近压马路。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" t="inlineStr">
+        <is>
+          <t>CHI-20261026-003</t>
+        </is>
+      </c>
+      <c r="B1365" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C1365" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1365" t="inlineStr">
+        <is>
+          <t>换血</t>
+        </is>
+      </c>
+      <c r="E1365" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1365" t="inlineStr">
+        <is>
+          <t>huàn xuè</t>
+        </is>
+      </c>
+      <c r="G1365" t="inlineStr">
+        <is>
+          <t>(조직/인력을) 대대적으로 쇄신하다, 전면 교체하다</t>
+        </is>
+      </c>
+      <c r="H1365" t="inlineStr">
+        <is>
+          <t>为了激发文旅产业的新活力，管理团队迎来了彻底的换血。</t>
+        </is>
+      </c>
+      <c r="I1365" t="inlineStr">
+        <is>
+          <t>公司为了突破瓶颈，高层管理人员进行了换血。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" t="inlineStr">
+        <is>
+          <t>CHI-20261026-004</t>
+        </is>
+      </c>
+      <c r="B1366" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C1366" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1366" t="inlineStr">
+        <is>
+          <t>占座位</t>
+        </is>
+      </c>
+      <c r="E1366" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1366" t="inlineStr">
+        <is>
+          <t>zhàn zuò wèi</t>
+        </is>
+      </c>
+      <c r="G1366" t="inlineStr">
+        <is>
+          <t>자리를 잡다, 찜하다</t>
+        </is>
+      </c>
+      <c r="H1366" t="inlineStr">
+        <is>
+          <t>在新升级的车站候车区里，旅客们再也不用提前占座位了。</t>
+        </is>
+      </c>
+      <c r="I1366" t="inlineStr">
+        <is>
+          <t>去图书馆自习的人很多，你需要早点去占座位。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" t="inlineStr">
+        <is>
+          <t>CHI-20261026-005</t>
+        </is>
+      </c>
+      <c r="B1367" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C1367" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1367" t="inlineStr">
+        <is>
+          <t>请大假</t>
+        </is>
+      </c>
+      <c r="E1367" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1367" t="inlineStr">
+        <is>
+          <t>qǐng dà jià</t>
+        </is>
+      </c>
+      <c r="G1367" t="inlineStr">
+        <is>
+          <t>장기 휴가를 내다</t>
+        </is>
+      </c>
+      <c r="H1367" t="inlineStr">
+        <is>
+          <t>忙完这个大型施工项目后，他打算好好请个大假休息一下。</t>
+        </is>
+      </c>
+      <c r="I1367" t="inlineStr">
+        <is>
+          <t>项目终于收尾了，我准备请个大假去旅游。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" t="inlineStr">
+        <is>
+          <t>CHI-20261026-006</t>
+        </is>
+      </c>
+      <c r="B1368" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C1368" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1368" t="inlineStr">
+        <is>
+          <t>变通</t>
+        </is>
+      </c>
+      <c r="E1368" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1368" t="inlineStr">
+        <is>
+          <t>biàn tōng</t>
+        </is>
+      </c>
+      <c r="G1368" t="inlineStr">
+        <is>
+          <t>융통성 있게 처리하다, 상황에 맞게 바꾸다</t>
+        </is>
+      </c>
+      <c r="H1368" t="inlineStr">
+        <is>
+          <t>面对小户型装修的局限，设计师灵活变通，打造出了高级感。</t>
+        </is>
+      </c>
+      <c r="I1368" t="inlineStr">
+        <is>
+          <t>规则是死的人是活的，遇到特殊情况要学会变通。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" t="inlineStr">
+        <is>
+          <t>CHI-20261026-007</t>
+        </is>
+      </c>
+      <c r="B1369" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C1369" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1369" t="inlineStr">
+        <is>
+          <t>搬砖</t>
+        </is>
+      </c>
+      <c r="E1369" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1369" t="inlineStr">
+        <is>
+          <t>bān zhuān</t>
+        </is>
+      </c>
+      <c r="G1369" t="inlineStr">
+        <is>
+          <t>(직장에서) 힘들게 일하다, 돈 벌러 가다</t>
+        </is>
+      </c>
+      <c r="H1369" t="inlineStr">
+        <is>
+          <t>假期一结束，职场人们又得打起精神回到岗位上搬砖了。</t>
+        </is>
+      </c>
+      <c r="I1369" t="inlineStr">
+        <is>
+          <t>不说了，我要准备去公司搬砖了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" t="inlineStr">
+        <is>
+          <t>CHI-20261026-008</t>
+        </is>
+      </c>
+      <c r="B1370" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C1370" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1370" t="inlineStr">
+        <is>
+          <t>出点子</t>
+        </is>
+      </c>
+      <c r="E1370" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1370" t="inlineStr">
+        <is>
+          <t>chū diǎn zi</t>
+        </is>
+      </c>
+      <c r="G1370" t="inlineStr">
+        <is>
+          <t>아이디어를 내다, 꾀를 내다</t>
+        </is>
+      </c>
+      <c r="H1370" t="inlineStr">
+        <is>
+          <t>大家纷纷为如何将文化流量转化为经济效益出点子。</t>
+        </is>
+      </c>
+      <c r="I1370" t="inlineStr">
+        <is>
+          <t>这次的推广方案全靠他帮忙出点子。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" t="inlineStr">
+        <is>
+          <t>CHI-20261026-009</t>
+        </is>
+      </c>
+      <c r="B1371" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C1371" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1371" t="inlineStr">
+        <is>
+          <t>算账</t>
+        </is>
+      </c>
+      <c r="E1371" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1371" t="inlineStr">
+        <is>
+          <t>suàn zhàng</t>
+        </is>
+      </c>
+      <c r="G1371" t="inlineStr">
+        <is>
+          <t>정산하다, 따지다/책임을 묻다</t>
+        </is>
+      </c>
+      <c r="H1371" t="inlineStr">
+        <is>
+          <t>企业之间要按约兑现，不能等到年底才来算总账。</t>
+        </is>
+      </c>
+      <c r="I1371" t="inlineStr">
+        <is>
+          <t>出了这么大的纰漏，公司肯定会找他算账。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-10-29 | 1386/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1371"/>
+  <dimension ref="A1:I1387"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64853,6 +64853,758 @@
         </is>
       </c>
     </row>
+    <row r="1372">
+      <c r="A1372" t="inlineStr">
+        <is>
+          <t>CHI-20261029-001</t>
+        </is>
+      </c>
+      <c r="B1372" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C1372" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1372" t="inlineStr">
+        <is>
+          <t>变现</t>
+        </is>
+      </c>
+      <c r="E1372" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1372" t="inlineStr">
+        <is>
+          <t>biàn xiàn</t>
+        </is>
+      </c>
+      <c r="G1372" t="inlineStr">
+        <is>
+          <t>현금화하다, 수익화하다 (주로 트래픽이나 IP를 돈으로 바꿀 때)</t>
+        </is>
+      </c>
+      <c r="H1372" t="inlineStr">
+        <is>
+          <t>인기나 콘텐츠(IP)를 실제 수익 모델로 연결할 때</t>
+        </is>
+      </c>
+      <c r="I1372" t="inlineStr">
+        <is>
+          <t>现在很多网红都面临流量变现的压力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" t="inlineStr">
+        <is>
+          <t>CHI-20261029-002</t>
+        </is>
+      </c>
+      <c r="B1373" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C1373" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1373" t="inlineStr">
+        <is>
+          <t>痛点</t>
+        </is>
+      </c>
+      <c r="E1373" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1373" t="inlineStr">
+        <is>
+          <t>tòng diǎn</t>
+        </is>
+      </c>
+      <c r="G1373" t="inlineStr">
+        <is>
+          <t>핵심 문제, 고객의 불편 사항(Pain Point)</t>
+        </is>
+      </c>
+      <c r="H1373" t="inlineStr">
+        <is>
+          <t>시장이나 비즈니스에서 해결해야 할 근본적인 니즈를 논할 때</t>
+        </is>
+      </c>
+      <c r="I1373" t="inlineStr">
+        <is>
+          <t>这款产品的设计精准抓住了用户的痛点。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" t="inlineStr">
+        <is>
+          <t>CHI-20261029-003</t>
+        </is>
+      </c>
+      <c r="B1374" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C1374" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1374" t="inlineStr">
+        <is>
+          <t>烧钱</t>
+        </is>
+      </c>
+      <c r="E1374" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1374" t="inlineStr">
+        <is>
+          <t>shāo qián</t>
+        </is>
+      </c>
+      <c r="G1374" t="inlineStr">
+        <is>
+          <t>돈이 많이 들다, 돈을 쏟아붓다</t>
+        </is>
+      </c>
+      <c r="H1374" t="inlineStr">
+        <is>
+          <t>프로젝트나 취미에 비용이 과도하게 들어갈 때</t>
+        </is>
+      </c>
+      <c r="I1374" t="inlineStr">
+        <is>
+          <t>摄影这个爱好真的太烧钱了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" t="inlineStr">
+        <is>
+          <t>CHI-20261029-004</t>
+        </is>
+      </c>
+      <c r="B1375" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C1375" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1375" t="inlineStr">
+        <is>
+          <t>抠门</t>
+        </is>
+      </c>
+      <c r="E1375" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1375" t="inlineStr">
+        <is>
+          <t>kōu mén</t>
+        </is>
+      </c>
+      <c r="G1375" t="inlineStr">
+        <is>
+          <t>짠돌이 같다, 구두쇠 같다</t>
+        </is>
+      </c>
+      <c r="H1375" t="inlineStr">
+        <is>
+          <t>작은 돈에도 지나치게 인색할 때</t>
+        </is>
+      </c>
+      <c r="I1375" t="inlineStr">
+        <is>
+          <t>他平时对自己很抠门，但对朋友却很大方。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" t="inlineStr">
+        <is>
+          <t>CHI-20261029-005</t>
+        </is>
+      </c>
+      <c r="B1376" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C1376" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1376" t="inlineStr">
+        <is>
+          <t>亮风采</t>
+        </is>
+      </c>
+      <c r="E1376" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1376" t="inlineStr">
+        <is>
+          <t>liàng fēng cǎi</t>
+        </is>
+      </c>
+      <c r="G1376" t="inlineStr">
+        <is>
+          <t>자신의 기량이나 멋진 모습을 마음껏 드러내다</t>
+        </is>
+      </c>
+      <c r="H1376" t="inlineStr">
+        <is>
+          <t>常规展示亮风采！</t>
+        </is>
+      </c>
+      <c r="I1376" t="inlineStr">
+        <is>
+          <t>在这次比赛中，大家都积极地展示才艺，亮出自己的风采。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" t="inlineStr">
+        <is>
+          <t>CHI-20261029-006</t>
+        </is>
+      </c>
+      <c r="B1377" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C1377" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1377" t="inlineStr">
+        <is>
+          <t>花样</t>
+        </is>
+      </c>
+      <c r="E1377" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1377" t="inlineStr">
+        <is>
+          <t>huā yàng</t>
+        </is>
+      </c>
+      <c r="G1377" t="inlineStr">
+        <is>
+          <t>새로운 방식, 묘수, 수법</t>
+        </is>
+      </c>
+      <c r="H1377" t="inlineStr">
+        <is>
+          <t>金山这所高校“玩”出新花样！</t>
+        </is>
+      </c>
+      <c r="I1377" t="inlineStr">
+        <is>
+          <t>现在的营销方式层出不穷，经常能玩出新花样。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" t="inlineStr">
+        <is>
+          <t>CHI-20261029-007</t>
+        </is>
+      </c>
+      <c r="B1378" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C1378" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1378" t="inlineStr">
+        <is>
+          <t>通堵点</t>
+        </is>
+      </c>
+      <c r="E1378" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1378" t="inlineStr">
+        <is>
+          <t>tōng dǔ diǎn</t>
+        </is>
+      </c>
+      <c r="G1378" t="inlineStr">
+        <is>
+          <t>병목 현상을 해결하다, 난제를 풀다</t>
+        </is>
+      </c>
+      <c r="H1378" t="inlineStr">
+        <is>
+          <t>夜探济南开源路通堵点</t>
+        </is>
+      </c>
+      <c r="I1378" t="inlineStr">
+        <is>
+          <t>政府正在努力通堵点，改善城市的交通拥堵状况。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="inlineStr">
+        <is>
+          <t>CHI-20261029-008</t>
+        </is>
+      </c>
+      <c r="B1379" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C1379" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1379" t="inlineStr">
+        <is>
+          <t>按约</t>
+        </is>
+      </c>
+      <c r="E1379" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1379" t="inlineStr">
+        <is>
+          <t>àn yuē</t>
+        </is>
+      </c>
+      <c r="G1379" t="inlineStr">
+        <is>
+          <t>약속대로, 계약대로</t>
+        </is>
+      </c>
+      <c r="H1379" t="inlineStr">
+        <is>
+          <t>让每一笔企业账款按约兑现.</t>
+        </is>
+      </c>
+      <c r="I1379" t="inlineStr">
+        <is>
+          <t>请务必按约完成项目，不要延误工期。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" t="inlineStr">
+        <is>
+          <t>CHI-20261029-009</t>
+        </is>
+      </c>
+      <c r="B1380" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C1380" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1380" t="inlineStr">
+        <is>
+          <t>追梦</t>
+        </is>
+      </c>
+      <c r="E1380" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1380" t="inlineStr">
+        <is>
+          <t>zhuī mèng</t>
+        </is>
+      </c>
+      <c r="G1380" t="inlineStr">
+        <is>
+          <t>꿈을 쫓다</t>
+        </is>
+      </c>
+      <c r="H1380" t="inlineStr">
+        <is>
+          <t>世界冠军敖金平走进阳新三所学校传递追梦力量.</t>
+        </is>
+      </c>
+      <c r="I1380" t="inlineStr">
+        <is>
+          <t>只要我们坚持追梦，总有一天能实现目标。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" t="inlineStr">
+        <is>
+          <t>CHI-20261029-010</t>
+        </is>
+      </c>
+      <c r="B1381" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C1381" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1381" t="inlineStr">
+        <is>
+          <t>擦亮</t>
+        </is>
+      </c>
+      <c r="E1381" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1381" t="inlineStr">
+        <is>
+          <t>cā liàng</t>
+        </is>
+      </c>
+      <c r="G1381" t="inlineStr">
+        <is>
+          <t>(브랜드 등을) 널리 알리다, 돋보이게 하다</t>
+        </is>
+      </c>
+      <c r="H1381" t="inlineStr">
+        <is>
+          <t>基层人大助力文旅产业擦亮“礼遇峄山”名片.</t>
+        </is>
+      </c>
+      <c r="I1381" t="inlineStr">
+        <is>
+          <t>我们应该多做宣传，擦亮这块金字招牌。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" t="inlineStr">
+        <is>
+          <t>CHI-20261029-011</t>
+        </is>
+      </c>
+      <c r="B1382" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C1382" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1382" t="inlineStr">
+        <is>
+          <t>留不住</t>
+        </is>
+      </c>
+      <c r="E1382" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1382" t="inlineStr">
+        <is>
+          <t>liú bu zhù</t>
+        </is>
+      </c>
+      <c r="G1382" t="inlineStr">
+        <is>
+          <t>붙잡을 수 없다, 유치할 수 없다</t>
+        </is>
+      </c>
+      <c r="H1382" t="inlineStr">
+        <is>
+          <t>手握水浒大IP，曾经留不住人！</t>
+        </is>
+      </c>
+      <c r="I1382" t="inlineStr">
+        <is>
+          <t>公司的薪资待遇太低，很难留住优秀人才。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" t="inlineStr">
+        <is>
+          <t>CHI-20261029-012</t>
+        </is>
+      </c>
+      <c r="B1383" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C1383" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1383" t="inlineStr">
+        <is>
+          <t>探访</t>
+        </is>
+      </c>
+      <c r="E1383" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1383" t="inlineStr">
+        <is>
+          <t>tàn fǎng</t>
+        </is>
+      </c>
+      <c r="G1383" t="inlineStr">
+        <is>
+          <t>방문하여 조사하다, 취재하다</t>
+        </is>
+      </c>
+      <c r="H1383" t="inlineStr">
+        <is>
+          <t>视频丨记者探访震区学校：</t>
+        </is>
+      </c>
+      <c r="I1383" t="inlineStr">
+        <is>
+          <t>记者深入灾区探访，了解灾后重建的情况。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" t="inlineStr">
+        <is>
+          <t>CHI-20261029-013</t>
+        </is>
+      </c>
+      <c r="B1384" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C1384" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1384" t="inlineStr">
+        <is>
+          <t>博弈</t>
+        </is>
+      </c>
+      <c r="E1384" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F1384" t="inlineStr">
+        <is>
+          <t>bó yì</t>
+        </is>
+      </c>
+      <c r="G1384" t="inlineStr">
+        <is>
+          <t>경쟁, 대결, 게임 이론에서의 대립</t>
+        </is>
+      </c>
+      <c r="H1384" t="inlineStr">
+        <is>
+          <t>AI赋能，劳动关系协调师巅峰对决.</t>
+        </is>
+      </c>
+      <c r="I1384" t="inlineStr">
+        <is>
+          <t>这是双方在市场份额上的激烈博弈。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" t="inlineStr">
+        <is>
+          <t>CHI-20261029-014</t>
+        </is>
+      </c>
+      <c r="B1385" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C1385" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1385" t="inlineStr">
+        <is>
+          <t>托底</t>
+        </is>
+      </c>
+      <c r="E1385" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1385" t="inlineStr">
+        <is>
+          <t>tuō dǐ</t>
+        </is>
+      </c>
+      <c r="G1385" t="inlineStr">
+        <is>
+          <t>뒷받침하다, 보장하다</t>
+        </is>
+      </c>
+      <c r="H1385" t="inlineStr">
+        <is>
+          <t>高校毕业生：创业和灵活就业，这些支持政策别错过.</t>
+        </is>
+      </c>
+      <c r="I1385" t="inlineStr">
+        <is>
+          <t>这项政策为低收入群体提供了生活托底。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" t="inlineStr">
+        <is>
+          <t>CHI-20261029-015</t>
+        </is>
+      </c>
+      <c r="B1386" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C1386" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1386" t="inlineStr">
+        <is>
+          <t>倒逼</t>
+        </is>
+      </c>
+      <c r="E1386" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1386" t="inlineStr">
+        <is>
+          <t>dào bī</t>
+        </is>
+      </c>
+      <c r="G1386" t="inlineStr">
+        <is>
+          <t>역으로 압박하여 변화를 강제하다</t>
+        </is>
+      </c>
+      <c r="H1386" t="inlineStr">
+        <is>
+          <t>促每笔账款按约兑现.</t>
+        </is>
+      </c>
+      <c r="I1386" t="inlineStr">
+        <is>
+          <t>市场的快速变化倒逼企业进行创新改革。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="inlineStr">
+        <is>
+          <t>CHI-20261029-016</t>
+        </is>
+      </c>
+      <c r="B1387" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C1387" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1387" t="inlineStr">
+        <is>
+          <t>上手</t>
+        </is>
+      </c>
+      <c r="E1387" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1387" t="inlineStr">
+        <is>
+          <t>shàng shǒu</t>
+        </is>
+      </c>
+      <c r="G1387" t="inlineStr">
+        <is>
+          <t>익숙해지다, 손에 익다</t>
+        </is>
+      </c>
+      <c r="H1387" t="inlineStr">
+        <is>
+          <t>AI赋能，劳动关系协调师巅峰对决.</t>
+        </is>
+      </c>
+      <c r="I1387" t="inlineStr">
+        <is>
+          <t>这个新软件很简单，你很快就能上手。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-10-30 | 1389/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1387"/>
+  <dimension ref="A1:I1390"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -65605,6 +65605,147 @@
         </is>
       </c>
     </row>
+    <row r="1388">
+      <c r="A1388" t="inlineStr">
+        <is>
+          <t>CHI-20261030-001</t>
+        </is>
+      </c>
+      <c r="B1388" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C1388" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1388" t="inlineStr">
+        <is>
+          <t>提亲</t>
+        </is>
+      </c>
+      <c r="E1388" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1388" t="inlineStr">
+        <is>
+          <t>tí qīn</t>
+        </is>
+      </c>
+      <c r="G1388" t="inlineStr">
+        <is>
+          <t>혼담을 꺼내다, 청혼하다</t>
+        </is>
+      </c>
+      <c r="H1388" t="inlineStr">
+        <is>
+          <t>传统民俗文化展上演了古时代地道而热闹的提亲仪式，吸引不少游客驻足。</t>
+        </is>
+      </c>
+      <c r="I1388" t="inlineStr">
+        <is>
+          <t>按我们当地的习俗，男方结婚前需要带上礼品去女方家提亲。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" t="inlineStr">
+        <is>
+          <t>CHI-20261030-002</t>
+        </is>
+      </c>
+      <c r="B1389" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C1389" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1389" t="inlineStr">
+        <is>
+          <t>爆棚</t>
+        </is>
+      </c>
+      <c r="E1389" t="inlineStr">
+        <is>
+          <t>형용사</t>
+        </is>
+      </c>
+      <c r="F1389" t="inlineStr">
+        <is>
+          <t>bào péng</t>
+        </is>
+      </c>
+      <c r="G1389" t="inlineStr">
+        <is>
+          <t>가득 차다, 포화 상태이다, 터져 나가다</t>
+        </is>
+      </c>
+      <c r="H1389" t="inlineStr">
+        <is>
+          <t>随着文旅景区的升级改造，商圈烟火气十足，周末的人气瞬间爆棚。</t>
+        </is>
+      </c>
+      <c r="I1389" t="inlineStr">
+        <is>
+          <t>那家新开的网红餐厅味道非常好，每天晚餐时间都是人气爆棚。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" t="inlineStr">
+        <is>
+          <t>CHI-20261030-003</t>
+        </is>
+      </c>
+      <c r="B1390" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C1390" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1390" t="inlineStr">
+        <is>
+          <t>耍花样</t>
+        </is>
+      </c>
+      <c r="E1390" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1390" t="inlineStr">
+        <is>
+          <t>shuǎ huā yàng</t>
+        </is>
+      </c>
+      <c r="G1390" t="inlineStr">
+        <is>
+          <t>잔머리를 굴리다, 수작을 부리다, 속임수를 쓰다</t>
+        </is>
+      </c>
+      <c r="H1390" t="inlineStr">
+        <is>
+          <t>跟客户签合同一定要坦诚实在，千万别在条款上耍花样。</t>
+        </is>
+      </c>
+      <c r="I1390" t="inlineStr">
+        <is>
+          <t>老板一眼就看出来他在报销单据上耍了花样。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>